<commit_message>
feat: update session details for "Il miglior Copilot è umano" and remove duplicate entry
</commit_message>
<xml_diff>
--- a/src/assets/sessionize/data-advanced.xlsx
+++ b/src/assets/sessionize/data-advanced.xlsx
@@ -148,43 +148,6 @@
     <t>46baee89-6771-4806-b4cd-9afd9bc68637</t>
   </si>
   <si>
-    <t>Il miglior Copilot è umano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Questa sessione sarà un'introduzione al pair programming; discuteremo casi d'uso, benefici, e la ricerca a riguardo._x000D_
-_x000D_
-Soprattutto ora che l'ai generativa è sempre più presente nella scrittura del codice, è fondamentale riconoscere l'importanza dell'interazione umana nel design del software._x000D_
-_x000D_
-Ottimizziamo i team di sviluppo per lavorare in parallelo: dividiamo i compiti, scriviamo il codice individualmente e poi lo uniamo. _x000D_
-Sembra efficiente, ma spesso non lo è, e ignora alcuni degli aspetti fondamentali dello sviluppo._x000D_
-_x000D_
-Scegliere consistentemente di programmare insieme mette in discussione questo approccio._x000D_
-Invece di dividere il lavoro, si concentra il pensiero: si considerano problemi e soluzioni da più punti di vista, c'è feedback continuo e condivisione implicita delle conoscenze._x000D_
-_x000D_
-In sintesi questa sessione suggerirà al pubblico di sperimentare una collaborazione più stretta e continuativa durante lo sviluppo e fornirà argomentazioni a favore di questo invito.</t>
-  </si>
-  <si>
-    <t>Jacopo Martellini</t>
-  </si>
-  <si>
-    <t>jack.lilhammers@gmail.com</t>
-  </si>
-  <si>
-    <t>Soft Skills</t>
-  </si>
-  <si>
-    <t>Introductory</t>
-  </si>
-  <si>
-    <t>English, Italian</t>
-  </si>
-  <si>
-    <t>Italia</t>
-  </si>
-  <si>
-    <t>82b493da-0b26-4e1f-9c81-54c9609a4b50</t>
-  </si>
-  <si>
     <t>Come fare il grande passo: da Sviluppatore a Manager</t>
   </si>
   <si>
@@ -197,6 +160,12 @@
   </si>
   <si>
     <t>lory1990@gmail.com</t>
+  </si>
+  <si>
+    <t>Soft Skills</t>
+  </si>
+  <si>
+    <t>Introductory</t>
   </si>
   <si>
     <t>IT</t>
@@ -339,6 +308,9 @@
     <t>monja+devfest@monjadariva.it</t>
   </si>
   <si>
+    <t>Italia</t>
+  </si>
+  <si>
     <t>cd06bc13-e8b8-46ff-87be-87d6f898da0f</t>
   </si>
   <si>
@@ -381,6 +353,9 @@
   </si>
   <si>
     <t>katarinazivkovic092@gmail.com</t>
+  </si>
+  <si>
+    <t>English, Italian</t>
   </si>
   <si>
     <t>04eb395e-7d8e-4723-8bb0-98d7aa6b15a6</t>
@@ -663,6 +638,31 @@
   </si>
   <si>
     <t>6b8ff0d1-1f43-49ee-9406-a3bd8605e2d2, 7dc22085-f2b0-4ef6-9147-93a5bf7bf994</t>
+  </si>
+  <si>
+    <t>Il miglior Copilot è umano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Questa sessione sarà un'introduzione al pair programming; discuteremo casi d'uso, benefici, e la ricerca a riguardo._x000D_
+_x000D_
+Soprattutto ora che l'ai generativa è sempre più presente nella scrittura del codice, è fondamentale riconoscere l'importanza dell'interazione umana nel design del software._x000D_
+_x000D_
+Ottimizziamo i team di sviluppo per lavorare in parallelo: dividiamo i compiti, scriviamo il codice individualmente e poi lo uniamo. _x000D_
+Sembra efficiente, ma spesso non lo è, e ignora alcuni degli aspetti fondamentali dello sviluppo._x000D_
+_x000D_
+Scegliere consistentemente di programmare insieme mette in discussione questo approccio._x000D_
+Invece di dividere il lavoro, si concentra il pensiero: si considerano problemi e soluzioni da più punti di vista, c'è feedback continuo e condivisione implicita delle conoscenze._x000D_
+_x000D_
+In sintesi questa sessione suggerirà al pubblico di sperimentare una collaborazione più stretta e continuativa durante lo sviluppo e fornirà argomentazioni a favore di questo invito.</t>
+  </si>
+  <si>
+    <t>Jacopo Martellini</t>
+  </si>
+  <si>
+    <t>jack.lilhammers@gmail.com</t>
+  </si>
+  <si>
+    <t>82b493da-0b26-4e1f-9c81-54c9609a4b50</t>
   </si>
   <si>
     <t>Agenti in produzione: come sbloccare il potenziale in sicurezza</t>
@@ -2225,7 +2225,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0">
-        <v>1149301</v>
+        <v>1149367</v>
       </c>
       <c r="B4" s="0" t="s">
         <v>42</v>
@@ -2246,7 +2246,7 @@
         <v>46</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="I4" s="0" t="s">
         <v>28</v>
@@ -2255,13 +2255,13 @@
         <v>47</v>
       </c>
       <c r="K4" s="0" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="L4" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M4" s="0" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N4" s="0" t="s">
         <v>31</v>
@@ -2276,30 +2276,30 @@
         <v>0</v>
       </c>
       <c r="V4" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0">
-        <v>1149367</v>
+        <v>1130592</v>
       </c>
       <c r="B5" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="E5" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="F5" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="0" t="s">
         <v>54</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="0" t="s">
-        <v>46</v>
       </c>
       <c r="H5" s="0" t="s">
         <v>39</v>
@@ -2308,7 +2308,7 @@
         <v>28</v>
       </c>
       <c r="J5" s="0" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="K5" s="0" t="s">
         <v>30</v>
@@ -2317,16 +2317,22 @@
         <v>31</v>
       </c>
       <c r="M5" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="N5" s="5">
+        <v>46087.776362002311</v>
+      </c>
+      <c r="O5" s="5">
+        <v>46087.7919412037</v>
+      </c>
+      <c r="P5" s="0" t="s">
         <v>55</v>
       </c>
-      <c r="N5" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="O5" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="0" t="s">
-        <v>28</v>
+      <c r="Q5" s="5">
+        <v>46130.416666666664</v>
+      </c>
+      <c r="R5" s="0">
+        <v>55</v>
       </c>
       <c r="U5" s="0">
         <v>0</v>
@@ -2337,7 +2343,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0">
-        <v>1130592</v>
+        <v>1147593</v>
       </c>
       <c r="B6" s="0" t="s">
         <v>57</v>
@@ -2355,7 +2361,7 @@
         <v>59</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="H6" s="0" t="s">
         <v>39</v>
@@ -2364,25 +2370,25 @@
         <v>28</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="K6" s="0" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="L6" s="0" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="M6" s="0" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="N6" s="5">
-        <v>46087.776362002311</v>
+        <v>46087.774690972219</v>
       </c>
       <c r="O6" s="5">
-        <v>46087.7919412037</v>
+        <v>46087.783132638884</v>
       </c>
       <c r="P6" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Q6" s="5">
         <v>46130.416666666664</v>
@@ -2394,116 +2400,116 @@
         <v>0</v>
       </c>
       <c r="V6" s="0" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0">
-        <v>1147593</v>
+        <v>1155551</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="J7" s="0" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="K7" s="0" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="L7" s="0" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M7" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="N7" s="5">
-        <v>46087.774690972219</v>
+        <v>46080.807078935184</v>
       </c>
       <c r="O7" s="5">
-        <v>46087.783132638884</v>
+        <v>46090.637796145835</v>
       </c>
       <c r="P7" s="0" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="Q7" s="5">
         <v>46130.416666666664</v>
       </c>
       <c r="R7" s="0">
-        <v>55</v>
+        <v>160</v>
       </c>
       <c r="U7" s="0">
         <v>0</v>
       </c>
       <c r="V7" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0">
-        <v>1155551</v>
+        <v>1155658</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G8" s="0" t="s">
         <v>26</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>77</v>
+        <v>39</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="J8" s="0" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="K8" s="0" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="N8" s="5">
-        <v>46080.807078935184</v>
+        <v>46087.777417476849</v>
       </c>
       <c r="O8" s="5">
-        <v>46090.637796145835</v>
+        <v>46087.804928587961</v>
       </c>
       <c r="P8" s="0" t="s">
         <v>80</v>
@@ -2512,7 +2518,7 @@
         <v>46130.416666666664</v>
       </c>
       <c r="R8" s="0">
-        <v>160</v>
+        <v>55</v>
       </c>
       <c r="U8" s="0">
         <v>0</v>
@@ -2523,7 +2529,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0">
-        <v>1155658</v>
+        <v>1134864</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>82</v>
@@ -2538,10 +2544,10 @@
         <v>85</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="H9" s="0" t="s">
         <v>39</v>
@@ -2553,25 +2559,25 @@
         <v>47</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L9" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="N9" s="5">
-        <v>46087.777417476849</v>
+        <v>46056.871177777779</v>
       </c>
       <c r="O9" s="5">
-        <v>46087.804928587961</v>
+        <v>46057.299867905094</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="Q9" s="5">
-        <v>46130.416666666664</v>
+        <v>46130.454861111109</v>
       </c>
       <c r="R9" s="0">
         <v>55</v>
@@ -2580,30 +2586,30 @@
         <v>0</v>
       </c>
       <c r="V9" s="0" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0">
-        <v>1134864</v>
+        <v>1141786</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="D10" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="E10" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="E10" s="0" t="s">
-        <v>92</v>
-      </c>
       <c r="F10" s="0" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="H10" s="0" t="s">
         <v>39</v>
@@ -2612,25 +2618,25 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="K10" s="0" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="L10" s="0" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="M10" s="0" t="s">
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="N10" s="5">
-        <v>46056.871177777779</v>
+        <v>46087.774690972219</v>
       </c>
       <c r="O10" s="5">
-        <v>46057.299867905094</v>
+        <v>46087.86314163194</v>
       </c>
       <c r="P10" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Q10" s="5">
         <v>46130.454861111109</v>
@@ -2647,7 +2653,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0">
-        <v>1141786</v>
+        <v>1148459</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>94</v>
@@ -2665,7 +2671,7 @@
         <v>96</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="H11" s="0" t="s">
         <v>39</v>
@@ -2677,22 +2683,22 @@
         <v>29</v>
       </c>
       <c r="K11" s="0" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="L11" s="0" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="M11" s="0" t="s">
-        <v>98</v>
+        <v>32</v>
       </c>
       <c r="N11" s="5">
-        <v>46087.774690972219</v>
-      </c>
-      <c r="O11" s="5">
-        <v>46087.86314163194</v>
+        <v>46087.777417476849</v>
+      </c>
+      <c r="O11" s="0" t="s">
+        <v>31</v>
       </c>
       <c r="P11" s="0" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="Q11" s="5">
         <v>46130.454861111109</v>
@@ -2709,7 +2715,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0">
-        <v>1148459</v>
+        <v>1098869</v>
       </c>
       <c r="B12" s="0" t="s">
         <v>100</v>
@@ -2733,90 +2739,90 @@
         <v>39</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="J12" s="0" t="s">
         <v>29</v>
       </c>
       <c r="K12" s="0" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="L12" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M12" s="0" t="s">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="N12" s="5">
-        <v>46087.777417476849</v>
-      </c>
-      <c r="O12" s="0" t="s">
-        <v>31</v>
+        <v>46044.86471519676</v>
+      </c>
+      <c r="O12" s="5">
+        <v>46044.872491863425</v>
       </c>
       <c r="P12" s="0" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="Q12" s="5">
-        <v>46130.454861111109</v>
+        <v>46130.493055555555</v>
       </c>
       <c r="R12" s="0">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="U12" s="0">
         <v>0</v>
       </c>
       <c r="V12" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0">
-        <v>1098869</v>
+        <v>1148344</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="H13" s="0" t="s">
         <v>39</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>109</v>
+        <v>28</v>
       </c>
       <c r="J13" s="0" t="s">
         <v>29</v>
       </c>
       <c r="K13" s="0" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="L13" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M13" s="0" t="s">
-        <v>110</v>
+        <v>32</v>
       </c>
       <c r="N13" s="5">
-        <v>46044.86471519676</v>
+        <v>46087.776362002311</v>
       </c>
       <c r="O13" s="5">
-        <v>46044.872491863425</v>
+        <v>46090.396714201386</v>
       </c>
       <c r="P13" s="0" t="s">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="Q13" s="5">
         <v>46130.493055555555</v>
@@ -2833,7 +2839,7 @@
     </row>
     <row r="14">
       <c r="A14" s="0">
-        <v>1148344</v>
+        <v>1155640</v>
       </c>
       <c r="B14" s="0" t="s">
         <v>112</v>
@@ -2848,10 +2854,10 @@
         <v>115</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="H14" s="0" t="s">
         <v>39</v>
@@ -2860,25 +2866,25 @@
         <v>28</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>29</v>
+        <v>117</v>
       </c>
       <c r="K14" s="0" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="M14" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N14" s="5">
-        <v>46087.776362002311</v>
+        <v>46087.774690972219</v>
       </c>
       <c r="O14" s="5">
-        <v>46090.396714201386</v>
+        <v>46090.30420543981</v>
       </c>
       <c r="P14" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Q14" s="5">
         <v>46130.493055555555</v>
@@ -2890,30 +2896,30 @@
         <v>0</v>
       </c>
       <c r="V14" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0">
-        <v>1155640</v>
+        <v>1129276</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F15" s="0" t="s">
         <v>121</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>38</v>
+        <v>123</v>
       </c>
       <c r="H15" s="0" t="s">
         <v>39</v>
@@ -2922,13 +2928,13 @@
         <v>28</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>122</v>
+        <v>29</v>
       </c>
       <c r="K15" s="0" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="M15" s="0" t="s">
         <v>32</v>
@@ -2937,13 +2943,13 @@
         <v>46087.774690972219</v>
       </c>
       <c r="O15" s="5">
-        <v>46090.30420543981</v>
+        <v>46088.308698113426</v>
       </c>
       <c r="P15" s="0" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="Q15" s="5">
-        <v>46130.493055555555</v>
+        <v>46130.583333333328</v>
       </c>
       <c r="R15" s="0">
         <v>50</v>
@@ -2952,30 +2958,30 @@
         <v>0</v>
       </c>
       <c r="V15" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0">
-        <v>1129276</v>
+        <v>1132787</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E16" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="F16" s="0" t="s">
         <v>127</v>
       </c>
-      <c r="F16" s="0" t="s">
-        <v>126</v>
-      </c>
       <c r="G16" s="0" t="s">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="H16" s="0" t="s">
         <v>39</v>
@@ -2984,25 +2990,25 @@
         <v>28</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="K16" s="0" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L16" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M16" s="0" t="s">
-        <v>32</v>
+        <v>129</v>
       </c>
       <c r="N16" s="5">
-        <v>46087.774690972219</v>
+        <v>46056.871177777779</v>
       </c>
       <c r="O16" s="5">
-        <v>46088.308698113426</v>
+        <v>46056.8941065162</v>
       </c>
       <c r="P16" s="0" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="Q16" s="5">
         <v>46130.583333333328</v>
@@ -3014,36 +3020,36 @@
         <v>0</v>
       </c>
       <c r="V16" s="0" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0">
-        <v>1132787</v>
+        <v>1133878</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E17" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="F17" s="0" t="s">
         <v>133</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>132</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>26</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="I17" s="0" t="s">
-        <v>28</v>
+        <v>135</v>
       </c>
       <c r="J17" s="0" t="s">
         <v>47</v>
@@ -3052,60 +3058,60 @@
         <v>30</v>
       </c>
       <c r="L17" s="0" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="M17" s="0" t="s">
-        <v>134</v>
+        <v>32</v>
       </c>
       <c r="N17" s="5">
-        <v>46056.871177777779</v>
+        <v>46085.527172766204</v>
       </c>
       <c r="O17" s="5">
-        <v>46056.8941065162</v>
+        <v>46085.540961030092</v>
       </c>
       <c r="P17" s="0" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="Q17" s="5">
         <v>46130.583333333328</v>
       </c>
       <c r="R17" s="0">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="U17" s="0">
         <v>0</v>
       </c>
       <c r="V17" s="0" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0">
-        <v>1133878</v>
+        <v>1148023</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="I18" s="0" t="s">
-        <v>140</v>
+        <v>28</v>
       </c>
       <c r="J18" s="0" t="s">
         <v>47</v>
@@ -3114,51 +3120,51 @@
         <v>30</v>
       </c>
       <c r="L18" s="0" t="s">
-        <v>69</v>
+        <v>31</v>
       </c>
       <c r="M18" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N18" s="5">
-        <v>46085.527172766204</v>
+        <v>46087.776362002311</v>
       </c>
       <c r="O18" s="5">
-        <v>46085.540961030092</v>
+        <v>46087.777946678238</v>
       </c>
       <c r="P18" s="0" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="Q18" s="5">
         <v>46130.583333333328</v>
       </c>
       <c r="R18" s="0">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="U18" s="0">
         <v>0</v>
       </c>
       <c r="V18" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0">
-        <v>1148023</v>
+        <v>1148693</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>46</v>
@@ -3179,19 +3185,19 @@
         <v>31</v>
       </c>
       <c r="M19" s="0" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="N19" s="5">
-        <v>46087.776362002311</v>
+        <v>46080.807078935184</v>
       </c>
       <c r="O19" s="5">
-        <v>46087.777946678238</v>
+        <v>46083.356493518513</v>
       </c>
       <c r="P19" s="0" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="Q19" s="5">
-        <v>46130.583333333328</v>
+        <v>46130.600694444445</v>
       </c>
       <c r="R19" s="0">
         <v>25</v>
@@ -3200,27 +3206,27 @@
         <v>0</v>
       </c>
       <c r="V19" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0">
-        <v>1148693</v>
+        <v>1149006</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E20" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="F20" s="0" t="s">
         <v>151</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>152</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>46</v>
@@ -3235,25 +3241,25 @@
         <v>47</v>
       </c>
       <c r="K20" s="0" t="s">
-        <v>30</v>
+        <v>98</v>
       </c>
       <c r="L20" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M20" s="0" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="N20" s="5">
-        <v>46080.807078935184</v>
-      </c>
-      <c r="O20" s="5">
-        <v>46083.356493518513</v>
+        <v>46087.776362002311</v>
+      </c>
+      <c r="O20" s="0" t="s">
+        <v>31</v>
       </c>
       <c r="P20" s="0" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="Q20" s="5">
-        <v>46130.600694444445</v>
+        <v>46130.618055555555</v>
       </c>
       <c r="R20" s="0">
         <v>25</v>
@@ -3267,7 +3273,7 @@
     </row>
     <row r="21">
       <c r="A21" s="0">
-        <v>1149006</v>
+        <v>1149336</v>
       </c>
       <c r="B21" s="0" t="s">
         <v>154</v>
@@ -3285,7 +3291,7 @@
         <v>156</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>46</v>
+        <v>123</v>
       </c>
       <c r="H21" s="0" t="s">
         <v>27</v>
@@ -3297,7 +3303,7 @@
         <v>47</v>
       </c>
       <c r="K21" s="0" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="L21" s="0" t="s">
         <v>31</v>
@@ -3306,13 +3312,13 @@
         <v>32</v>
       </c>
       <c r="N21" s="5">
-        <v>46087.776362002311</v>
-      </c>
-      <c r="O21" s="0" t="s">
-        <v>31</v>
+        <v>46087.774690972219</v>
+      </c>
+      <c r="O21" s="5">
+        <v>46087.965924965276</v>
       </c>
       <c r="P21" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="Q21" s="5">
         <v>46130.618055555555</v>
@@ -3329,7 +3335,7 @@
     </row>
     <row r="22">
       <c r="A22" s="0">
-        <v>1149336</v>
+        <v>1154402</v>
       </c>
       <c r="B22" s="0" t="s">
         <v>159</v>
@@ -3347,7 +3353,7 @@
         <v>161</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="H22" s="0" t="s">
         <v>27</v>
@@ -3359,7 +3365,7 @@
         <v>47</v>
       </c>
       <c r="K22" s="0" t="s">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="L22" s="0" t="s">
         <v>31</v>
@@ -3368,13 +3374,13 @@
         <v>32</v>
       </c>
       <c r="N22" s="5">
-        <v>46087.774690972219</v>
+        <v>46085.583816053237</v>
       </c>
       <c r="O22" s="5">
-        <v>46087.965924965276</v>
+        <v>46089.419183252314</v>
       </c>
       <c r="P22" s="0" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="Q22" s="5">
         <v>46130.618055555555</v>
@@ -3391,7 +3397,7 @@
     </row>
     <row r="23">
       <c r="A23" s="0">
-        <v>1154402</v>
+        <v>1148589</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>164</v>
@@ -3406,10 +3412,10 @@
         <v>167</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>26</v>
+        <v>169</v>
       </c>
       <c r="H23" s="0" t="s">
         <v>27</v>
@@ -3418,10 +3424,10 @@
         <v>28</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="K23" s="0" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="L23" s="0" t="s">
         <v>31</v>
@@ -3430,16 +3436,16 @@
         <v>32</v>
       </c>
       <c r="N23" s="5">
-        <v>46085.583816053237</v>
+        <v>46080.807078935184</v>
       </c>
       <c r="O23" s="5">
-        <v>46089.419183252314</v>
+        <v>46083.334888888887</v>
       </c>
       <c r="P23" s="0" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="Q23" s="5">
-        <v>46130.618055555555</v>
+        <v>46130.635416666664</v>
       </c>
       <c r="R23" s="0">
         <v>25</v>
@@ -3448,30 +3454,30 @@
         <v>0</v>
       </c>
       <c r="V23" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0">
-        <v>1148589</v>
+        <v>1149301</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F24" s="0" t="s">
         <v>173</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="H24" s="0" t="s">
         <v>27</v>
@@ -3480,25 +3486,25 @@
         <v>28</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>29</v>
+        <v>47</v>
       </c>
       <c r="K24" s="0" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="L24" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M24" s="0" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="N24" s="5">
-        <v>46080.807078935184</v>
+        <v>46095.713437997685</v>
       </c>
       <c r="O24" s="5">
-        <v>46083.334888888887</v>
+        <v>46095.732204745371</v>
       </c>
       <c r="P24" s="0" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="Q24" s="5">
         <v>46130.635416666664</v>
@@ -3560,7 +3566,7 @@
         <v>46090.663122534723</v>
       </c>
       <c r="P25" s="0" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="Q25" s="5">
         <v>46130.635416666664</v>
@@ -3622,7 +3628,7 @@
         <v>46087.779189814813</v>
       </c>
       <c r="P26" s="0" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="Q26" s="5">
         <v>46130.652777777774</v>
@@ -3657,7 +3663,7 @@
         <v>188</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="H27" s="0" t="s">
         <v>39</v>
@@ -3669,13 +3675,13 @@
         <v>47</v>
       </c>
       <c r="K27" s="0" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="L27" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M27" s="0" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="N27" s="5">
         <v>46080.807078935184</v>
@@ -3684,7 +3690,7 @@
         <v>46090.182709374996</v>
       </c>
       <c r="P27" s="0" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="Q27" s="5">
         <v>46130.652777777774</v>
@@ -3746,7 +3752,7 @@
         <v>46046.3336130787</v>
       </c>
       <c r="P28" s="0" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="Q28" s="5">
         <v>46130.670138888891</v>
@@ -3781,7 +3787,7 @@
         <v>199</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="H29" s="0" t="s">
         <v>39</v>
@@ -3808,7 +3814,7 @@
         <v>46087.792176655094</v>
       </c>
       <c r="P29" s="0" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="Q29" s="5">
         <v>46130.708333333328</v>
@@ -3855,7 +3861,7 @@
         <v>47</v>
       </c>
       <c r="K30" s="0" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="L30" s="0" t="s">
         <v>31</v>
@@ -3870,7 +3876,7 @@
         <v>46058.74419375</v>
       </c>
       <c r="P30" s="0" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="Q30" s="5">
         <v>46130.708333333328</v>
@@ -3932,7 +3938,7 @@
         <v>46087.79654938657</v>
       </c>
       <c r="P31" s="0" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="Q31" s="5">
         <v>46130.708333333328</v>
@@ -3976,7 +3982,7 @@
         <v>28</v>
       </c>
       <c r="J32" s="0" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="K32" s="0" t="s">
         <v>30</v>
@@ -3994,7 +4000,7 @@
         <v>46045.370912303239</v>
       </c>
       <c r="P32" s="0" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="Q32" s="5">
         <v>46130.743055555555</v>
@@ -4029,7 +4035,7 @@
         <v>220</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="H33" s="0" t="s">
         <v>39</v>
@@ -4041,10 +4047,10 @@
         <v>47</v>
       </c>
       <c r="K33" s="0" t="s">
-        <v>48</v>
+        <v>98</v>
       </c>
       <c r="L33" s="0" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="M33" s="0" t="s">
         <v>222</v>
@@ -4056,7 +4062,7 @@
         <v>46076.880179664353</v>
       </c>
       <c r="P33" s="0" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="Q33" s="5">
         <v>46130.743055555555</v>
@@ -4118,7 +4124,7 @@
         <v>46088.7549028125</v>
       </c>
       <c r="P34" s="0" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="Q34" s="5">
         <v>46130.743055555555</v>
@@ -4183,7 +4189,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>242</v>
@@ -4192,7 +4198,7 @@
         <v>243</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="E2" s="0" t="s">
         <v>244</v>
@@ -4212,7 +4218,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>248</v>
@@ -4221,7 +4227,7 @@
         <v>249</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E3" s="0" t="s">
         <v>250</v>
@@ -4421,7 +4427,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>305</v>
@@ -4430,7 +4436,7 @@
         <v>306</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E10" s="0" t="s">
         <v>307</v>
@@ -4453,7 +4459,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>313</v>
@@ -4462,7 +4468,7 @@
         <v>314</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E11" s="0" t="s">
         <v>315</v>
@@ -4529,7 +4535,7 @@
         <v>333</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="E13" s="0" t="s">
         <v>334</v>
@@ -4616,7 +4622,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>358</v>
@@ -4625,7 +4631,7 @@
         <v>359</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="E16" s="0" t="s">
         <v>360</v>
@@ -4721,7 +4727,7 @@
         <v>386</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E19" s="0" t="s">
         <v>387</v>
@@ -4750,7 +4756,7 @@
         <v>394</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="E20" s="0" t="s">
         <v>395</v>
@@ -4819,7 +4825,7 @@
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>50</v>
+        <v>175</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>412</v>
@@ -4828,7 +4834,7 @@
         <v>413</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>45</v>
+        <v>174</v>
       </c>
       <c r="E23" s="0" t="s">
         <v>414</v>
@@ -4883,7 +4889,7 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>428</v>
@@ -4892,7 +4898,7 @@
         <v>429</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="E25" s="0" t="s">
         <v>430</v>
@@ -4950,7 +4956,7 @@
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B27" s="0" t="s">
         <v>428</v>
@@ -4959,7 +4965,7 @@
         <v>445</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="E27" s="0" t="s">
         <v>446</v>
@@ -4982,7 +4988,7 @@
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B28" s="0" t="s">
         <v>452</v>
@@ -4991,7 +4997,7 @@
         <v>453</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E28" s="0" t="s">
         <v>454</v>
@@ -5020,7 +5026,7 @@
         <v>461</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E29" s="0" t="s">
         <v>462</v>
@@ -5110,7 +5116,7 @@
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B32" s="0" t="s">
         <v>487</v>
@@ -5119,7 +5125,7 @@
         <v>488</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E32" s="0" t="s">
         <v>489</v>
@@ -5174,7 +5180,7 @@
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B34" s="0" t="s">
         <v>502</v>
@@ -5183,7 +5189,7 @@
         <v>503</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="E34" s="0" t="s">
         <v>504</v>
@@ -5241,7 +5247,7 @@
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B36" s="0" t="s">
         <v>519</v>
@@ -5250,7 +5256,7 @@
         <v>520</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="E36" s="0" t="s">
         <v>521</v>
@@ -5279,7 +5285,7 @@
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B37" s="0" t="s">
         <v>529</v>
@@ -5288,7 +5294,7 @@
         <v>530</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E37" s="0" t="s">
         <v>531</v>
@@ -5343,7 +5349,7 @@
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B39" s="0" t="s">
         <v>436</v>
@@ -5352,7 +5358,7 @@
         <v>547</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="E39" s="0" t="s">
         <v>548</v>
@@ -5384,7 +5390,7 @@
         <v>556</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="E40" s="0" t="s">
         <v>557</v>
@@ -5404,7 +5410,7 @@
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B41" s="0" t="s">
         <v>562</v>
@@ -5413,7 +5419,7 @@
         <v>563</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E41" s="0" t="s">
         <v>564</v>
@@ -5442,7 +5448,7 @@
     </row>
     <row r="42">
       <c r="A42" s="0" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B42" s="0" t="s">
         <v>571</v>
@@ -5451,7 +5457,7 @@
         <v>572</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="E42" s="0" t="s">
         <v>573</v>

</xml_diff>

<commit_message>
update session languages and speaker blog links
</commit_message>
<xml_diff>
--- a/src/assets/sessionize/data-advanced.xlsx
+++ b/src/assets/sessionize/data-advanced.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="553">
   <si>
     <t>Session Id</t>
   </si>
@@ -203,9 +203,6 @@
     <t>Short (20min)</t>
   </si>
   <si>
-    <t>English, Italian</t>
-  </si>
-  <si>
     <t>9ef3c98b-1d3d-482e-97c0-7489ff355bd8</t>
   </si>
   <si>
@@ -238,9 +235,6 @@
   </si>
   <si>
     <t>me@gionn.net</t>
-  </si>
-  <si>
-    <t>Italian, English</t>
   </si>
   <si>
     <t>b11e5877-5635-4943-8a71-3ea1a8a1908f</t>
@@ -584,6 +578,9 @@
     <t>jack.lilhammers@gmail.com</t>
   </si>
   <si>
+    <t>English, Italian</t>
+  </si>
+  <si>
     <t>82b493da-0b26-4e1f-9c81-54c9609a4b50</t>
   </si>
   <si>
@@ -856,12 +853,12 @@
     <t>Company Website</t>
   </si>
   <si>
+    <t>Instagram</t>
+  </si>
+  <si>
     <t>Blog</t>
   </si>
   <si>
-    <t>Instagram</t>
-  </si>
-  <si>
     <t>Facebook</t>
   </si>
   <si>
@@ -904,7 +901,7 @@
     <t>https://www.klarna.com/it/</t>
   </si>
   <si>
-    <t>https://sessionize.com/image/156d-400o400o1-GVgNeZWye39woHvSTXjmFS.jpg</t>
+    <t>https://sessionize.com/image/d9c1-400o400o1-suawNqFLCc9haUwdaT2PBf.png</t>
   </si>
   <si>
     <t>05ed4b4a-5d57-4602-bb4e-8d55efad3e0f</t>
@@ -933,10 +930,10 @@
     <t>https://devdojo.it</t>
   </si>
   <si>
+    <t>https://www.instagram.com/pixu1980/</t>
+  </si>
+  <si>
     <t>https://dout.dev</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/pixu1980/</t>
   </si>
   <si>
     <t>https://sessionize.com/image/fd3b-400o400o1-BwkHXp3qRbEw3D5V2gPbAY.png</t>
@@ -1136,10 +1133,10 @@
     <t>https://fractal.cloud</t>
   </si>
   <si>
+    <t>https://www.instagram.com/michel_murabito/</t>
+  </si>
+  <si>
     <t>https://michelmurabito.com</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/michel_murabito/</t>
   </si>
   <si>
     <t>https://www.facebook.com/michelmurabito</t>
@@ -1225,10 +1222,10 @@
     <t>https://bit.ly/pantarei-mb</t>
   </si>
   <si>
+    <t>https://instagram.com/pantarei_mb</t>
+  </si>
+  <si>
     <t>https://sites.google.com/view/pantarei-mb-en/blog</t>
-  </si>
-  <si>
-    <t>https://instagram.com/pantarei_mb</t>
   </si>
   <si>
     <t>https://sessionize.com/image/677e-400o400o1-shpurTgXp4EfDBWu3fPXrZ.jpg</t>
@@ -1448,10 +1445,10 @@
     <t>https://pescara.python.it/</t>
   </si>
   <si>
+    <t>https://www.instagram.com/luca_di_vita_</t>
+  </si>
+  <si>
     <t>https://www.lucadivita.it/</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/luca_di_vita_</t>
   </si>
   <si>
     <t>https://sessionize.com/image/77c6-400o400o1-hMWZzLKMh7xt3XWNZALNnt.jpg</t>
@@ -1528,10 +1525,10 @@
     <t>https://devmy.it</t>
   </si>
   <si>
+    <t>https://www.instagram.com/Devmy.it/</t>
+  </si>
+  <si>
     <t>https://devmy.it/blog</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/Devmy.it/</t>
   </si>
   <si>
     <t>https://www.facebook.com/francesco.sciuti/</t>
@@ -1661,10 +1658,10 @@
     <t>https://monjadariva.it</t>
   </si>
   <si>
+    <t>https://instagram.com/monja.dariva</t>
+  </si>
+  <si>
     <t>https://monjadariva.it/blog</t>
-  </si>
-  <si>
-    <t>https://instagram.com/monja.dariva</t>
   </si>
   <si>
     <t>https://sessionize.com/image/3e16-400o400o1-7jvdkF5R8VCzcbkb33Ty6R.jpg</t>
@@ -1713,12 +1710,12 @@
     <t>https://www.mann-ai.com/</t>
   </si>
   <si>
+    <t>https://www.instagram.com/mortadha_mannai/</t>
+  </si>
+  <si>
     <t>https://manaimortadha.medium.com/</t>
   </si>
   <si>
-    <t>https://www.instagram.com/mortadha_mannai/</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/profile.php?id=100004306062352</t>
   </si>
   <si>
@@ -1743,10 +1740,10 @@
     <t>https://www.thinktecture.com</t>
   </si>
   <si>
+    <t>https://www.instagram.com/chliebel/</t>
+  </si>
+  <si>
     <t>https://christianliebel.com</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/chliebel/</t>
   </si>
   <si>
     <t>https://www.facebook.com/christianliebel</t>
@@ -2244,7 +2241,7 @@
         <v>50</v>
       </c>
       <c r="K5" s="0" t="s">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="L5" s="0" t="s">
         <v>31</v>
@@ -2271,7 +2268,7 @@
         <v>0</v>
       </c>
       <c r="V5" s="0" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -2279,10 +2276,10 @@
         <v>1155551</v>
       </c>
       <c r="B6" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="0" t="s">
         <v>61</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>62</v>
       </c>
       <c r="D6" s="0" t="s">
         <v>37</v>
@@ -2297,10 +2294,10 @@
         <v>39</v>
       </c>
       <c r="H6" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="I6" s="0" t="s">
         <v>63</v>
-      </c>
-      <c r="I6" s="0" t="s">
-        <v>64</v>
       </c>
       <c r="J6" s="0" t="s">
         <v>29</v>
@@ -2321,7 +2318,7 @@
         <v>46090.637796145835</v>
       </c>
       <c r="P6" s="0" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Q6" s="5">
         <v>46130.4375</v>
@@ -2341,19 +2338,19 @@
         <v>1129276</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="D7" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="E7" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="E7" s="0" t="s">
-        <v>69</v>
-      </c>
       <c r="F7" s="0" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G7" s="0" t="s">
         <v>57</v>
@@ -2368,7 +2365,7 @@
         <v>29</v>
       </c>
       <c r="K7" s="0" t="s">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="L7" s="0" t="s">
         <v>31</v>
@@ -2395,7 +2392,7 @@
         <v>0</v>
       </c>
       <c r="V7" s="0" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8">
@@ -2403,22 +2400,22 @@
         <v>1134864</v>
       </c>
       <c r="B8" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="0" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="E8" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="F8" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="0" t="s">
         <v>74</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>74</v>
-      </c>
-      <c r="G8" s="0" t="s">
-        <v>76</v>
       </c>
       <c r="H8" s="0" t="s">
         <v>27</v>
@@ -2436,7 +2433,7 @@
         <v>31</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N8" s="5">
         <v>46056.871177777779</v>
@@ -2457,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="V8" s="0" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9">
@@ -2465,19 +2462,19 @@
         <v>1148459</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="E9" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="D9" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="0" t="s">
-        <v>82</v>
-      </c>
       <c r="F9" s="0" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>39</v>
@@ -2519,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="V9" s="0" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10">
@@ -2527,19 +2524,19 @@
         <v>1098869</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="E10" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="D10" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>87</v>
-      </c>
       <c r="F10" s="0" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G10" s="0" t="s">
         <v>39</v>
@@ -2548,7 +2545,7 @@
         <v>27</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="J10" s="0" t="s">
         <v>29</v>
@@ -2560,7 +2557,7 @@
         <v>31</v>
       </c>
       <c r="M10" s="0" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="N10" s="5">
         <v>46044.86471519676</v>
@@ -2581,7 +2578,7 @@
         <v>0</v>
       </c>
       <c r="V10" s="0" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11">
@@ -2589,22 +2586,22 @@
         <v>1141786</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="E11" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="F11" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="0" t="s">
         <v>93</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="F11" s="0" t="s">
-        <v>93</v>
-      </c>
-      <c r="G11" s="0" t="s">
-        <v>95</v>
       </c>
       <c r="H11" s="0" t="s">
         <v>27</v>
@@ -2622,7 +2619,7 @@
         <v>41</v>
       </c>
       <c r="M11" s="0" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="N11" s="5">
         <v>46087.774690972219</v>
@@ -2643,7 +2640,7 @@
         <v>0</v>
       </c>
       <c r="V11" s="0" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12">
@@ -2651,22 +2648,22 @@
         <v>1148344</v>
       </c>
       <c r="B12" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="E12" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="D12" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>101</v>
-      </c>
       <c r="F12" s="0" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H12" s="0" t="s">
         <v>27</v>
@@ -2705,7 +2702,7 @@
         <v>0</v>
       </c>
       <c r="V12" s="0" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -2713,19 +2710,19 @@
         <v>1132787</v>
       </c>
       <c r="B13" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="E13" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="0" t="s">
-        <v>105</v>
-      </c>
-      <c r="E13" s="0" t="s">
-        <v>106</v>
-      </c>
       <c r="F13" s="0" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="G13" s="0" t="s">
         <v>39</v>
@@ -2746,7 +2743,7 @@
         <v>31</v>
       </c>
       <c r="M13" s="0" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="N13" s="5">
         <v>46056.871177777779</v>
@@ -2767,7 +2764,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="0" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14">
@@ -2775,28 +2772,28 @@
         <v>1133878</v>
       </c>
       <c r="B14" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="D14" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="E14" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="D14" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="E14" s="0" t="s">
-        <v>112</v>
-      </c>
       <c r="F14" s="0" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G14" s="0" t="s">
         <v>39</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I14" s="0" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J14" s="0" t="s">
         <v>50</v>
@@ -2817,7 +2814,7 @@
         <v>46085.540961030092</v>
       </c>
       <c r="P14" s="0" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Q14" s="5">
         <v>46130.583333333328</v>
@@ -2829,7 +2826,7 @@
         <v>0</v>
       </c>
       <c r="V14" s="0" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15">
@@ -2837,22 +2834,22 @@
         <v>1148023</v>
       </c>
       <c r="B15" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="D15" s="0" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="E15" s="0" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="F15" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="E15" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="F15" s="0" t="s">
-        <v>119</v>
-      </c>
       <c r="G15" s="0" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H15" s="0" t="s">
         <v>58</v>
@@ -2891,7 +2888,7 @@
         <v>0</v>
       </c>
       <c r="V15" s="0" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16">
@@ -2899,22 +2896,22 @@
         <v>1155640</v>
       </c>
       <c r="B16" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="0" t="s">
         <v>121</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="E16" s="0" t="s">
         <v>122</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="F16" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="E16" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="F16" s="0" t="s">
-        <v>125</v>
-      </c>
       <c r="G16" s="0" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H16" s="0" t="s">
         <v>27</v>
@@ -2923,7 +2920,7 @@
         <v>28</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K16" s="0" t="s">
         <v>30</v>
@@ -2953,7 +2950,7 @@
         <v>0</v>
       </c>
       <c r="V16" s="0" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17">
@@ -2961,22 +2958,22 @@
         <v>1148693</v>
       </c>
       <c r="B17" s="0" t="s">
+        <v>126</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="D17" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="E17" s="0" t="s">
         <v>129</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="F17" s="0" t="s">
         <v>130</v>
       </c>
-      <c r="E17" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>132</v>
-      </c>
       <c r="G17" s="0" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H17" s="0" t="s">
         <v>58</v>
@@ -2994,7 +2991,7 @@
         <v>31</v>
       </c>
       <c r="M17" s="0" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N17" s="5">
         <v>46080.807078935184</v>
@@ -3015,7 +3012,7 @@
         <v>0</v>
       </c>
       <c r="V17" s="0" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18">
@@ -3023,22 +3020,22 @@
         <v>1147593</v>
       </c>
       <c r="B18" s="0" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="E18" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="D18" s="0" t="s">
-        <v>136</v>
-      </c>
-      <c r="E18" s="0" t="s">
-        <v>137</v>
-      </c>
       <c r="F18" s="0" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H18" s="0" t="s">
         <v>27</v>
@@ -3056,7 +3053,7 @@
         <v>41</v>
       </c>
       <c r="M18" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="N18" s="5">
         <v>46087.774690972219</v>
@@ -3077,7 +3074,7 @@
         <v>0</v>
       </c>
       <c r="V18" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19">
@@ -3085,22 +3082,22 @@
         <v>1149006</v>
       </c>
       <c r="B19" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="D19" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="E19" s="0" t="s">
         <v>141</v>
       </c>
-      <c r="D19" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="E19" s="0" t="s">
-        <v>143</v>
-      </c>
       <c r="F19" s="0" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H19" s="0" t="s">
         <v>58</v>
@@ -3112,7 +3109,7 @@
         <v>50</v>
       </c>
       <c r="K19" s="0" t="s">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="L19" s="0" t="s">
         <v>31</v>
@@ -3123,8 +3120,8 @@
       <c r="N19" s="5">
         <v>46087.776362002311</v>
       </c>
-      <c r="O19" s="0" t="s">
-        <v>31</v>
+      <c r="O19" s="5">
+        <v>46103.887877349538</v>
       </c>
       <c r="P19" s="0" t="s">
         <v>33</v>
@@ -3139,7 +3136,7 @@
         <v>0</v>
       </c>
       <c r="V19" s="0" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20">
@@ -3147,19 +3144,19 @@
         <v>1154402</v>
       </c>
       <c r="B20" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="0" t="s">
         <v>145</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="E20" s="0" t="s">
         <v>146</v>
       </c>
-      <c r="D20" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>148</v>
-      </c>
       <c r="F20" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>39</v>
@@ -3201,7 +3198,7 @@
         <v>0</v>
       </c>
       <c r="V20" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21">
@@ -3209,22 +3206,22 @@
         <v>1149301</v>
       </c>
       <c r="B21" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="D21" s="0" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="E21" s="0" t="s">
         <v>151</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="E21" s="0" t="s">
-        <v>153</v>
-      </c>
       <c r="F21" s="0" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H21" s="0" t="s">
         <v>58</v>
@@ -3236,13 +3233,13 @@
         <v>50</v>
       </c>
       <c r="K21" s="0" t="s">
-        <v>59</v>
+        <v>152</v>
       </c>
       <c r="L21" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M21" s="0" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N21" s="5">
         <v>46095.713437997685</v>
@@ -3263,7 +3260,7 @@
         <v>0</v>
       </c>
       <c r="V21" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22">
@@ -3271,19 +3268,19 @@
         <v>1149383</v>
       </c>
       <c r="B22" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="C22" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="D22" s="0" t="s">
         <v>156</v>
       </c>
-      <c r="D22" s="0" t="s">
+      <c r="E22" s="0" t="s">
         <v>157</v>
       </c>
-      <c r="E22" s="0" t="s">
-        <v>158</v>
-      </c>
       <c r="F22" s="0" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G22" s="0" t="s">
         <v>39</v>
@@ -3325,7 +3322,7 @@
         <v>0</v>
       </c>
       <c r="V22" s="0" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23">
@@ -3333,19 +3330,19 @@
         <v>1151362</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="0" t="s">
         <v>160</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="D23" s="0" t="s">
         <v>161</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="E23" s="0" t="s">
         <v>162</v>
       </c>
-      <c r="E23" s="0" t="s">
-        <v>163</v>
-      </c>
       <c r="F23" s="0" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>39</v>
@@ -3387,7 +3384,7 @@
         <v>0</v>
       </c>
       <c r="V23" s="0" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24">
@@ -3395,22 +3392,22 @@
         <v>1155630</v>
       </c>
       <c r="B24" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="C24" s="0" t="s">
         <v>165</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="D24" s="0" t="s">
         <v>166</v>
       </c>
-      <c r="D24" s="0" t="s">
+      <c r="E24" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="F24" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="G24" s="0" t="s">
         <v>168</v>
-      </c>
-      <c r="F24" s="0" t="s">
-        <v>167</v>
-      </c>
-      <c r="G24" s="0" t="s">
-        <v>169</v>
       </c>
       <c r="H24" s="0" t="s">
         <v>27</v>
@@ -3428,7 +3425,7 @@
         <v>31</v>
       </c>
       <c r="M24" s="0" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="N24" s="5">
         <v>46080.807078935184</v>
@@ -3449,7 +3446,7 @@
         <v>0</v>
       </c>
       <c r="V24" s="0" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25">
@@ -3457,22 +3454,22 @@
         <v>1105608</v>
       </c>
       <c r="B25" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="C25" s="0" t="s">
         <v>171</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="D25" s="0" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="E25" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="E25" s="0" t="s">
+      <c r="F25" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="G25" s="0" t="s">
         <v>174</v>
-      </c>
-      <c r="F25" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="G25" s="0" t="s">
-        <v>175</v>
       </c>
       <c r="H25" s="0" t="s">
         <v>58</v>
@@ -3511,7 +3508,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26">
@@ -3519,19 +3516,19 @@
         <v>1145869</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>177</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="D26" s="0" t="s">
         <v>178</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="E26" s="0" t="s">
         <v>179</v>
       </c>
-      <c r="E26" s="0" t="s">
-        <v>180</v>
-      </c>
       <c r="F26" s="0" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G26" s="0" t="s">
         <v>39</v>
@@ -3573,7 +3570,7 @@
         <v>0</v>
       </c>
       <c r="V26" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27">
@@ -3581,22 +3578,22 @@
         <v>1124260</v>
       </c>
       <c r="B27" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="C27" s="0" t="s">
         <v>182</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="D27" s="0" t="s">
         <v>183</v>
       </c>
-      <c r="D27" s="0" t="s">
+      <c r="E27" s="0" t="s">
         <v>184</v>
       </c>
-      <c r="E27" s="0" t="s">
-        <v>185</v>
-      </c>
       <c r="F27" s="0" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H27" s="0" t="s">
         <v>27</v>
@@ -3635,7 +3632,7 @@
         <v>0</v>
       </c>
       <c r="V27" s="0" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28">
@@ -3643,22 +3640,22 @@
         <v>1125184</v>
       </c>
       <c r="B28" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="C28" s="0" t="s">
         <v>187</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="D28" s="0" t="s">
         <v>188</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="E28" s="0" t="s">
         <v>189</v>
       </c>
-      <c r="E28" s="0" t="s">
+      <c r="F28" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="G28" s="0" t="s">
         <v>190</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>189</v>
-      </c>
-      <c r="G28" s="0" t="s">
-        <v>191</v>
       </c>
       <c r="H28" s="0" t="s">
         <v>27</v>
@@ -3697,7 +3694,7 @@
         <v>0</v>
       </c>
       <c r="V28" s="0" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29">
@@ -3705,19 +3702,19 @@
         <v>1147845</v>
       </c>
       <c r="B29" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="C29" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="D29" s="0" t="s">
         <v>194</v>
       </c>
-      <c r="D29" s="0" t="s">
+      <c r="E29" s="0" t="s">
         <v>195</v>
       </c>
-      <c r="E29" s="0" t="s">
-        <v>196</v>
-      </c>
       <c r="F29" s="0" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>39</v>
@@ -3759,7 +3756,7 @@
         <v>0</v>
       </c>
       <c r="V29" s="0" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30">
@@ -3767,19 +3764,19 @@
         <v>1093465</v>
       </c>
       <c r="B30" s="0" t="s">
+        <v>197</v>
+      </c>
+      <c r="C30" s="0" t="s">
         <v>198</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="D30" s="0" t="s">
         <v>199</v>
       </c>
-      <c r="D30" s="0" t="s">
+      <c r="E30" s="0" t="s">
         <v>200</v>
       </c>
-      <c r="E30" s="0" t="s">
-        <v>201</v>
-      </c>
       <c r="F30" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G30" s="0" t="s">
         <v>39</v>
@@ -3791,7 +3788,7 @@
         <v>28</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K30" s="0" t="s">
         <v>30</v>
@@ -3821,7 +3818,7 @@
         <v>0</v>
       </c>
       <c r="V30" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="31">
@@ -3829,22 +3826,22 @@
         <v>1148589</v>
       </c>
       <c r="B31" s="0" t="s">
+        <v>202</v>
+      </c>
+      <c r="C31" s="0" t="s">
         <v>203</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="D31" s="0" t="s">
         <v>204</v>
       </c>
-      <c r="D31" s="0" t="s">
+      <c r="E31" s="0" t="s">
         <v>205</v>
       </c>
-      <c r="E31" s="0" t="s">
+      <c r="F31" s="0" t="s">
         <v>206</v>
       </c>
-      <c r="F31" s="0" t="s">
-        <v>207</v>
-      </c>
       <c r="G31" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H31" s="0" t="s">
         <v>58</v>
@@ -3883,7 +3880,7 @@
         <v>0</v>
       </c>
       <c r="V31" s="0" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="32">
@@ -3891,22 +3888,22 @@
         <v>1154675</v>
       </c>
       <c r="B32" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="C32" s="0" t="s">
         <v>209</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="D32" s="0" t="s">
         <v>210</v>
       </c>
-      <c r="D32" s="0" t="s">
+      <c r="E32" s="0" t="s">
         <v>211</v>
       </c>
-      <c r="E32" s="0" t="s">
+      <c r="F32" s="0" t="s">
         <v>212</v>
       </c>
-      <c r="F32" s="0" t="s">
-        <v>213</v>
-      </c>
       <c r="G32" s="0" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H32" s="0" t="s">
         <v>27</v>
@@ -3945,7 +3942,7 @@
         <v>0</v>
       </c>
       <c r="V32" s="0" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="33">
@@ -3953,22 +3950,22 @@
         <v>1143717</v>
       </c>
       <c r="B33" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="C33" s="0" t="s">
         <v>215</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="D33" s="0" t="s">
         <v>216</v>
       </c>
-      <c r="D33" s="0" t="s">
+      <c r="E33" s="0" t="s">
         <v>217</v>
       </c>
-      <c r="E33" s="0" t="s">
-        <v>218</v>
-      </c>
       <c r="F33" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H33" s="0" t="s">
         <v>58</v>
@@ -3986,7 +3983,7 @@
         <v>41</v>
       </c>
       <c r="M33" s="0" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="N33" s="5">
         <v>46063.895173379628</v>
@@ -4007,7 +4004,7 @@
         <v>0</v>
       </c>
       <c r="V33" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -4022,278 +4019,278 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B2" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>233</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="D2" s="0" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="0" t="s">
         <v>234</v>
       </c>
-      <c r="D2" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="0" t="s">
+      <c r="F2" s="0" t="s">
         <v>235</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G2" s="0" t="s">
         <v>236</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H2" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="L2" s="0" t="s">
         <v>237</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>237</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B3" s="0" t="s">
+        <v>238</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>239</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="D3" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="0" t="s">
         <v>240</v>
       </c>
-      <c r="D3" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="E3" s="0" t="s">
+      <c r="F3" s="0" t="s">
         <v>241</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="G3" s="0" t="s">
         <v>242</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="H3" s="0" t="s">
         <v>243</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="L3" s="0" t="s">
         <v>244</v>
-      </c>
-      <c r="L3" s="0" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>246</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="C4" s="0" t="s">
         <v>247</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="D4" s="0" t="s">
         <v>248</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="E4" s="0" t="s">
         <v>249</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="F4" s="0" t="s">
         <v>250</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="G4" s="0" t="s">
         <v>251</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="H4" s="0" t="s">
         <v>252</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="I4" s="0" t="s">
         <v>253</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="J4" s="0" t="s">
         <v>254</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="L4" s="0" t="s">
         <v>255</v>
-      </c>
-      <c r="L4" s="0" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="B5" s="0" t="s">
         <v>257</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="C5" s="0" t="s">
         <v>258</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>259</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="E5" s="0" t="s">
         <v>260</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="F5" s="0" t="s">
         <v>261</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="G5" s="0" t="s">
         <v>262</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="H5" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="L5" s="0" t="s">
         <v>264</v>
-      </c>
-      <c r="L5" s="0" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B6" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="C6" s="0" t="s">
         <v>266</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="D6" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>267</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>196</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="F6" s="0" t="s">
         <v>268</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="G6" s="0" t="s">
         <v>269</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="H6" s="0" t="s">
         <v>270</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="J6" s="0" t="s">
         <v>271</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="L6" s="0" t="s">
         <v>272</v>
-      </c>
-      <c r="L6" s="0" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>273</v>
+      </c>
+      <c r="C7" s="0" t="s">
         <v>274</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="D7" s="0" t="s">
+        <v>167</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>275</v>
       </c>
-      <c r="D7" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="E7" s="0" t="s">
+      <c r="F7" s="0" t="s">
         <v>276</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="G7" s="0" t="s">
         <v>277</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="L7" s="0" t="s">
         <v>278</v>
-      </c>
-      <c r="L7" s="0" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>280</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="C8" s="0" t="s">
         <v>281</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="D8" s="0" t="s">
         <v>282</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="E8" s="0" t="s">
         <v>283</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="F8" s="0" t="s">
         <v>284</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="G8" s="0" t="s">
         <v>285</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="H8" s="0" t="s">
         <v>286</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="L8" s="0" t="s">
         <v>287</v>
-      </c>
-      <c r="L8" s="0" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>289</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="D9" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="E9" s="0" t="s">
         <v>290</v>
       </c>
-      <c r="D9" s="0" t="s">
-        <v>158</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="F9" s="0" t="s">
         <v>291</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="G9" s="0" t="s">
         <v>292</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="H9" s="0" t="s">
         <v>293</v>
       </c>
-      <c r="H9" s="0" t="s">
+      <c r="L9" s="0" t="s">
         <v>294</v>
-      </c>
-      <c r="L9" s="0" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="10">
@@ -4301,953 +4298,953 @@
         <v>34</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>295</v>
+      </c>
+      <c r="C10" s="0" t="s">
         <v>296</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>297</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>25</v>
       </c>
       <c r="E10" s="0" t="s">
+        <v>297</v>
+      </c>
+      <c r="F10" s="0" t="s">
         <v>298</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="G10" s="0" t="s">
         <v>299</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="H10" s="0" t="s">
         <v>300</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="J10" s="0" t="s">
         <v>301</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="L10" s="0" t="s">
         <v>302</v>
-      </c>
-      <c r="L10" s="0" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>303</v>
+      </c>
+      <c r="C11" s="0" t="s">
         <v>304</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="D11" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="E11" s="0" t="s">
         <v>305</v>
       </c>
-      <c r="D11" s="0" t="s">
-        <v>148</v>
-      </c>
-      <c r="E11" s="0" t="s">
+      <c r="F11" s="0" t="s">
         <v>306</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="G11" s="0" t="s">
         <v>307</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="I11" s="0" t="s">
         <v>308</v>
       </c>
-      <c r="J11" s="0" t="s">
+      <c r="L11" s="0" t="s">
         <v>309</v>
-      </c>
-      <c r="L11" s="0" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
+        <v>310</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>311</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="C12" s="0" t="s">
         <v>312</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="D12" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="E12" s="0" t="s">
         <v>313</v>
       </c>
-      <c r="D12" s="0" t="s">
-        <v>212</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="F12" s="0" t="s">
         <v>314</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="G12" s="0" t="s">
         <v>315</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="H12" s="0" t="s">
         <v>316</v>
       </c>
-      <c r="H12" s="0" t="s">
+      <c r="I12" s="0" t="s">
         <v>317</v>
       </c>
-      <c r="I12" s="0" t="s">
+      <c r="J12" s="0" t="s">
         <v>318</v>
       </c>
-      <c r="J12" s="0" t="s">
+      <c r="K12" s="0" t="s">
         <v>319</v>
       </c>
-      <c r="K12" s="0" t="s">
+      <c r="L12" s="0" t="s">
         <v>320</v>
-      </c>
-      <c r="L12" s="0" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
+        <v>321</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>322</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="C13" s="0" t="s">
         <v>323</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>324</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>48</v>
       </c>
       <c r="E13" s="0" t="s">
+        <v>324</v>
+      </c>
+      <c r="F13" s="0" t="s">
         <v>325</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="G13" s="0" t="s">
         <v>326</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="H13" s="0" t="s">
         <v>327</v>
       </c>
-      <c r="H13" s="0" t="s">
+      <c r="L13" s="0" t="s">
         <v>328</v>
-      </c>
-      <c r="L13" s="0" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
+        <v>329</v>
+      </c>
+      <c r="B14" s="0" t="s">
         <v>330</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="C14" s="0" t="s">
         <v>331</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="D14" s="0" t="s">
         <v>332</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="E14" s="0" t="s">
         <v>333</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="F14" s="0" t="s">
         <v>334</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="G14" s="0" t="s">
         <v>335</v>
       </c>
-      <c r="G14" s="0" t="s">
+      <c r="H14" s="0" t="s">
         <v>336</v>
       </c>
-      <c r="H14" s="0" t="s">
+      <c r="J14" s="0" t="s">
         <v>337</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="L14" s="0" t="s">
         <v>338</v>
-      </c>
-      <c r="L14" s="0" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B15" s="0" t="s">
+        <v>339</v>
+      </c>
+      <c r="C15" s="0" t="s">
         <v>340</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="D15" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="0" t="s">
         <v>341</v>
       </c>
-      <c r="D15" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="E15" s="0" t="s">
+      <c r="F15" s="0" t="s">
         <v>342</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="G15" s="0" t="s">
         <v>343</v>
       </c>
-      <c r="G15" s="0" t="s">
+      <c r="H15" s="0" t="s">
         <v>344</v>
       </c>
-      <c r="H15" s="0" t="s">
+      <c r="I15" s="0" t="s">
         <v>345</v>
       </c>
-      <c r="I15" s="0" t="s">
+      <c r="J15" s="0" t="s">
         <v>346</v>
       </c>
-      <c r="J15" s="0" t="s">
+      <c r="L15" s="0" t="s">
         <v>347</v>
-      </c>
-      <c r="L15" s="0" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B16" s="0" t="s">
+        <v>348</v>
+      </c>
+      <c r="C16" s="0" t="s">
         <v>349</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="D16" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="E16" s="0" t="s">
         <v>350</v>
       </c>
-      <c r="D16" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="E16" s="0" t="s">
+      <c r="F16" s="0" t="s">
         <v>351</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="G16" s="0" t="s">
         <v>352</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="H16" s="0" t="s">
         <v>353</v>
       </c>
-      <c r="H16" s="0" t="s">
+      <c r="J16" s="0" t="s">
         <v>354</v>
       </c>
-      <c r="I16" s="0" t="s">
+      <c r="K16" s="0" t="s">
         <v>355</v>
       </c>
-      <c r="K16" s="0" t="s">
+      <c r="L16" s="0" t="s">
         <v>356</v>
-      </c>
-      <c r="L16" s="0" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
+        <v>357</v>
+      </c>
+      <c r="B17" s="0" t="s">
         <v>358</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="C17" s="0" t="s">
         <v>359</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="D17" s="0" t="s">
         <v>360</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="E17" s="0" t="s">
         <v>361</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="F17" s="0" t="s">
         <v>362</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="G17" s="0" t="s">
         <v>363</v>
       </c>
-      <c r="G17" s="0" t="s">
+      <c r="L17" s="0" t="s">
         <v>364</v>
-      </c>
-      <c r="L17" s="0" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
+        <v>365</v>
+      </c>
+      <c r="B18" s="0" t="s">
         <v>366</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="C18" s="0" t="s">
         <v>367</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="D18" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="E18" s="0" t="s">
         <v>368</v>
       </c>
-      <c r="D18" s="0" t="s">
-        <v>206</v>
-      </c>
-      <c r="E18" s="0" t="s">
+      <c r="F18" s="0" t="s">
         <v>369</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="G18" s="0" t="s">
         <v>370</v>
       </c>
-      <c r="G18" s="0" t="s">
+      <c r="H18" s="0" t="s">
         <v>371</v>
       </c>
-      <c r="H18" s="0" t="s">
+      <c r="L18" s="0" t="s">
         <v>372</v>
-      </c>
-      <c r="L18" s="0" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
+        <v>373</v>
+      </c>
+      <c r="B19" s="0" t="s">
         <v>374</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="C19" s="0" t="s">
         <v>375</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="D19" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="E19" s="0" t="s">
         <v>376</v>
       </c>
-      <c r="D19" s="0" t="s">
-        <v>131</v>
-      </c>
-      <c r="E19" s="0" t="s">
+      <c r="F19" s="0" t="s">
         <v>377</v>
       </c>
-      <c r="F19" s="0" t="s">
+      <c r="H19" s="0" t="s">
+        <v>286</v>
+      </c>
+      <c r="L19" s="0" t="s">
         <v>378</v>
-      </c>
-      <c r="H19" s="0" t="s">
-        <v>287</v>
-      </c>
-      <c r="L19" s="0" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
+        <v>379</v>
+      </c>
+      <c r="B20" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="C20" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="D20" s="0" t="s">
         <v>382</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="E20" s="0" t="s">
         <v>383</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="F20" s="0" t="s">
         <v>384</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="L20" s="0" t="s">
         <v>385</v>
-      </c>
-      <c r="L20" s="0" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B21" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="C21" s="0" t="s">
         <v>387</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="D21" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="E21" s="0" t="s">
         <v>388</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="E21" s="0" t="s">
+      <c r="F21" s="0" t="s">
         <v>389</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="G21" s="0" t="s">
         <v>390</v>
       </c>
-      <c r="G21" s="0" t="s">
+      <c r="H21" s="0" t="s">
         <v>391</v>
       </c>
-      <c r="H21" s="0" t="s">
+      <c r="L21" s="0" t="s">
         <v>392</v>
-      </c>
-      <c r="L21" s="0" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B22" s="0" t="s">
+        <v>393</v>
+      </c>
+      <c r="C22" s="0" t="s">
         <v>394</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="D22" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="E22" s="0" t="s">
         <v>395</v>
       </c>
-      <c r="D22" s="0" t="s">
-        <v>153</v>
-      </c>
-      <c r="E22" s="0" t="s">
+      <c r="F22" s="0" t="s">
         <v>396</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="G22" s="0" t="s">
         <v>397</v>
       </c>
-      <c r="G22" s="0" t="s">
+      <c r="H22" s="0" t="s">
         <v>398</v>
       </c>
-      <c r="H22" s="0" t="s">
+      <c r="I22" s="0" t="s">
         <v>399</v>
       </c>
-      <c r="J22" s="0" t="s">
+      <c r="L22" s="0" t="s">
         <v>400</v>
-      </c>
-      <c r="L22" s="0" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>401</v>
+      </c>
+      <c r="C23" s="0" t="s">
         <v>402</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="D23" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="E23" s="0" t="s">
         <v>403</v>
       </c>
-      <c r="D23" s="0" t="s">
-        <v>218</v>
-      </c>
-      <c r="E23" s="0" t="s">
+      <c r="F23" s="0" t="s">
         <v>404</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="G23" s="0" t="s">
         <v>405</v>
       </c>
-      <c r="G23" s="0" t="s">
+      <c r="H23" s="0" t="s">
         <v>406</v>
       </c>
-      <c r="H23" s="0" t="s">
+      <c r="J23" s="0" t="s">
         <v>407</v>
       </c>
-      <c r="I23" s="0" t="s">
+      <c r="L23" s="0" t="s">
         <v>408</v>
-      </c>
-      <c r="L23" s="0" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B24" s="0" t="s">
+        <v>409</v>
+      </c>
+      <c r="C24" s="0" t="s">
         <v>410</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="D24" s="0" t="s">
+        <v>200</v>
+      </c>
+      <c r="E24" s="0" t="s">
         <v>411</v>
       </c>
-      <c r="D24" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="E24" s="0" t="s">
+      <c r="F24" s="0" t="s">
         <v>412</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="G24" s="0" t="s">
         <v>413</v>
       </c>
-      <c r="G24" s="0" t="s">
+      <c r="H24" s="0" t="s">
         <v>414</v>
       </c>
-      <c r="H24" s="0" t="s">
+      <c r="I24" s="0" t="s">
         <v>415</v>
       </c>
-      <c r="I24" s="0" t="s">
+      <c r="J24" s="0" t="s">
         <v>416</v>
       </c>
-      <c r="J24" s="0" t="s">
+      <c r="L24" s="0" t="s">
         <v>417</v>
-      </c>
-      <c r="L24" s="0" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B25" s="0" t="s">
+        <v>418</v>
+      </c>
+      <c r="C25" s="0" t="s">
         <v>419</v>
-      </c>
-      <c r="C25" s="0" t="s">
-        <v>420</v>
       </c>
       <c r="D25" s="0" t="s">
         <v>56</v>
       </c>
       <c r="E25" s="0" t="s">
+        <v>420</v>
+      </c>
+      <c r="F25" s="0" t="s">
         <v>421</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="G25" s="0" t="s">
         <v>422</v>
       </c>
-      <c r="G25" s="0" t="s">
+      <c r="H25" s="0" t="s">
         <v>423</v>
       </c>
-      <c r="H25" s="0" t="s">
+      <c r="I25" s="0" t="s">
         <v>424</v>
       </c>
-      <c r="J25" s="0" t="s">
+      <c r="L25" s="0" t="s">
         <v>425</v>
-      </c>
-      <c r="L25" s="0" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>426</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>427</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="D26" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="E26" s="0" t="s">
         <v>428</v>
       </c>
-      <c r="D26" s="0" t="s">
-        <v>69</v>
-      </c>
-      <c r="E26" s="0" t="s">
+      <c r="F26" s="0" t="s">
         <v>429</v>
       </c>
-      <c r="F26" s="0" t="s">
+      <c r="G26" s="0" t="s">
         <v>430</v>
       </c>
-      <c r="G26" s="0" t="s">
+      <c r="J26" s="0" t="s">
         <v>431</v>
       </c>
-      <c r="I26" s="0" t="s">
+      <c r="L26" s="0" t="s">
         <v>432</v>
-      </c>
-      <c r="L26" s="0" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
+        <v>433</v>
+      </c>
+      <c r="B27" s="0" t="s">
         <v>434</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="C27" s="0" t="s">
         <v>435</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="D27" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E27" s="0" t="s">
         <v>436</v>
       </c>
-      <c r="D27" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="E27" s="0" t="s">
+      <c r="F27" s="0" t="s">
         <v>437</v>
       </c>
-      <c r="F27" s="0" t="s">
+      <c r="G27" s="0" t="s">
         <v>438</v>
       </c>
-      <c r="G27" s="0" t="s">
+      <c r="H27" s="0" t="s">
         <v>439</v>
       </c>
-      <c r="H27" s="0" t="s">
+      <c r="I27" s="0" t="s">
         <v>440</v>
       </c>
-      <c r="I27" s="0" t="s">
+      <c r="J27" s="0" t="s">
         <v>441</v>
       </c>
-      <c r="J27" s="0" t="s">
+      <c r="K27" s="0" t="s">
         <v>442</v>
       </c>
-      <c r="K27" s="0" t="s">
+      <c r="L27" s="0" t="s">
         <v>443</v>
-      </c>
-      <c r="L27" s="0" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
+        <v>444</v>
+      </c>
+      <c r="B28" s="0" t="s">
         <v>445</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="C28" s="0" t="s">
         <v>446</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="D28" s="0" t="s">
         <v>447</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="E28" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="E28" s="0" t="s">
+      <c r="F28" s="0" t="s">
         <v>449</v>
       </c>
-      <c r="F28" s="0" t="s">
+      <c r="G28" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="G28" s="0" t="s">
+      <c r="I28" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="J28" s="0" t="s">
+      <c r="K28" s="0" t="s">
         <v>452</v>
       </c>
-      <c r="K28" s="0" t="s">
+      <c r="L28" s="0" t="s">
         <v>453</v>
-      </c>
-      <c r="L28" s="0" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B29" s="0" t="s">
+        <v>454</v>
+      </c>
+      <c r="C29" s="0" t="s">
         <v>455</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="D29" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="E29" s="0" t="s">
         <v>456</v>
       </c>
-      <c r="D29" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="E29" s="0" t="s">
+      <c r="F29" s="0" t="s">
         <v>457</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="G29" s="0" t="s">
         <v>458</v>
       </c>
-      <c r="G29" s="0" t="s">
+      <c r="I29" s="0" t="s">
         <v>459</v>
       </c>
-      <c r="J29" s="0" t="s">
+      <c r="L29" s="0" t="s">
         <v>460</v>
-      </c>
-      <c r="L29" s="0" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B30" s="0" t="s">
+        <v>461</v>
+      </c>
+      <c r="C30" s="0" t="s">
         <v>462</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="D30" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="E30" s="0" t="s">
         <v>463</v>
       </c>
-      <c r="D30" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="E30" s="0" t="s">
+      <c r="F30" s="0" t="s">
         <v>464</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="G30" s="0" t="s">
         <v>465</v>
       </c>
-      <c r="G30" s="0" t="s">
+      <c r="H30" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="H30" s="0" t="s">
+      <c r="I30" s="0" t="s">
         <v>467</v>
       </c>
-      <c r="J30" s="0" t="s">
+      <c r="L30" s="0" t="s">
         <v>468</v>
-      </c>
-      <c r="L30" s="0" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B31" s="0" t="s">
+        <v>469</v>
+      </c>
+      <c r="C31" s="0" t="s">
         <v>470</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="D31" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="E31" s="0" t="s">
         <v>471</v>
       </c>
-      <c r="D31" s="0" t="s">
-        <v>185</v>
-      </c>
-      <c r="E31" s="0" t="s">
+      <c r="F31" s="0" t="s">
         <v>472</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="G31" s="0" t="s">
         <v>473</v>
       </c>
-      <c r="G31" s="0" t="s">
+      <c r="H31" s="0" t="s">
         <v>474</v>
       </c>
-      <c r="H31" s="0" t="s">
+      <c r="J31" s="0" t="s">
+        <v>474</v>
+      </c>
+      <c r="L31" s="0" t="s">
         <v>475</v>
-      </c>
-      <c r="I31" s="0" t="s">
-        <v>475</v>
-      </c>
-      <c r="L31" s="0" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B32" s="0" t="s">
+        <v>476</v>
+      </c>
+      <c r="C32" s="0" t="s">
         <v>477</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="D32" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="E32" s="0" t="s">
         <v>478</v>
       </c>
-      <c r="D32" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="E32" s="0" t="s">
+      <c r="F32" s="0" t="s">
         <v>479</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="G32" s="0" t="s">
         <v>480</v>
       </c>
-      <c r="G32" s="0" t="s">
+      <c r="H32" s="0" t="s">
         <v>481</v>
       </c>
-      <c r="H32" s="0" t="s">
+      <c r="I32" s="0" t="s">
         <v>482</v>
       </c>
-      <c r="I32" s="0" t="s">
+      <c r="J32" s="0" t="s">
         <v>483</v>
       </c>
-      <c r="J32" s="0" t="s">
+      <c r="L32" s="0" t="s">
         <v>484</v>
-      </c>
-      <c r="L32" s="0" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B33" s="0" t="s">
+        <v>485</v>
+      </c>
+      <c r="C33" s="0" t="s">
         <v>486</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="D33" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="E33" s="0" t="s">
         <v>487</v>
       </c>
-      <c r="D33" s="0" t="s">
-        <v>190</v>
-      </c>
-      <c r="E33" s="0" t="s">
+      <c r="F33" s="0" t="s">
         <v>488</v>
       </c>
-      <c r="F33" s="0" t="s">
+      <c r="G33" s="0" t="s">
         <v>489</v>
       </c>
-      <c r="G33" s="0" t="s">
+      <c r="H33" s="0" t="s">
         <v>490</v>
       </c>
-      <c r="H33" s="0" t="s">
+      <c r="J33" s="0" t="s">
         <v>491</v>
       </c>
-      <c r="I33" s="0" t="s">
+      <c r="L33" s="0" t="s">
         <v>492</v>
-      </c>
-      <c r="L33" s="0" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B34" s="0" t="s">
+        <v>493</v>
+      </c>
+      <c r="C34" s="0" t="s">
         <v>494</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="D34" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="E34" s="0" t="s">
         <v>495</v>
       </c>
-      <c r="D34" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="E34" s="0" t="s">
+      <c r="F34" s="0" t="s">
         <v>496</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="G34" s="0" t="s">
         <v>497</v>
       </c>
-      <c r="G34" s="0" t="s">
+      <c r="H34" s="0" t="s">
         <v>498</v>
       </c>
-      <c r="H34" s="0" t="s">
+      <c r="I34" s="0" t="s">
         <v>499</v>
       </c>
-      <c r="I34" s="0" t="s">
+      <c r="J34" s="0" t="s">
         <v>500</v>
       </c>
-      <c r="J34" s="0" t="s">
+      <c r="K34" s="0" t="s">
         <v>501</v>
       </c>
-      <c r="K34" s="0" t="s">
+      <c r="L34" s="0" t="s">
         <v>502</v>
-      </c>
-      <c r="L34" s="0" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B35" s="0" t="s">
+        <v>503</v>
+      </c>
+      <c r="C35" s="0" t="s">
         <v>504</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="D35" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="0" t="s">
         <v>505</v>
       </c>
-      <c r="D35" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="E35" s="0" t="s">
+      <c r="F35" s="0" t="s">
         <v>506</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="G35" s="0" t="s">
         <v>507</v>
       </c>
-      <c r="G35" s="0" t="s">
+      <c r="H35" s="0" t="s">
         <v>508</v>
       </c>
-      <c r="H35" s="0" t="s">
+      <c r="I35" s="0" t="s">
         <v>509</v>
       </c>
-      <c r="I35" s="0" t="s">
+      <c r="J35" s="0" t="s">
         <v>510</v>
       </c>
-      <c r="J35" s="0" t="s">
+      <c r="K35" s="0" t="s">
         <v>511</v>
       </c>
-      <c r="K35" s="0" t="s">
+      <c r="L35" s="0" t="s">
         <v>512</v>
-      </c>
-      <c r="L35" s="0" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
+        <v>513</v>
+      </c>
+      <c r="B36" s="0" t="s">
         <v>514</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="C36" s="0" t="s">
         <v>515</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="D36" s="0" t="s">
         <v>516</v>
       </c>
-      <c r="D36" s="0" t="s">
+      <c r="E36" s="0" t="s">
         <v>517</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="F36" s="0" t="s">
         <v>518</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="G36" s="0" t="s">
         <v>519</v>
       </c>
-      <c r="G36" s="0" t="s">
+      <c r="L36" s="0" t="s">
         <v>520</v>
-      </c>
-      <c r="L36" s="0" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C37" s="0" t="s">
+        <v>521</v>
+      </c>
+      <c r="D37" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="E37" s="0" t="s">
         <v>522</v>
       </c>
-      <c r="D37" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="E37" s="0" t="s">
+      <c r="F37" s="0" t="s">
         <v>523</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="G37" s="0" t="s">
         <v>524</v>
       </c>
-      <c r="G37" s="0" t="s">
+      <c r="H37" s="0" t="s">
         <v>525</v>
       </c>
-      <c r="H37" s="0" t="s">
+      <c r="J37" s="0" t="s">
         <v>526</v>
       </c>
-      <c r="I37" s="0" t="s">
+      <c r="L37" s="0" t="s">
         <v>527</v>
-      </c>
-      <c r="L37" s="0" t="s">
-        <v>528</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
+        <v>528</v>
+      </c>
+      <c r="B38" s="0" t="s">
         <v>529</v>
       </c>
-      <c r="B38" s="0" t="s">
+      <c r="C38" s="0" t="s">
         <v>530</v>
       </c>
-      <c r="C38" s="0" t="s">
+      <c r="D38" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="E38" s="0" t="s">
         <v>531</v>
       </c>
-      <c r="D38" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="E38" s="0" t="s">
+      <c r="F38" s="0" t="s">
         <v>532</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="G38" s="0" t="s">
         <v>533</v>
       </c>
-      <c r="G38" s="0" t="s">
+      <c r="J38" s="0" t="s">
         <v>534</v>
       </c>
-      <c r="I38" s="0" t="s">
+      <c r="L38" s="0" t="s">
         <v>535</v>
-      </c>
-      <c r="L38" s="0" t="s">
-        <v>536</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B39" s="0" t="s">
+        <v>536</v>
+      </c>
+      <c r="C39" s="0" t="s">
         <v>537</v>
       </c>
-      <c r="C39" s="0" t="s">
+      <c r="D39" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="E39" s="0" t="s">
         <v>538</v>
       </c>
-      <c r="D39" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="E39" s="0" t="s">
+      <c r="F39" s="0" t="s">
         <v>539</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="G39" s="0" t="s">
         <v>540</v>
       </c>
-      <c r="G39" s="0" t="s">
+      <c r="H39" s="0" t="s">
         <v>541</v>
-      </c>
-      <c r="H39" s="0" t="s">
-        <v>542</v>
       </c>
       <c r="I39" s="0" t="s">
         <v>542</v>
       </c>
       <c r="J39" s="0" t="s">
+        <v>541</v>
+      </c>
+      <c r="K39" s="0" t="s">
         <v>543</v>
       </c>
-      <c r="K39" s="0" t="s">
+      <c r="L39" s="0" t="s">
         <v>544</v>
-      </c>
-      <c r="L39" s="0" t="s">
-        <v>545</v>
       </c>
     </row>
     <row r="40">
@@ -5255,31 +5252,31 @@
         <v>44</v>
       </c>
       <c r="B40" s="0" t="s">
+        <v>545</v>
+      </c>
+      <c r="C40" s="0" t="s">
         <v>546</v>
-      </c>
-      <c r="C40" s="0" t="s">
-        <v>547</v>
       </c>
       <c r="D40" s="0" t="s">
         <v>38</v>
       </c>
       <c r="E40" s="0" t="s">
+        <v>547</v>
+      </c>
+      <c r="F40" s="0" t="s">
         <v>548</v>
       </c>
-      <c r="F40" s="0" t="s">
+      <c r="G40" s="0" t="s">
         <v>549</v>
       </c>
-      <c r="G40" s="0" t="s">
+      <c r="H40" s="0" t="s">
         <v>550</v>
       </c>
-      <c r="H40" s="0" t="s">
+      <c r="J40" s="0" t="s">
         <v>551</v>
       </c>
-      <c r="I40" s="0" t="s">
+      <c r="L40" s="0" t="s">
         <v>552</v>
-      </c>
-      <c r="L40" s="0" t="s">
-        <v>553</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update session and speaker details, add new speakers and modify existing session information
</commit_message>
<xml_diff>
--- a/src/assets/sessionize/data-advanced.xlsx
+++ b/src/assets/sessionize/data-advanced.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="553">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="559">
   <si>
     <t>Session Id</t>
   </si>
@@ -328,32 +328,25 @@
     <t>d3f982bf-06f2-4a7a-ac5a-2479f4cec0b2</t>
   </si>
   <si>
-    <t>Warp Pipes and Prefetching: Navigating the Web at Mario Speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long wait times are the "Bowser" of the good user experience. Even if your site looks great, slow transitions or blank loading screens can make users feel like they’ve fallen down a bottomless pit. But what if your website could predict the future, stay resilient offline, and move between pages as smoothly as a Warp Pipe?_x000D_
-_x000D_
-In this session, we’ll explore the "Power-Up" trio of modern web development:_x000D_
-- Speculation Rules API: See how prefetching and prerendering can load pages before users click._x000D_
-- Service Workers: Find out how to build a caching layer so your assets are always ready, even when the network is out of "lives"._x000D_
-- View Transition API: Use animations to help users move smoothly through your "world map" with ease._x000D_
-_x000D_
-We’ll break down the technical plumbing required to make these APIs work nicely together. You will leave this session with the cheat codes needed to deliver a fast, seamless experience that will have your users saying, "Mamma Mia, that’s fast!"</t>
-  </si>
-  <si>
-    <t>Rowdy Rabouw</t>
-  </si>
-  <si>
-    <t>hi@rowdy.codes</t>
+    <t>What’s New in Web? 2026 Edition</t>
+  </si>
+  <si>
+    <t>Christian is a member of the World Wide Web’s architecture board, the Technical Architecture Group (TAG) of W3C. As such, he has insights into what’s going on in the web platform. In his session, you'll gain insights into the latest discussions among standards bodies, browser vendors, and web developers. And you have the opportunity to report your wishes back to the Web’s architecture board. Don't miss this opportunity to stay updated on the forefront of web technologies.</t>
+  </si>
+  <si>
+    <t>Christian Liebel</t>
+  </si>
+  <si>
+    <t>christian@liebel.org</t>
   </si>
   <si>
     <t>Web</t>
   </si>
   <si>
-    <t>The Netherlands</t>
-  </si>
-  <si>
-    <t>f5c30de4-cd93-4022-97f6-b0a58c92197c</t>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>d7da8026-334b-42d8-aec9-324bf1bb6ec4</t>
   </si>
   <si>
     <t>From shy contributor to (kinda) confident community leader</t>
@@ -504,22 +497,30 @@
     <t>7b344585-bf7f-4436-8d09-99c57f125009, 26ccbcbd-1d78-471c-b98e-fa7854526c2a</t>
   </si>
   <si>
-    <t>What’s New in Web? 2026 Edition</t>
-  </si>
-  <si>
-    <t>Christian is a member of the World Wide Web’s architecture board, the Technical Architecture Group (TAG) of W3C. As such, he has insights into what’s going on in the web platform. In his session, you'll gain insights into the latest discussions among standards bodies, browser vendors, and web developers. And you have the opportunity to report your wishes back to the Web’s architecture board. Don't miss this opportunity to stay updated on the forefront of web technologies.</t>
-  </si>
-  <si>
-    <t>Christian Liebel</t>
-  </si>
-  <si>
-    <t>christian@liebel.org</t>
-  </si>
-  <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t>d7da8026-334b-42d8-aec9-324bf1bb6ec4</t>
+    <t xml:space="preserve">Superset, dashboard, embedding  e dolori</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superset, per chi non lo conoscesse, è un potente tool open-source per la creazione di dashboard e visualizzazioni a partire dai dati presenti nei nostri database. In teoria, uno strumento che permette di risparmiare molto tempo nello sviluppo di visualizzatori — più o meno belli — da offrire ai nostri utenti._x000D_
+_x000D_
+Io e il mio collega Fabrizio Baldazzi ci siamo però trovati ad affrontare una sfida che, sulla carta, sembrava una banalità: effettuare l’embedding delle dashboard di Superset all’interno di un applicativo aziendale. Nella pratica, complice una documentazione ufficiale poco chiara e una scarsità di esempi ed esperienze condivise dalla community, il percorso si è rivelato tutt’altro che semplice._x000D_
+_x000D_
+In questo talk racconteremo un use case reale, analizzando i problemi incontrati, le soluzioni adottate e le scelte architetturali che ci hanno permesso di arrivare a un risultato solido e manutenibile._x000D_
+L’obiettivo è fornire indicazioni concrete e subito applicabili a chi si trova — o si troverà — nella stessa situazione, evitando di perdere settimane di lavoro su aspetti apparentemente secondari.</t>
+  </si>
+  <si>
+    <t>Giorgio Basile</t>
+  </si>
+  <si>
+    <t>giorgiobasile631@gmail.com</t>
+  </si>
+  <si>
+    <t>Giorgio Basile, Fabrizio Baldazzi</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>d1f80578-6fe5-45f4-ba37-5020a69f550f, b3fd818c-10c9-4e96-a32b-d95deba9fc21</t>
   </si>
   <si>
     <t>Senior Engineer ≠ More Code: A Git History Tell-All</t>
@@ -657,9 +658,6 @@
     <t>juna.salviati@gmail.com</t>
   </si>
   <si>
-    <t>Other</t>
-  </si>
-  <si>
     <t>baa96c7b-6106-4cb5-8d88-124af5027adc</t>
   </si>
   <si>
@@ -1499,6 +1497,27 @@
     <t>https://sessionize.com/image/56d9-400o400o1-P2kemErpqogrPsG2zXiUxQ.jpg</t>
   </si>
   <si>
+    <t>b3fd818c-10c9-4e96-a32b-d95deba9fc21</t>
+  </si>
+  <si>
+    <t>Fabrizio</t>
+  </si>
+  <si>
+    <t>Baldazzi</t>
+  </si>
+  <si>
+    <t>f.baldazzi@tiscali.it</t>
+  </si>
+  <si>
+    <t>Solution Archityect</t>
+  </si>
+  <si>
+    <t>I have a degree in computer science and have been working in this field since the 1990s. I deal with architectural solutions and development in various languages, such as Java, Angular, Python, and so on.</t>
+  </si>
+  <si>
+    <t>https://sessionize.com/image/7123-400o400o1-wFgsBEnphmM2rKKLn7Xf3Q.jpg</t>
+  </si>
+  <si>
     <t>b8b99b42-456a-4934-a1ac-414d4ba2990b</t>
   </si>
   <si>
@@ -1665,6 +1684,31 @@
   </si>
   <si>
     <t>https://sessionize.com/image/3e16-400o400o1-7jvdkF5R8VCzcbkb33Ty6R.jpg</t>
+  </si>
+  <si>
+    <t>d1f80578-6fe5-45f4-ba37-5020a69f550f</t>
+  </si>
+  <si>
+    <t>Giorgio</t>
+  </si>
+  <si>
+    <t>Basile</t>
+  </si>
+  <si>
+    <t>Angular Frontend Developer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I am a young man born in 2000 and I am currently finishing my studies in computer science at the Ca' Foscari University of Venice, located in Mestre, in addition to being a full-time web developer._x000D_
+In addition to studying, I love playing role-playing games, skateboarding and playing Magic the Gathering.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/giorgiobasile00/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/bacarotechofficial/</t>
+  </si>
+  <si>
+    <t>https://sessionize.com/image/291e-400o400o1-fZ88yJQ1jSUdb8xqVryTQ5.jpg</t>
   </si>
   <si>
     <t>Federico</t>
@@ -1824,33 +1868,6 @@
   </si>
   <si>
     <t>https://sessionize.com/image/bbe0-400o400o1-GC45U3jx4Sw9b64DsYA27P.jpg</t>
-  </si>
-  <si>
-    <t>Rowdy</t>
-  </si>
-  <si>
-    <t>Rabouw</t>
-  </si>
-  <si>
-    <t>Front-End Focused Senior DevOps Engineer</t>
-  </si>
-  <si>
-    <t>Rowdy Rabouw is a Google Developer Expert in Web Technologies with over 25 years of experience in HTML, CSS and JavaScript. Currently, he works as a Front-End-Focused Senior DevOps Engineer on Vue, Node, and NestJS projects, with a focus on usability and accessibility. Rowdy loves his electronic drum kit and dabbles in creating music on his laptop.</t>
-  </si>
-  <si>
-    <t>http://nl.linkedin.com/in/rowdyrabouw</t>
-  </si>
-  <si>
-    <t>https://rowdy.codes</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/rowdyrabouw/</t>
-  </si>
-  <si>
-    <t>https://www.facebook.com/rowdy.rabouw</t>
-  </si>
-  <si>
-    <t>https://sessionize.com/image/f20e-400o400o1-LqCirkShubcxGkm5Ac1CrN.jpg</t>
   </si>
   <si>
     <t>Daniela</t>
@@ -2583,7 +2600,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0">
-        <v>1141786</v>
+        <v>1147593</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>89</v>
@@ -2610,7 +2627,7 @@
         <v>28</v>
       </c>
       <c r="J11" s="0" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="K11" s="0" t="s">
         <v>40</v>
@@ -2625,7 +2642,7 @@
         <v>46087.774690972219</v>
       </c>
       <c r="O11" s="5">
-        <v>46087.86314163194</v>
+        <v>46087.783132638884</v>
       </c>
       <c r="P11" s="0" t="s">
         <v>43</v>
@@ -3017,7 +3034,7 @@
     </row>
     <row r="18">
       <c r="A18" s="0">
-        <v>1147593</v>
+        <v>1123087</v>
       </c>
       <c r="B18" s="0" t="s">
         <v>132</v>
@@ -3032,10 +3049,10 @@
         <v>135</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>93</v>
+        <v>137</v>
       </c>
       <c r="H18" s="0" t="s">
         <v>27</v>
@@ -3047,19 +3064,19 @@
         <v>50</v>
       </c>
       <c r="K18" s="0" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L18" s="0" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="M18" s="0" t="s">
-        <v>136</v>
+        <v>75</v>
       </c>
       <c r="N18" s="5">
-        <v>46087.774690972219</v>
+        <v>46110.370604861106</v>
       </c>
       <c r="O18" s="5">
-        <v>46087.783132638884</v>
+        <v>46110.417713541661</v>
       </c>
       <c r="P18" s="0" t="s">
         <v>43</v>
@@ -3074,7 +3091,7 @@
         <v>0</v>
       </c>
       <c r="V18" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19">
@@ -3082,19 +3099,19 @@
         <v>1149006</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E19" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" s="0" t="s">
         <v>141</v>
-      </c>
-      <c r="F19" s="0" t="s">
-        <v>140</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>74</v>
@@ -3136,7 +3153,7 @@
         <v>0</v>
       </c>
       <c r="V19" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20">
@@ -3144,19 +3161,19 @@
         <v>1154402</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E20" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="F20" s="0" t="s">
         <v>146</v>
-      </c>
-      <c r="F20" s="0" t="s">
-        <v>145</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>39</v>
@@ -3198,7 +3215,7 @@
         <v>0</v>
       </c>
       <c r="V20" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21">
@@ -3206,19 +3223,19 @@
         <v>1149301</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E21" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="F21" s="0" t="s">
         <v>151</v>
-      </c>
-      <c r="F21" s="0" t="s">
-        <v>150</v>
       </c>
       <c r="G21" s="0" t="s">
         <v>74</v>
@@ -3233,7 +3250,7 @@
         <v>50</v>
       </c>
       <c r="K21" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="L21" s="0" t="s">
         <v>31</v>
@@ -3260,7 +3277,7 @@
         <v>0</v>
       </c>
       <c r="V21" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22">
@@ -3268,19 +3285,19 @@
         <v>1149383</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E22" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="F22" s="0" t="s">
         <v>157</v>
-      </c>
-      <c r="F22" s="0" t="s">
-        <v>156</v>
       </c>
       <c r="G22" s="0" t="s">
         <v>39</v>
@@ -3322,7 +3339,7 @@
         <v>0</v>
       </c>
       <c r="V22" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23">
@@ -3330,19 +3347,19 @@
         <v>1151362</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E23" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="F23" s="0" t="s">
         <v>162</v>
-      </c>
-      <c r="F23" s="0" t="s">
-        <v>161</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>39</v>
@@ -3384,7 +3401,7 @@
         <v>0</v>
       </c>
       <c r="V23" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24">
@@ -3392,22 +3409,22 @@
         <v>1155630</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E24" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="F24" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="F24" s="0" t="s">
-        <v>166</v>
-      </c>
       <c r="G24" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H24" s="0" t="s">
         <v>27</v>
@@ -3425,7 +3442,7 @@
         <v>31</v>
       </c>
       <c r="M24" s="0" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="N24" s="5">
         <v>46080.807078935184</v>
@@ -3446,7 +3463,7 @@
         <v>0</v>
       </c>
       <c r="V24" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25">
@@ -3454,22 +3471,22 @@
         <v>1105608</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E25" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="F25" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="F25" s="0" t="s">
-        <v>172</v>
-      </c>
       <c r="G25" s="0" t="s">
-        <v>174</v>
+        <v>137</v>
       </c>
       <c r="H25" s="0" t="s">
         <v>58</v>
@@ -3593,7 +3610,7 @@
         <v>183</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H27" s="0" t="s">
         <v>27</v>
@@ -3841,7 +3858,7 @@
         <v>206</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H31" s="0" t="s">
         <v>58</v>
@@ -3965,7 +3982,7 @@
         <v>216</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H33" s="0" t="s">
         <v>58</v>
@@ -4014,7 +4031,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4086,7 +4103,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>238</v>
@@ -4095,7 +4112,7 @@
         <v>239</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E3" s="0" t="s">
         <v>240</v>
@@ -4211,7 +4228,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>273</v>
@@ -4220,7 +4237,7 @@
         <v>274</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>275</v>
@@ -4266,7 +4283,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>288</v>
@@ -4275,7 +4292,7 @@
         <v>289</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E9" s="0" t="s">
         <v>290</v>
@@ -4327,7 +4344,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>303</v>
@@ -4336,7 +4353,7 @@
         <v>304</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E11" s="0" t="s">
         <v>305</v>
@@ -4490,7 +4507,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>348</v>
@@ -4499,7 +4516,7 @@
         <v>349</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E16" s="0" t="s">
         <v>350</v>
@@ -4658,7 +4675,7 @@
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B22" s="0" t="s">
         <v>393</v>
@@ -4667,7 +4684,7 @@
         <v>394</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E22" s="0" t="s">
         <v>395</v>
@@ -4827,88 +4844,82 @@
         <v>435</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>122</v>
+        <v>436</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>437</v>
-      </c>
-      <c r="G27" s="0" t="s">
         <v>438</v>
       </c>
-      <c r="H27" s="0" t="s">
+      <c r="L27" s="0" t="s">
         <v>439</v>
-      </c>
-      <c r="I27" s="0" t="s">
-        <v>440</v>
-      </c>
-      <c r="J27" s="0" t="s">
-        <v>441</v>
-      </c>
-      <c r="K27" s="0" t="s">
-        <v>442</v>
-      </c>
-      <c r="L27" s="0" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
+        <v>440</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>441</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>442</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>443</v>
+      </c>
+      <c r="F28" s="0" t="s">
         <v>444</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="G28" s="0" t="s">
         <v>445</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="H28" s="0" t="s">
         <v>446</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="I28" s="0" t="s">
         <v>447</v>
       </c>
-      <c r="E28" s="0" t="s">
+      <c r="J28" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="F28" s="0" t="s">
+      <c r="K28" s="0" t="s">
         <v>449</v>
       </c>
-      <c r="G28" s="0" t="s">
+      <c r="L28" s="0" t="s">
         <v>450</v>
-      </c>
-      <c r="I28" s="0" t="s">
-        <v>451</v>
-      </c>
-      <c r="K28" s="0" t="s">
-        <v>452</v>
-      </c>
-      <c r="L28" s="0" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>175</v>
+        <v>451</v>
       </c>
       <c r="B29" s="0" t="s">
+        <v>452</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>453</v>
+      </c>
+      <c r="D29" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="E29" s="0" t="s">
         <v>455</v>
       </c>
-      <c r="D29" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="E29" s="0" t="s">
+      <c r="F29" s="0" t="s">
         <v>456</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="G29" s="0" t="s">
         <v>457</v>
       </c>
-      <c r="G29" s="0" t="s">
+      <c r="I29" s="0" t="s">
         <v>458</v>
       </c>
-      <c r="I29" s="0" t="s">
+      <c r="K29" s="0" t="s">
         <v>459</v>
       </c>
       <c r="L29" s="0" t="s">
@@ -4917,7 +4928,7 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="B30" s="0" t="s">
         <v>461</v>
@@ -4926,7 +4937,7 @@
         <v>462</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>99</v>
+        <v>174</v>
       </c>
       <c r="E30" s="0" t="s">
         <v>463</v>
@@ -4937,42 +4948,39 @@
       <c r="G30" s="0" t="s">
         <v>465</v>
       </c>
-      <c r="H30" s="0" t="s">
+      <c r="I30" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="I30" s="0" t="s">
+      <c r="L30" s="0" t="s">
         <v>467</v>
-      </c>
-      <c r="L30" s="0" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>185</v>
+        <v>100</v>
       </c>
       <c r="B31" s="0" t="s">
+        <v>468</v>
+      </c>
+      <c r="C31" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="D31" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="E31" s="0" t="s">
         <v>470</v>
       </c>
-      <c r="D31" s="0" t="s">
-        <v>184</v>
-      </c>
-      <c r="E31" s="0" t="s">
+      <c r="F31" s="0" t="s">
         <v>471</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="G31" s="0" t="s">
         <v>472</v>
       </c>
-      <c r="G31" s="0" t="s">
+      <c r="H31" s="0" t="s">
         <v>473</v>
       </c>
-      <c r="H31" s="0" t="s">
-        <v>474</v>
-      </c>
-      <c r="J31" s="0" t="s">
+      <c r="I31" s="0" t="s">
         <v>474</v>
       </c>
       <c r="L31" s="0" t="s">
@@ -4981,7 +4989,7 @@
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>76</v>
+        <v>185</v>
       </c>
       <c r="B32" s="0" t="s">
         <v>476</v>
@@ -4990,7 +4998,7 @@
         <v>477</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>73</v>
+        <v>184</v>
       </c>
       <c r="E32" s="0" t="s">
         <v>478</v>
@@ -5004,51 +5012,51 @@
       <c r="H32" s="0" t="s">
         <v>481</v>
       </c>
-      <c r="I32" s="0" t="s">
+      <c r="J32" s="0" t="s">
+        <v>481</v>
+      </c>
+      <c r="L32" s="0" t="s">
         <v>482</v>
-      </c>
-      <c r="J32" s="0" t="s">
-        <v>483</v>
-      </c>
-      <c r="L32" s="0" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
-        <v>191</v>
+        <v>76</v>
       </c>
       <c r="B33" s="0" t="s">
+        <v>483</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>484</v>
+      </c>
+      <c r="D33" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="E33" s="0" t="s">
         <v>485</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="F33" s="0" t="s">
         <v>486</v>
       </c>
-      <c r="D33" s="0" t="s">
-        <v>189</v>
-      </c>
-      <c r="E33" s="0" t="s">
+      <c r="G33" s="0" t="s">
         <v>487</v>
       </c>
-      <c r="F33" s="0" t="s">
+      <c r="H33" s="0" t="s">
         <v>488</v>
       </c>
-      <c r="G33" s="0" t="s">
+      <c r="I33" s="0" t="s">
         <v>489</v>
       </c>
-      <c r="H33" s="0" t="s">
+      <c r="J33" s="0" t="s">
         <v>490</v>
       </c>
-      <c r="J33" s="0" t="s">
+      <c r="L33" s="0" t="s">
         <v>491</v>
-      </c>
-      <c r="L33" s="0" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>88</v>
+        <v>492</v>
       </c>
       <c r="B34" s="0" t="s">
         <v>493</v>
@@ -5057,7 +5065,7 @@
         <v>494</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>85</v>
+        <v>135</v>
       </c>
       <c r="E34" s="0" t="s">
         <v>495</v>
@@ -5068,112 +5076,118 @@
       <c r="G34" s="0" t="s">
         <v>497</v>
       </c>
-      <c r="H34" s="0" t="s">
+      <c r="I34" s="0" t="s">
         <v>498</v>
       </c>
-      <c r="I34" s="0" t="s">
+      <c r="J34" s="0" t="s">
+        <v>497</v>
+      </c>
+      <c r="L34" s="0" t="s">
         <v>499</v>
-      </c>
-      <c r="J34" s="0" t="s">
-        <v>500</v>
-      </c>
-      <c r="K34" s="0" t="s">
-        <v>501</v>
-      </c>
-      <c r="L34" s="0" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>137</v>
+        <v>191</v>
       </c>
       <c r="B35" s="0" t="s">
+        <v>500</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>501</v>
+      </c>
+      <c r="D35" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="E35" s="0" t="s">
+        <v>502</v>
+      </c>
+      <c r="F35" s="0" t="s">
         <v>503</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="G35" s="0" t="s">
         <v>504</v>
       </c>
-      <c r="D35" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="E35" s="0" t="s">
+      <c r="H35" s="0" t="s">
         <v>505</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="J35" s="0" t="s">
         <v>506</v>
       </c>
-      <c r="G35" s="0" t="s">
+      <c r="L35" s="0" t="s">
         <v>507</v>
-      </c>
-      <c r="H35" s="0" t="s">
-        <v>508</v>
-      </c>
-      <c r="I35" s="0" t="s">
-        <v>509</v>
-      </c>
-      <c r="J35" s="0" t="s">
-        <v>510</v>
-      </c>
-      <c r="K35" s="0" t="s">
-        <v>511</v>
-      </c>
-      <c r="L35" s="0" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>508</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>509</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="E36" s="0" t="s">
+        <v>510</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>511</v>
+      </c>
+      <c r="G36" s="0" t="s">
+        <v>512</v>
+      </c>
+      <c r="H36" s="0" t="s">
         <v>513</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="I36" s="0" t="s">
         <v>514</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="J36" s="0" t="s">
         <v>515</v>
       </c>
-      <c r="D36" s="0" t="s">
+      <c r="K36" s="0" t="s">
         <v>516</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="L36" s="0" t="s">
         <v>517</v>
-      </c>
-      <c r="F36" s="0" t="s">
-        <v>518</v>
-      </c>
-      <c r="G36" s="0" t="s">
-        <v>519</v>
-      </c>
-      <c r="L36" s="0" t="s">
-        <v>520</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>409</v>
+        <v>518</v>
       </c>
       <c r="C37" s="0" t="s">
+        <v>519</v>
+      </c>
+      <c r="D37" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="E37" s="0" t="s">
+        <v>520</v>
+      </c>
+      <c r="F37" s="0" t="s">
         <v>521</v>
       </c>
-      <c r="D37" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="E37" s="0" t="s">
+      <c r="G37" s="0" t="s">
         <v>522</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="H37" s="0" t="s">
         <v>523</v>
       </c>
-      <c r="G37" s="0" t="s">
+      <c r="I37" s="0" t="s">
         <v>524</v>
       </c>
-      <c r="H37" s="0" t="s">
+      <c r="J37" s="0" t="s">
         <v>525</v>
       </c>
-      <c r="J37" s="0" t="s">
+      <c r="K37" s="0" t="s">
         <v>526</v>
       </c>
       <c r="L37" s="0" t="s">
@@ -5191,18 +5205,15 @@
         <v>530</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>116</v>
+        <v>531</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>533</v>
-      </c>
-      <c r="J38" s="0" t="s">
         <v>534</v>
       </c>
       <c r="L38" s="0" t="s">
@@ -5211,72 +5222,95 @@
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
       <c r="B39" s="0" t="s">
+        <v>409</v>
+      </c>
+      <c r="C39" s="0" t="s">
         <v>536</v>
       </c>
-      <c r="C39" s="0" t="s">
+      <c r="D39" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="0" t="s">
         <v>537</v>
       </c>
-      <c r="D39" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="E39" s="0" t="s">
+      <c r="F39" s="0" t="s">
         <v>538</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="G39" s="0" t="s">
         <v>539</v>
       </c>
-      <c r="G39" s="0" t="s">
+      <c r="H39" s="0" t="s">
         <v>540</v>
-      </c>
-      <c r="H39" s="0" t="s">
-        <v>541</v>
-      </c>
-      <c r="I39" s="0" t="s">
-        <v>542</v>
       </c>
       <c r="J39" s="0" t="s">
         <v>541</v>
       </c>
-      <c r="K39" s="0" t="s">
-        <v>543</v>
-      </c>
       <c r="L39" s="0" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
+        <v>543</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>544</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>545</v>
+      </c>
+      <c r="D40" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="E40" s="0" t="s">
+        <v>546</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>547</v>
+      </c>
+      <c r="G40" s="0" t="s">
+        <v>548</v>
+      </c>
+      <c r="J40" s="0" t="s">
+        <v>549</v>
+      </c>
+      <c r="L40" s="0" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="s">
         <v>44</v>
       </c>
-      <c r="B40" s="0" t="s">
-        <v>545</v>
-      </c>
-      <c r="C40" s="0" t="s">
-        <v>546</v>
-      </c>
-      <c r="D40" s="0" t="s">
+      <c r="B41" s="0" t="s">
+        <v>551</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>552</v>
+      </c>
+      <c r="D41" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="E40" s="0" t="s">
-        <v>547</v>
-      </c>
-      <c r="F40" s="0" t="s">
-        <v>548</v>
-      </c>
-      <c r="G40" s="0" t="s">
-        <v>549</v>
-      </c>
-      <c r="H40" s="0" t="s">
-        <v>550</v>
-      </c>
-      <c r="J40" s="0" t="s">
-        <v>551</v>
-      </c>
-      <c r="L40" s="0" t="s">
-        <v>552</v>
+      <c r="E41" s="0" t="s">
+        <v>553</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>554</v>
+      </c>
+      <c r="G41" s="0" t="s">
+        <v>555</v>
+      </c>
+      <c r="H41" s="0" t="s">
+        <v>556</v>
+      </c>
+      <c r="J41" s="0" t="s">
+        <v>557</v>
+      </c>
+      <c r="L41" s="0" t="s">
+        <v>558</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update session data and speaker profiles; add new sessions and modify existing ones
</commit_message>
<xml_diff>
--- a/src/assets/sessionize/data-advanced.xlsx
+++ b/src/assets/sessionize/data-advanced.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="579">
   <si>
     <t>Session Id</t>
   </si>
@@ -251,31 +251,6 @@
     <t>b11e5877-5635-4943-8a71-3ea1a8a1908f</t>
   </si>
   <si>
-    <t>Costruiamo agenti con ADK-js</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Siamo nell’era degli agenti! Non quelli di 007 ma quelli dell’AI!_x000D_
-Ma come funzionano? Come posso crearli? E come posso renderli più specifici per i miei casi d’uso?_x000D_
-Bene in questo workshop vedrai come con ADK-js di Google sia possibile creare agenti e farli interagire tra loro per creare dei workflow completamente gestiti dall’AI._x000D_
-Imparerai le basi e come muovere i primi passi con questo framework in modo da iniziare a capire come integrarli nella tua codebase._x000D_
-Se ti sembra interessante, ci vediamo lì!</t>
-  </si>
-  <si>
-    <t>Luca Del Puppo</t>
-  </si>
-  <si>
-    <t>luca@delpuppo.net</t>
-  </si>
-  <si>
-    <t>Workshop (1+ hr)</t>
-  </si>
-  <si>
-    <t>2ore</t>
-  </si>
-  <si>
-    <t>df577d1f-1e8c-491a-a9de-5c8bbdb91bd7</t>
-  </si>
-  <si>
     <t>Pattern Recognition: identificare il codice invisibile dei non detti</t>
   </si>
   <si>
@@ -333,6 +308,29 @@
     <t>04eb395e-7d8e-4723-8bb0-98d7aa6b15a6</t>
   </si>
   <si>
+    <t>Inferenza locale o remota: un viaggio andata e ritorno!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Come possiamo rendere una nostra web application resiliente, in modo che si possa fare inferenza in locale con Gemini Nano o in remoto con il potente Gemini Pro e far si che il lavoro offline non sia più un problema?_x000D_
+_x000D_
+Beh, in questo workshop avremo modo di capire insieme come fare e come pensare alle strategie per una soluzione basata su modelli locali e modelli SOTA...il tutto in salsa Gemini!</t>
+  </si>
+  <si>
+    <t>Francesco Sciuti</t>
+  </si>
+  <si>
+    <t>francesco@acadevmy.it</t>
+  </si>
+  <si>
+    <t>Workshop (1+ hr)</t>
+  </si>
+  <si>
+    <t>1h 30m</t>
+  </si>
+  <si>
+    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b</t>
+  </si>
+  <si>
     <t>Building Agentic AI Workflows with xAI on Vertex AI: From Code to Action</t>
   </si>
   <si>
@@ -478,12 +476,6 @@
 _x000D_
 Facciamo una scorpacciata di criteri chiari, esempi riutilizzabili e animazioni fluide su browser e webview reali...con una coppia che solo a vederla vi farà passare il reflow!_x000D_
 </t>
-  </si>
-  <si>
-    <t>Francesco Sciuti</t>
-  </si>
-  <si>
-    <t>francesco@acadevmy.it</t>
   </si>
   <si>
     <t>Francesco Sciuti, Emiliano Pisu</t>
@@ -688,6 +680,21 @@
     <t>9bf00943-d891-4eb3-9400-430ab2430d1e</t>
   </si>
   <si>
+    <t>IWD Panel: Quando il futuro era donna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nel 1967 Cosmopolitan dedicava un articolo alle "Computer Girls": la programmazione era il lavoro del futuro e quel futuro era immaginato al femminile. Oggi il settore tech è ancora a forte prevalenza maschile._x000D_
+Cosa è successo nel mezzo e cosa possiamo fare adesso?_x000D_
+_x000D_
+Chiara modera il panel con speaker a confronto su un tema che sembra storico ma è urgente: come mai l'informatica, un settore che negli anni '60 immaginava le donne come protagoniste naturali, è diventato uno dei più sbilanciati in termini di genere?_x000D_
+_x000D_
+Attraverso domande aperte e prospettive diverse, il panel esplora le dinamiche culturali e sistemiche che hanno costruito questo divario, e i segnali, ancora fragili, di un cambiamento possibile._x000D_
+</t>
+  </si>
+  <si>
+    <t>e57ecc81-7677-4f95-a6ed-fc1ed67ec883</t>
+  </si>
+  <si>
     <t>L'essenziale è invisibile agli occhi (ma non a Python): un’introduzione alla steganografia</t>
   </si>
   <si>
@@ -755,6 +762,28 @@
   </si>
   <si>
     <t>d26a7c22-25fc-466d-89ff-c0a77c93f820</t>
+  </si>
+  <si>
+    <t>Costruiamo agenti con ADK-js</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siamo nell’era degli agenti! Non quelli di 007 ma quelli dell’AI!_x000D_
+Ma come funzionano? Come posso crearli? E come posso renderli più specifici per i miei casi d’uso?_x000D_
+Bene in questo workshop vedrai come con ADK-js di Google sia possibile creare agenti e farli interagire tra loro per creare dei workflow completamente gestiti dall’AI._x000D_
+Imparerai le basi e come muovere i primi passi con questo framework in modo da iniziare a capire come integrarli nella tua codebase._x000D_
+Se ti sembra interessante, ci vediamo lì!</t>
+  </si>
+  <si>
+    <t>Luca Del Puppo</t>
+  </si>
+  <si>
+    <t>luca@delpuppo.net</t>
+  </si>
+  <si>
+    <t>2ore</t>
+  </si>
+  <si>
+    <t>df577d1f-1e8c-491a-a9de-5c8bbdb91bd7</t>
   </si>
   <si>
     <t>LLM Testing 101: qualità e metriche di valutazione per sistemi GenAI</t>
@@ -866,12 +895,12 @@
     <t>Bio</t>
   </si>
   <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
     <t>Company Website</t>
   </si>
   <si>
-    <t>LinkedIn</t>
-  </si>
-  <si>
     <t>Instagram</t>
   </si>
   <si>
@@ -914,12 +943,12 @@
     <t xml:space="preserve">I have 9 years of experience as backend developer. I worked on both self hosted and saas solutions and always involved in integration works with different technologies. </t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/luigi-de-bianchi-881309120/</t>
+  </si>
+  <si>
     <t>https://www.klarna.com/it/</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/luigi-de-bianchi-881309120/</t>
-  </si>
-  <si>
     <t>https://sessionize.com/image/d9c1-400o400o1-suawNqFLCc9haUwdaT2PBf.png</t>
   </si>
   <si>
@@ -943,12 +972,12 @@
 I am deeply committed to knowledge sharing and mentorship: through my experience as Sensei @ Dev Dojo IT, I actively support those who want to grow in the frontend world and in designing accessible and scalable interfaces.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/pixu1980</t>
+  </si>
+  <si>
     <t>https://devdojo.it</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/pixu1980</t>
-  </si>
-  <si>
     <t>https://www.instagram.com/pixu1980/</t>
   </si>
   <si>
@@ -976,12 +1005,12 @@
     <t>Federica Merenda is a Post-doc Researcher in Feminist AI. Her dual background in International Law and Political Philosophy coupled with her technical expertise in AI and Robotics shapes her research on the human rights and ethical impact of digital technologies. She is a feminist scholar committed to equal rights and social justice. Her first book on AI in EU migration governance “La condizione disumana. Hannah Arendt, l’intelligenza artificiale e le frontiere digitali” just came out.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/federica-merenda-979b2aba?utm_source=share&amp;utm_campaign=share_via&amp;utm_content=profile&amp;utm_medium=ios_app</t>
+  </si>
+  <si>
     <t>https://www.santannapisa.it/it/federica-merenda</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/federica-merenda-979b2aba?utm_source=share&amp;utm_campaign=share_via&amp;utm_content=profile&amp;utm_medium=ios_app</t>
-  </si>
-  <si>
     <t>https://sessionize.com/image/442b-400o400o1-9XRUwCu9oubMHygXNLLMiH.jpg</t>
   </si>
   <si>
@@ -997,10 +1026,10 @@
     <t>Irene è AI Team Leader in una società di consulenza strategica. Guida un team su progetti di Document AI, RAG e agenti LLM, provando ogni giorno a tenere insieme qualità del codice, architettura, aspettative di business e la realtà, che non sempre collabora. Ha scoperto che la distanza fra una demo che funziona e un sistema in produzione è più lunga di quanto chiunque voglia ammettere. Porta lezioni pratiche, senza hype.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/ireneburresi/</t>
+  </si>
+  <si>
     <t>https://www.valuepartners.com/homepage</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/ireneburresi/</t>
   </si>
   <si>
     <t>https://ireneburresi.dev/</t>
@@ -1047,12 +1076,12 @@
 Sviluppo di applicazioni a microservizi in Java, GoLang e utilizzo di typescript, HTML, CSS per applicazioni web front-end con particolare attenzione alla progettazione grafica.</t>
   </si>
   <si>
+    <t>https://it.linkedin.com/in/valentina-giuffr%C3%A8-coco-972467209</t>
+  </si>
+  <si>
     <t>https://www.tdgroupitalia.it/</t>
   </si>
   <si>
-    <t>https://it.linkedin.com/in/valentina-giuffr%C3%A8-coco-972467209</t>
-  </si>
-  <si>
     <t>https://sessionize.com/image/2909-400o400o1-SLTUqYTrM6P2DUHrK6mxRW.jpg</t>
   </si>
   <si>
@@ -1068,12 +1097,12 @@
     <t>Gregory Pardini è un ingegnere informatico e Tech Lead @ Rosso. Lavora da oltre 6 anni con Flutter in startup. Ha guidato lo sviluppo e il rilascio di prodotti app e web end-to-end, coordinando team tecnici. Si occupa di architetture scalabili, qualità del codice e integrazione di AI agents nei processi di sviluppo.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/gregorypardini/</t>
+  </si>
+  <si>
     <t>https://donarosso.it</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/gregorypardini/</t>
-  </si>
-  <si>
     <t>https://sessionize.com/image/dc92-400o400o1-UPgFd7NbfeQSgtj5jXioLQ.jpg</t>
   </si>
   <si>
@@ -1093,10 +1122,10 @@
 I focus on cloud-native implementations, scalability, continuous delivery practices, resiliency, performance, and observability.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/fornasa/</t>
+  </si>
+  <si>
     <t>https://fornasa.it/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/fornasa/</t>
   </si>
   <si>
     <t>https://www.linkedin.com/in/fornasa</t>
@@ -1146,10 +1175,10 @@
 I'm a Tech Evangelist @Fractal Cloud and a Cloud Native Computing Foundation (CNCF) Ambassador. I'm also an organizer of the Cloud Native Days Italy, fostering collaboration and innovation within the cloud native ecosystem.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/mich-murabito</t>
+  </si>
+  <si>
     <t>https://fractal.cloud</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/mich-murabito</t>
   </si>
   <si>
     <t>https://www.instagram.com/michel_murabito/</t>
@@ -1180,12 +1209,12 @@
 I was also Speaker Director in Radioeco, the Univsersity Radio in Pisa, managing the whole broadcasting platform and curating a Tech-related liveshow</t>
   </si>
   <si>
+    <t>https://linkedin.com/in/pietempesti</t>
+  </si>
+  <si>
     <t>https://it.nttdata.com/</t>
   </si>
   <si>
-    <t>https://linkedin.com/in/pietempesti</t>
-  </si>
-  <si>
     <t>https://sessionize.com/image/2f6e-400o400o1-DwaqfqEXmgdSCX13tkEEey.jpg</t>
   </si>
   <si>
@@ -1209,12 +1238,12 @@
 More on: https://castograziano.com/</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/castograziano/</t>
+  </si>
+  <si>
     <t>https://akamas.io/</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/castograziano/</t>
-  </si>
-  <si>
     <t>https://castograziano.com</t>
   </si>
   <si>
@@ -1235,12 +1264,12 @@
 More info: https://bit.ly/pantarei-mb</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/michela-bertaina</t>
+  </si>
+  <si>
     <t>https://bit.ly/pantarei-mb</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/michela-bertaina</t>
-  </si>
-  <si>
     <t>https://instagram.com/pantarei_mb</t>
   </si>
   <si>
@@ -1262,10 +1291,10 @@
     <t>Giacomo Sergio ha 25 anni di esperienza nel settore IT. Dopo la laurea in Ingegneria e un'esperienza presso il Consorzio Pisa Ricerche, si trasferisce a Vienna lavorando come sviluppatore software in ambito finanziario. Nel 2008 fonda Wondersys. Sotto la sua guida, Wondersys cresce fino a contare oltre 20 dipendenti e fornire servizi e soluzioni IT innovative sia in Italia che all'estero. Appassionatosi ai temi dell'AI ne promuove l'introduzione nelle applicazioni software offerte dall'azienda.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/giacomo-sergio-5047752/</t>
+  </si>
+  <si>
     <t>https://www.wonder-sys.com/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/giacomo-sergio-5047752/</t>
   </si>
   <si>
     <t>https://www.wonder-sys.com/blog-2/</t>
@@ -1318,10 +1347,10 @@
     <t xml:space="preserve">As a computer engineering graduate, I pursued further studies to earn a Master's degree in Bioinformatics and Digital Health Engineering, blending my passion for technology with healthcare.  I currently work as a mobile developer, with a focus on Android software development.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/donatellapasquale/</t>
+  </si>
+  <si>
     <t>https://www.garmin.com</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/donatellapasquale/</t>
   </si>
   <si>
     <t>https://sessionize.com/image/aacf-400o400o1-wdmTqmpTYiomyzL7Nkdd2S.png</t>
@@ -1379,10 +1408,10 @@
     <t>Diego Giorgini is a Head of AI at AI Technologies, based in Pisa, where he develops language models for building Enterprise GenAI Solutions. Always passionate about Artificial Intelligence, he graduated from the University of Pisa with a Master's degree in Computer Science.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/diego-giorgini/</t>
+  </si>
+  <si>
     <t>https://www.linkedin.com/company/aitechnologies</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/diego-giorgini/</t>
   </si>
   <si>
     <t>https://sessionize.com/image/3015-400o400o1-QzueZrtRLaYXfVSqUTKKEj.jpg</t>
@@ -1403,12 +1432,12 @@
 </t>
   </si>
   <si>
+    <t>https://linkedin.com/in/jacopomartellini</t>
+  </si>
+  <si>
     <t>https://aurasensae.com/</t>
   </si>
   <si>
-    <t>https://linkedin.com/in/jacopomartellini</t>
-  </si>
-  <si>
     <t>https://www.instagram.com/jack.lilhammers</t>
   </si>
   <si>
@@ -1433,10 +1462,10 @@
 In his free time, he loves podcasting and running.</t>
   </si>
   <si>
+    <t>https://linkedin.com/in/cortinico</t>
+  </si>
+  <si>
     <t>https://www.reactnative.dev</t>
-  </si>
-  <si>
-    <t>https://linkedin.com/in/cortinico</t>
   </si>
   <si>
     <t>http://ncorti.com</t>
@@ -1458,10 +1487,10 @@
 More on my blog: https://www.lucadivita.it/</t>
   </si>
   <si>
+    <t>https://it.linkedin.com/in/lucadivit</t>
+  </si>
+  <si>
     <t>https://pescara.python.it/</t>
-  </si>
-  <si>
-    <t>https://it.linkedin.com/in/lucadivit</t>
   </si>
   <si>
     <t>https://www.instagram.com/luca_di_vita_</t>
@@ -1488,12 +1517,12 @@
 Cristian has 3 kids, 2 dogs and a Computer Science Degree. </t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/cristian-burrini/</t>
+  </si>
+  <si>
     <t>https://www.google.com</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/cristian-burrini/</t>
-  </si>
-  <si>
     <t>https://sessionize.com/image/9741-400o400o1-GHAp4zQg5wpcoTK2JkEMsH.png</t>
   </si>
   <si>
@@ -1509,12 +1538,12 @@
     <t>Lorenzo Spiridioni is a software engineer at Roxpay with a background in cloud engineering. He designs and operates cloud-native systems, focusing on using modern infrastructure effectively in real-world applications. His work spans performance-sensitive services and machine learning systems in production, with an emphasis on reproducibility, automation, and the practices required to build reliable, scalable systems.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/lorenzo-spiridioni/</t>
+  </si>
+  <si>
     <t>https://www.roxpay.eu/</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/lorenzo-spiridioni/</t>
-  </si>
-  <si>
     <t>https://www.instagram.com/lospiri/</t>
   </si>
   <si>
@@ -1561,9 +1590,6 @@
   </si>
   <si>
     <t>https://sessionize.com/image/7123-400o400o1-wFgsBEnphmM2rKKLn7Xf3Q.jpg</t>
-  </si>
-  <si>
-    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b</t>
   </si>
   <si>
     <t>Francesco</t>
@@ -1583,10 +1609,10 @@
 </t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/francescosciuti/</t>
+  </si>
+  <si>
     <t>https://devmy.it</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/francescosciuti/</t>
   </si>
   <si>
     <t>https://www.instagram.com/Devmy.it/</t>
@@ -1667,12 +1693,12 @@
     <t>As a Green Software Advocate and Tech Sustainability Consultant, my mission is helping companies and professionals build more sustainable, low-carbon digital solutions. Since discovering technology's environmental impact in early 2023, I've become a recognized speaker at major tech conferences and co-founded Green Software Italia community. I believe in responsible technology that creates positive impact for both businesses and the environment.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/valeria-salis/</t>
+  </si>
+  <si>
     <t>https://valeriasalis.com/</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/valeria-salis/</t>
-  </si>
-  <si>
     <t>https://www.instagram.com/_valls_/</t>
   </si>
   <si>
@@ -1691,12 +1717,12 @@
     <t>Passionate about technology work in the IT industry since 2015. From Android through the web to Flutter helps companies to get their target.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/camillo-bucciarelli/</t>
+  </si>
+  <si>
     <t>https://camillobucciarelli.dev</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/camillo-bucciarelli/</t>
-  </si>
-  <si>
     <t>https://sessionize.com/image/a56c-400o400o1-GdsMQ2AQ18rTTXnCK3zt6S.jpg</t>
   </si>
   <si>
@@ -1716,10 +1742,10 @@
 Crede negli spazi dove ogni differenza - di genere, etnia, corpo, neurodiversità - sia accolta. Nomina i bias, li riconosce, ci lavora ogni giorno.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/monjadariva/</t>
+  </si>
+  <si>
     <t>https://monjadariva.it</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/monjadariva/</t>
   </si>
   <si>
     <t>https://instagram.com/monja.dariva</t>
@@ -1747,10 +1773,10 @@
 In addition to studying, I love playing role-playing games, skateboarding and playing Magic the Gathering.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/giorgiobasile00/</t>
+  </si>
+  <si>
     <t>https://bacarotech.github.io/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/giorgiobasile00/</t>
   </si>
   <si>
     <t>https://www.instagram.com/bacarotechofficial/</t>
@@ -1772,12 +1798,12 @@
 </t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/federico-paolinelli-2374954/</t>
+  </si>
+  <si>
     <t>https://www.redhat.com/en</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/federico-paolinelli-2374954/</t>
-  </si>
-  <si>
     <t>https://fedepaol.github.io</t>
   </si>
   <si>
@@ -1796,12 +1822,12 @@
     <t xml:space="preserve">Senior AI Engineer @Netflix |  PHD candidate in xAI |AI Expert Consultant @Tegus &amp; @Wivenn |Technical Reviewer@Packt |2024 AI Apprentice@Google | International AI Speaker(Linkedin Top Voice) </t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/mannai-mortadha/</t>
+  </si>
+  <si>
     <t>https://www.mann-ai.com/</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/mannai-mortadha/</t>
-  </si>
-  <si>
     <t>https://www.instagram.com/mortadha_mannai/</t>
   </si>
   <si>
@@ -1826,10 +1852,10 @@
     <t>Christian Liebel is a developer with a passion for modern web technologies. He has been recognized as a Microsoft Most Valuable Professional (MVP) and a Google Developer Expert (GDE) and speaks at user groups and conferences worldwide. As a member of the W3C Technical Architecture Group (TAG), he helps push the boundaries of the web.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/christianliebel/</t>
+  </si>
+  <si>
     <t>https://www.thinktecture.com</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/christianliebel/</t>
   </si>
   <si>
     <t>https://www.instagram.com/chliebel/</t>
@@ -1880,21 +1906,18 @@
 In my free time, I love studying new technologies, improving myself, creating YouTube content or writing technical articles. I can’t stay without trail running and love to do it in my love Dolomiti.</t>
   </si>
   <si>
+    <t>https://www.linkedin.com/in/lucadelpuppo/</t>
+  </si>
+  <si>
     <t>https://www.nearform.com/</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/lucadelpuppo/</t>
-  </si>
-  <si>
     <t>https://www.delpuppo.net/</t>
   </si>
   <si>
     <t>https://sessionize.com/image/09ed-400o400o1-Mtu422U1R2UjEixBL8dDea.jpg</t>
   </si>
   <si>
-    <t>e57ecc81-7677-4f95-a6ed-fc1ed67ec883</t>
-  </si>
-  <si>
     <t>Chiara</t>
   </si>
   <si>
@@ -1930,10 +1953,10 @@
     <t>Daniela Petruzalek is a developer relations engineer at Google focused on Google Cloud Platform. Her specialisation is backend development and data engineering. She has previously worked at companies like JPMorgan, Oracle and ThoughtWorks. On her spare time she contributes to open source, plays video games and pets random cats on the streets.</t>
   </si>
   <si>
+    <t>https://linkedin.com/in/petruzalek</t>
+  </si>
+  <si>
     <t>https://cloud.google.com</t>
-  </si>
-  <si>
-    <t>https://linkedin.com/in/petruzalek</t>
   </si>
   <si>
     <t>https://danicat.dev</t>
@@ -2017,7 +2040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A1:V34"/>
+  <dimension ref="A1:V36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2462,7 +2485,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0">
-        <v>1133878</v>
+        <v>1134864</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>73</v>
@@ -2480,13 +2503,13 @@
         <v>75</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
       <c r="J8" s="0" t="s">
         <v>58</v>
@@ -2495,25 +2518,25 @@
         <v>42</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="M8" s="0" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
       <c r="N8" s="5">
-        <v>46085.527172766204</v>
+        <v>46056.871177777779</v>
       </c>
       <c r="O8" s="5">
-        <v>46085.540961030092</v>
+        <v>46057.299867905094</v>
       </c>
       <c r="P8" s="0" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="Q8" s="5">
         <v>46130.465277777774</v>
       </c>
       <c r="R8" s="0">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="U8" s="0">
         <v>0</v>
@@ -2524,7 +2547,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0">
-        <v>1134864</v>
+        <v>1148459</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>80</v>
@@ -2542,7 +2565,7 @@
         <v>82</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="H9" s="0" t="s">
         <v>40</v>
@@ -2551,25 +2574,25 @@
         <v>28</v>
       </c>
       <c r="J9" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L9" s="0" t="s">
         <v>33</v>
       </c>
       <c r="M9" s="0" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="N9" s="5">
-        <v>46056.871177777779</v>
-      </c>
-      <c r="O9" s="5">
-        <v>46057.299867905094</v>
+        <v>46087.777417476849</v>
+      </c>
+      <c r="O9" s="0" t="s">
+        <v>33</v>
       </c>
       <c r="P9" s="0" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Q9" s="5">
         <v>46130.465277777774</v>
@@ -2581,63 +2604,63 @@
         <v>0</v>
       </c>
       <c r="V9" s="0" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0">
-        <v>1148459</v>
+        <v>1203376</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="E10" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="D10" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>90</v>
-      </c>
       <c r="F10" s="0" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G10" s="0" t="s">
         <v>26</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>40</v>
+        <v>89</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>28</v>
+        <v>90</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="K10" s="0" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="L10" s="0" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="M10" s="0" t="s">
         <v>43</v>
       </c>
       <c r="N10" s="5">
-        <v>46087.777417476849</v>
+        <v>46120.84242144676</v>
       </c>
       <c r="O10" s="0" t="s">
         <v>33</v>
       </c>
       <c r="P10" s="0" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="Q10" s="5">
         <v>46130.465277777774</v>
       </c>
       <c r="R10" s="0">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="U10" s="0">
         <v>0</v>
@@ -2790,7 +2813,7 @@
         <v>108</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H13" s="0" t="s">
         <v>40</v>
@@ -2914,7 +2937,7 @@
         <v>121</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H15" s="0" t="s">
         <v>66</v>
@@ -2979,7 +3002,7 @@
         <v>26</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="I16" s="0" t="s">
         <v>125</v>
@@ -3009,7 +3032,7 @@
         <v>46130.597222222219</v>
       </c>
       <c r="R16" s="0">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="U16" s="0">
         <v>0</v>
@@ -3029,13 +3052,13 @@
         <v>127</v>
       </c>
       <c r="D17" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="0" t="s">
         <v>128</v>
-      </c>
-      <c r="E17" s="0" t="s">
-        <v>129</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>130</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>103</v>
@@ -3077,7 +3100,7 @@
         <v>0</v>
       </c>
       <c r="V17" s="0" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18">
@@ -3085,22 +3108,22 @@
         <v>1148693</v>
       </c>
       <c r="B18" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" s="0" t="s">
         <v>132</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="E18" s="0" t="s">
         <v>133</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="F18" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="E18" s="0" t="s">
-        <v>135</v>
-      </c>
-      <c r="F18" s="0" t="s">
-        <v>136</v>
-      </c>
       <c r="G18" s="0" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H18" s="0" t="s">
         <v>66</v>
@@ -3118,7 +3141,7 @@
         <v>33</v>
       </c>
       <c r="M18" s="0" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="N18" s="5">
         <v>46080.807078935184</v>
@@ -3139,7 +3162,7 @@
         <v>0</v>
       </c>
       <c r="V18" s="0" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19">
@@ -3147,22 +3170,22 @@
         <v>1123087</v>
       </c>
       <c r="B19" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" s="0" t="s">
         <v>138</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="E19" s="0" t="s">
         <v>139</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="F19" s="0" t="s">
         <v>140</v>
       </c>
-      <c r="E19" s="0" t="s">
+      <c r="G19" s="0" t="s">
         <v>141</v>
-      </c>
-      <c r="F19" s="0" t="s">
-        <v>142</v>
-      </c>
-      <c r="G19" s="0" t="s">
-        <v>143</v>
       </c>
       <c r="H19" s="0" t="s">
         <v>40</v>
@@ -3180,7 +3203,7 @@
         <v>33</v>
       </c>
       <c r="M19" s="0" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="N19" s="5">
         <v>46110.370604861106</v>
@@ -3201,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="V19" s="0" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20">
@@ -3209,22 +3232,22 @@
         <v>1149006</v>
       </c>
       <c r="B20" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="0" t="s">
         <v>145</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="E20" s="0" t="s">
         <v>146</v>
       </c>
-      <c r="D20" s="0" t="s">
-        <v>147</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>148</v>
-      </c>
       <c r="F20" s="0" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G20" s="0" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H20" s="0" t="s">
         <v>66</v>
@@ -3263,7 +3286,7 @@
         <v>0</v>
       </c>
       <c r="V20" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21">
@@ -3271,19 +3294,19 @@
         <v>1154402</v>
       </c>
       <c r="B21" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="D21" s="0" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="E21" s="0" t="s">
         <v>151</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>152</v>
-      </c>
-      <c r="E21" s="0" t="s">
-        <v>153</v>
-      </c>
       <c r="F21" s="0" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G21" s="0" t="s">
         <v>26</v>
@@ -3325,7 +3348,7 @@
         <v>0</v>
       </c>
       <c r="V21" s="0" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="22">
@@ -3333,22 +3356,22 @@
         <v>1149301</v>
       </c>
       <c r="B22" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="D22" s="0" t="s">
         <v>155</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="E22" s="0" t="s">
         <v>156</v>
       </c>
-      <c r="D22" s="0" t="s">
-        <v>157</v>
-      </c>
-      <c r="E22" s="0" t="s">
-        <v>158</v>
-      </c>
       <c r="F22" s="0" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H22" s="0" t="s">
         <v>66</v>
@@ -3360,13 +3383,13 @@
         <v>58</v>
       </c>
       <c r="K22" s="0" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="L22" s="0" t="s">
         <v>33</v>
       </c>
       <c r="M22" s="0" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="N22" s="5">
         <v>46095.713437997685</v>
@@ -3387,7 +3410,7 @@
         <v>0</v>
       </c>
       <c r="V22" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="23">
@@ -3395,19 +3418,19 @@
         <v>1149383</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="D23" s="0" t="s">
         <v>161</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="E23" s="0" t="s">
         <v>162</v>
       </c>
-      <c r="D23" s="0" t="s">
-        <v>163</v>
-      </c>
-      <c r="E23" s="0" t="s">
-        <v>164</v>
-      </c>
       <c r="F23" s="0" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>26</v>
@@ -3449,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="V23" s="0" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24">
@@ -3457,19 +3480,19 @@
         <v>1151362</v>
       </c>
       <c r="B24" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="D24" s="0" t="s">
         <v>166</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="E24" s="0" t="s">
         <v>167</v>
       </c>
-      <c r="D24" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="E24" s="0" t="s">
-        <v>169</v>
-      </c>
       <c r="F24" s="0" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G24" s="0" t="s">
         <v>26</v>
@@ -3511,7 +3534,7 @@
         <v>0</v>
       </c>
       <c r="V24" s="0" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25">
@@ -3519,22 +3542,22 @@
         <v>1155630</v>
       </c>
       <c r="B25" s="0" t="s">
+        <v>169</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" s="0" t="s">
         <v>171</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="E25" s="0" t="s">
         <v>172</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="F25" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="G25" s="0" t="s">
         <v>173</v>
-      </c>
-      <c r="E25" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="F25" s="0" t="s">
-        <v>173</v>
-      </c>
-      <c r="G25" s="0" t="s">
-        <v>175</v>
       </c>
       <c r="H25" s="0" t="s">
         <v>40</v>
@@ -3573,7 +3596,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="0" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26">
@@ -3581,19 +3604,19 @@
         <v>1200474</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="D26" s="0" t="s">
         <v>177</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="E26" s="0" t="s">
         <v>178</v>
       </c>
-      <c r="D26" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="E26" s="0" t="s">
-        <v>180</v>
-      </c>
       <c r="F26" s="0" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G26" s="0" t="s">
         <v>26</v>
@@ -3608,19 +3631,19 @@
         <v>29</v>
       </c>
       <c r="K26" s="0" t="s">
-        <v>159</v>
+        <v>42</v>
       </c>
       <c r="L26" s="0" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="M26" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="N26" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="O26" s="0" t="s">
-        <v>33</v>
+      <c r="N26" s="5">
+        <v>46120.84242144676</v>
+      </c>
+      <c r="O26" s="5">
+        <v>46120.882133599538</v>
       </c>
       <c r="P26" s="0" t="s">
         <v>44</v>
@@ -3635,30 +3658,30 @@
         <v>0</v>
       </c>
       <c r="V26" s="0" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0">
-        <v>1105608</v>
+        <v>1203288</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>185</v>
+        <v>119</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>186</v>
+        <v>120</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>185</v>
+        <v>119</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>143</v>
+        <v>77</v>
       </c>
       <c r="H27" s="0" t="s">
         <v>66</v>
@@ -3679,16 +3702,16 @@
         <v>43</v>
       </c>
       <c r="N27" s="5">
-        <v>46044.86471519676</v>
+        <v>46120.84242144676</v>
       </c>
       <c r="O27" s="5">
-        <v>46046.3336130787</v>
+        <v>46120.846439814813</v>
       </c>
       <c r="P27" s="0" t="s">
         <v>51</v>
       </c>
       <c r="Q27" s="5">
-        <v>46130.684027777774</v>
+        <v>46130.666666666664</v>
       </c>
       <c r="R27" s="0">
         <v>25</v>
@@ -3697,30 +3720,30 @@
         <v>0</v>
       </c>
       <c r="V27" s="0" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0">
-        <v>1145869</v>
+        <v>1105608</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>26</v>
+        <v>141</v>
       </c>
       <c r="H28" s="0" t="s">
         <v>66</v>
@@ -3729,7 +3752,7 @@
         <v>28</v>
       </c>
       <c r="J28" s="0" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="K28" s="0" t="s">
         <v>42</v>
@@ -3741,13 +3764,13 @@
         <v>43</v>
       </c>
       <c r="N28" s="5">
-        <v>46100.503021724537</v>
+        <v>46044.86471519676</v>
       </c>
       <c r="O28" s="5">
-        <v>46100.520990243051</v>
+        <v>46046.3336130787</v>
       </c>
       <c r="P28" s="0" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="Q28" s="5">
         <v>46130.684027777774</v>
@@ -3759,33 +3782,33 @@
         <v>0</v>
       </c>
       <c r="V28" s="0" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0">
-        <v>1124260</v>
+        <v>1145869</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>175</v>
+        <v>26</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="I29" s="0" t="s">
         <v>28</v>
@@ -3803,48 +3826,48 @@
         <v>43</v>
       </c>
       <c r="N29" s="5">
-        <v>46087.774690972219</v>
+        <v>46100.503021724537</v>
       </c>
       <c r="O29" s="5">
-        <v>46087.792176655094</v>
+        <v>46100.520990243051</v>
       </c>
       <c r="P29" s="0" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="Q29" s="5">
-        <v>46130.722222222219</v>
+        <v>46130.684027777774</v>
       </c>
       <c r="R29" s="0">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="U29" s="0">
         <v>0</v>
       </c>
       <c r="V29" s="0" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0">
-        <v>1125184</v>
+        <v>1124260</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>202</v>
+        <v>173</v>
       </c>
       <c r="H30" s="0" t="s">
         <v>40</v>
@@ -3853,10 +3876,10 @@
         <v>28</v>
       </c>
       <c r="J30" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="K30" s="0" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="L30" s="0" t="s">
         <v>33</v>
@@ -3865,13 +3888,13 @@
         <v>43</v>
       </c>
       <c r="N30" s="5">
-        <v>46044.86471519676</v>
+        <v>46087.774690972219</v>
       </c>
       <c r="O30" s="5">
-        <v>46058.74419375</v>
+        <v>46087.792176655094</v>
       </c>
       <c r="P30" s="0" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="Q30" s="5">
         <v>46130.722222222219</v>
@@ -3883,30 +3906,30 @@
         <v>0</v>
       </c>
       <c r="V30" s="0" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0">
-        <v>1147845</v>
+        <v>1125184</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="E31" s="0" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>26</v>
+        <v>203</v>
       </c>
       <c r="H31" s="0" t="s">
         <v>40</v>
@@ -3915,10 +3938,10 @@
         <v>28</v>
       </c>
       <c r="J31" s="0" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="K31" s="0" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L31" s="0" t="s">
         <v>33</v>
@@ -3927,13 +3950,13 @@
         <v>43</v>
       </c>
       <c r="N31" s="5">
-        <v>46087.777417476849</v>
+        <v>46044.86471519676</v>
       </c>
       <c r="O31" s="5">
-        <v>46087.79654938657</v>
+        <v>46058.74419375</v>
       </c>
       <c r="P31" s="0" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="Q31" s="5">
         <v>46130.722222222219</v>
@@ -3945,92 +3968,92 @@
         <v>0</v>
       </c>
       <c r="V31" s="0" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0">
-        <v>1148589</v>
+        <v>1133878</v>
       </c>
       <c r="B32" s="0" t="s">
+        <v>205</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="D32" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="G32" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="H32" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="I32" s="0" t="s">
         <v>209</v>
       </c>
-      <c r="C32" s="0" t="s">
-        <v>210</v>
-      </c>
-      <c r="D32" s="0" t="s">
-        <v>211</v>
-      </c>
-      <c r="E32" s="0" t="s">
-        <v>212</v>
-      </c>
-      <c r="F32" s="0" t="s">
-        <v>213</v>
-      </c>
-      <c r="G32" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="H32" s="0" t="s">
-        <v>66</v>
-      </c>
-      <c r="I32" s="0" t="s">
-        <v>28</v>
-      </c>
       <c r="J32" s="0" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="K32" s="0" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="L32" s="0" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="M32" s="0" t="s">
         <v>43</v>
       </c>
       <c r="N32" s="5">
-        <v>46080.807078935184</v>
+        <v>46085.527172766204</v>
       </c>
       <c r="O32" s="5">
-        <v>46083.334888888887</v>
+        <v>46085.540961030092</v>
       </c>
       <c r="P32" s="0" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="Q32" s="5">
-        <v>46130.756944444445</v>
+        <v>46130.722222222219</v>
       </c>
       <c r="R32" s="0">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="U32" s="0">
         <v>0</v>
       </c>
       <c r="V32" s="0" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0">
-        <v>1154675</v>
+        <v>1147845</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>202</v>
+        <v>26</v>
       </c>
       <c r="H33" s="0" t="s">
         <v>40</v>
@@ -4051,16 +4074,16 @@
         <v>43</v>
       </c>
       <c r="N33" s="5">
-        <v>46087.776362002311</v>
+        <v>46087.777417476849</v>
       </c>
       <c r="O33" s="5">
-        <v>46088.7549028125</v>
+        <v>46087.79654938657</v>
       </c>
       <c r="P33" s="0" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Q33" s="5">
-        <v>46130.756944444445</v>
+        <v>46130.722222222219</v>
       </c>
       <c r="R33" s="0">
         <v>50</v>
@@ -4069,30 +4092,30 @@
         <v>0</v>
       </c>
       <c r="V33" s="0" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0">
-        <v>1143717</v>
+        <v>1148589</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H34" s="0" t="s">
         <v>66</v>
@@ -4101,28 +4124,28 @@
         <v>28</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="K34" s="0" t="s">
         <v>30</v>
       </c>
       <c r="L34" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="M34" s="0" t="s">
-        <v>225</v>
+        <v>43</v>
       </c>
       <c r="N34" s="5">
-        <v>46063.895173379628</v>
+        <v>46080.807078935184</v>
       </c>
       <c r="O34" s="5">
-        <v>46076.880179664353</v>
+        <v>46083.334888888887</v>
       </c>
       <c r="P34" s="0" t="s">
         <v>34</v>
       </c>
       <c r="Q34" s="5">
-        <v>46130.774305555555</v>
+        <v>46130.756944444445</v>
       </c>
       <c r="R34" s="0">
         <v>25</v>
@@ -4131,7 +4154,131 @@
         <v>0</v>
       </c>
       <c r="V34" s="0" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0">
+        <v>1154675</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="D35" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="E35" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="F35" s="0" t="s">
         <v>226</v>
+      </c>
+      <c r="G35" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="H35" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="I35" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="J35" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="K35" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="L35" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="M35" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="N35" s="5">
+        <v>46087.776362002311</v>
+      </c>
+      <c r="O35" s="5">
+        <v>46088.7549028125</v>
+      </c>
+      <c r="P35" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q35" s="5">
+        <v>46130.756944444445</v>
+      </c>
+      <c r="R35" s="0">
+        <v>50</v>
+      </c>
+      <c r="U35" s="0">
+        <v>0</v>
+      </c>
+      <c r="V35" s="0" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0">
+        <v>1143717</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="E36" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="G36" s="0" t="s">
+        <v>173</v>
+      </c>
+      <c r="H36" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="I36" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="J36" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="K36" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="L36" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="M36" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="N36" s="5">
+        <v>46063.895173379628</v>
+      </c>
+      <c r="O36" s="5">
+        <v>46076.880179664353</v>
+      </c>
+      <c r="P36" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q36" s="5">
+        <v>46130.774305555555</v>
+      </c>
+      <c r="R36" s="0">
+        <v>25</v>
+      </c>
+      <c r="U36" s="0">
+        <v>0</v>
+      </c>
+      <c r="V36" s="0" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -4146,278 +4293,278 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="L5" s="0" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="L6" s="0" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>283</v>
-      </c>
-      <c r="H7" s="0" t="s">
-        <v>284</v>
+        <v>290</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>291</v>
       </c>
       <c r="L7" s="0" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10">
@@ -4425,159 +4572,159 @@
         <v>52</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>49</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="L10" s="0" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>313</v>
-      </c>
-      <c r="H11" s="0" t="s">
-        <v>314</v>
+        <v>320</v>
+      </c>
+      <c r="G11" s="0" t="s">
+        <v>321</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="L11" s="0" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="K12" s="0" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="L12" s="0" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>56</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="L13" s="0" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
     </row>
     <row r="15">
@@ -4585,266 +4732,266 @@
         <v>116</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>114</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="K16" s="0" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="L16" s="0" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="H17" s="0" t="s">
-        <v>370</v>
+        <v>376</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>377</v>
       </c>
       <c r="L17" s="0" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="L18" s="0" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>384</v>
-      </c>
-      <c r="G19" s="0" t="s">
-        <v>292</v>
+        <v>391</v>
+      </c>
+      <c r="H19" s="0" t="s">
+        <v>300</v>
       </c>
       <c r="L19" s="0" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="L20" s="0" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>400</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>401</v>
+      </c>
+      <c r="D21" s="0" t="s">
         <v>192</v>
       </c>
-      <c r="B21" s="0" t="s">
-        <v>393</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>394</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>191</v>
-      </c>
       <c r="E21" s="0" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="L21" s="0" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="L22" s="0" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="L23" s="0" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
     </row>
     <row r="24">
@@ -4852,63 +4999,63 @@
         <v>45</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="D24" s="0" t="s">
         <v>39</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="L24" s="0" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="L25" s="0" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
     </row>
     <row r="26">
@@ -4916,31 +5063,31 @@
         <v>67</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="D26" s="0" t="s">
         <v>64</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="L26" s="0" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
     </row>
     <row r="27">
@@ -4948,150 +5095,150 @@
         <v>72</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="D27" s="0" t="s">
         <v>71</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>443</v>
-      </c>
-      <c r="H27" s="0" t="s">
-        <v>444</v>
+        <v>450</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>451</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="L27" s="0" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="L28" s="0" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>454</v>
+        <v>91</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>129</v>
+        <v>88</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>457</v>
+        <v>463</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
       <c r="J29" s="0" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
       <c r="K29" s="0" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
       <c r="L29" s="0" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>470</v>
-      </c>
-      <c r="H30" s="0" t="s">
-        <v>471</v>
+        <v>476</v>
+      </c>
+      <c r="G30" s="0" t="s">
+        <v>477</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
       <c r="K30" s="0" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
       <c r="L30" s="0" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>481</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>482</v>
+      </c>
+      <c r="D31" s="0" t="s">
         <v>187</v>
       </c>
-      <c r="B31" s="0" t="s">
-        <v>475</v>
-      </c>
-      <c r="C31" s="0" t="s">
-        <v>476</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>186</v>
-      </c>
       <c r="E31" s="0" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>478</v>
-      </c>
-      <c r="H31" s="0" t="s">
-        <v>479</v>
+        <v>484</v>
+      </c>
+      <c r="G31" s="0" t="s">
+        <v>485</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="L31" s="0" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
     </row>
     <row r="32">
@@ -5099,165 +5246,165 @@
         <v>110</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
       <c r="D32" s="0" t="s">
         <v>109</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
       <c r="L32" s="0" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>496</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>497</v>
+      </c>
+      <c r="D33" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="B33" s="0" t="s">
-        <v>490</v>
-      </c>
-      <c r="C33" s="0" t="s">
-        <v>491</v>
-      </c>
-      <c r="D33" s="0" t="s">
-        <v>196</v>
-      </c>
       <c r="E33" s="0" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="J33" s="0" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="L33" s="0" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="L34" s="0" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="I35" s="0" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="J35" s="0" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="L35" s="0" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="J36" s="0" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
     </row>
     <row r="37">
@@ -5265,37 +5412,37 @@
         <v>98</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D37" s="0" t="s">
         <v>95</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="I37" s="0" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="J37" s="0" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="K37" s="0" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="L37" s="0" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="38">
@@ -5303,124 +5450,124 @@
         <v>105</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="D38" s="0" t="s">
         <v>102</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="J38" s="0" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="K38" s="0" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="L38" s="0" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="E39" s="0" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="F39" s="0" t="s">
-        <v>548</v>
-      </c>
-      <c r="H39" s="0" t="s">
-        <v>549</v>
+        <v>554</v>
+      </c>
+      <c r="G39" s="0" t="s">
+        <v>555</v>
       </c>
       <c r="L39" s="0" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
-        <v>79</v>
+        <v>210</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>76</v>
+        <v>208</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="L40" s="0" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>558</v>
+        <v>183</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="D41" s="0" t="s">
         <v>120</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>562</v>
-      </c>
-      <c r="H41" s="0" t="s">
-        <v>563</v>
+        <v>567</v>
+      </c>
+      <c r="G41" s="0" t="s">
+        <v>568</v>
       </c>
       <c r="J41" s="0" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="L41" s="0" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
     </row>
     <row r="42">
@@ -5428,31 +5575,31 @@
         <v>35</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="D42" s="0" t="s">
         <v>25</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="F42" s="0" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
       <c r="H42" s="0" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="J42" s="0" t="s">
-        <v>572</v>
+        <v>577</v>
       </c>
       <c r="L42" s="0" t="s">
-        <v>573</v>
+        <v>578</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update session details and add new speakers; modify workshop requirements and styles
</commit_message>
<xml_diff>
--- a/src/assets/sessionize/data-advanced.xlsx
+++ b/src/assets/sessionize/data-advanced.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="606">
   <si>
     <t>Session Id</t>
   </si>
@@ -81,10 +81,10 @@
     <t>Speaker Ids</t>
   </si>
   <si>
-    <t>Advanced Techniques for Building Agents with ADK and Vertex AI</t>
-  </si>
-  <si>
-    <t>Agent Development Kit (ADK) is an open source agent development framework built by Google. In this talk we are going to see how to leverage Vertex AI to make production-ready agents that include features like memory, session management, artifact management, RAG and others. The session will walk you through the development of an “Executive Assistant” agent that will learn not only about your tasks, but your preferences. Even if you have never built an agent before, in this talk you will learn how to quickly ramp up using Gemini CLI, the developer knowledge MCP and codewiki, for a truly modern agent development experience.</t>
+    <t>Build your own executive assistant with ADK and Gemini</t>
+  </si>
+  <si>
+    <t>Agent Development Kit (ADK) is an open source agent development framework built by Google. In this talk we are going to see how to leverage ADK and Gemini to make production-ready agents that include features like memory, session management, tools and others. The session will walk you through the development of an “Executive Assistant” agent that will learn not only about your tasks, but your preferences. Even if you have never built an agent before, in this talk you will learn how to quickly ramp up using Gemini CLI, the developer knowledge MCP and codewiki, for a truly modern agent development experience.</t>
   </si>
   <si>
     <t>Daniela Petruzalek</t>
@@ -308,27 +308,20 @@
     <t>04eb395e-7d8e-4723-8bb0-98d7aa6b15a6</t>
   </si>
   <si>
-    <t>Inferenza locale o remota: un viaggio andata e ritorno!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Come possiamo rendere una nostra web application resiliente, in modo che si possa fare inferenza in locale con Gemini Nano o in remoto con il potente Gemini Pro e far si che il lavoro offline non sia più un problema?_x000D_
-_x000D_
-Beh, in questo workshop avremo modo di capire insieme come fare e come pensare alle strategie per una soluzione basata su modelli locali e modelli SOTA...il tutto in salsa Gemini!</t>
-  </si>
-  <si>
-    <t>Francesco Sciuti</t>
-  </si>
-  <si>
-    <t>francesco@acadevmy.it</t>
+    <t>Build a photo restoration app using Genkit Go and Nano Banana Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In this codelab, we are going to build GlowUp, a photo restoration tool. GlowUp uses AI to restore old, damaged, or black-and-white photos, creating high-quality 4K color images. You can use this tool to give a new life to your family photos, or even adapt it to restore damaged illustrations, drawings, paintings or other forms of images._x000D_
+_x000D_
+You will use Genkit Go to implement the application logic and Gemini 3 Pro Image (also known as Nano Banana Pro) as the model to process the photos._x000D_
+_x000D_
+Previous knowledge of Go is not strictly required, but recommended.</t>
   </si>
   <si>
     <t>Workshop (1+ hr)</t>
   </si>
   <si>
-    <t>1h 30m</t>
-  </si>
-  <si>
-    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b</t>
+    <t>It is doable in 1 hour, but can be done in a more relaxed pace if more time is allocated</t>
   </si>
   <si>
     <t>Building Agentic AI Workflows with xAI on Vertex AI: From Code to Action</t>
@@ -360,27 +353,6 @@
   </si>
   <si>
     <t>d3f982bf-06f2-4a7a-ac5a-2479f4cec0b2</t>
-  </si>
-  <si>
-    <t>What’s New in Web? 2026 Edition</t>
-  </si>
-  <si>
-    <t>Christian is a member of the World Wide Web’s architecture board, the Technical Architecture Group (TAG) of W3C. As such, he has insights into what’s going on in the web platform. In his session, you'll gain insights into the latest discussions among standards bodies, browser vendors, and web developers. And you have the opportunity to report your wishes back to the Web’s architecture board. Don't miss this opportunity to stay updated on the forefront of web technologies.</t>
-  </si>
-  <si>
-    <t>Christian Liebel</t>
-  </si>
-  <si>
-    <t>christian@liebel.org</t>
-  </si>
-  <si>
-    <t>Web</t>
-  </si>
-  <si>
-    <t>Germany</t>
-  </si>
-  <si>
-    <t>d7da8026-334b-42d8-aec9-324bf1bb6ec4</t>
   </si>
   <si>
     <t>From shy contributor to (kinda) confident community leader</t>
@@ -399,6 +371,32 @@
     <t>bc261ce0-3d86-40a4-9c62-764d0115dc92</t>
   </si>
   <si>
+    <t>60fps o niente: Rendering Pipeline a suon di esempi pratici!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se un'animazione scatta o una UI risponde in ritardo, non imprecare: la colpa non e' sempre del browser! Hai mai sentito parlare della rendering pipeline? Se la risposta è no, ti assicuriamo che avresti dovuto!_x000D_
+_x000D_
+Ottenere le giuste performance non è sempre gratis...impariamo quindi cosa sia la render pipeline e capiamo come quanto stupefacente ottimizzare ogni scelta alle API e alle proprieta coinvolte, sia lato CSS sia lato JavaScript._x000D_
+_x000D_
+Facciamo una scorpacciata di criteri chiari, esempi riutilizzabili e animazioni fluide su browser e webview reali...con una coppia che solo a vederla vi farà passare il reflow!_x000D_
+</t>
+  </si>
+  <si>
+    <t>Francesco Sciuti</t>
+  </si>
+  <si>
+    <t>francesco@acadevmy.it</t>
+  </si>
+  <si>
+    <t>Francesco Sciuti, Emiliano Pisu</t>
+  </si>
+  <si>
+    <t>Web</t>
+  </si>
+  <si>
+    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b, 05ed4b4a-5d57-4602-bb4e-8d55efad3e0f</t>
+  </si>
+  <si>
     <t>Developer Mezzosangue: Padroneggiare l'Alchimia dell'IA e del Personal Branding</t>
   </si>
   <si>
@@ -432,6 +430,24 @@
     <t>4d9b6e94-52a6-4d13-a981-e9bbf8acc867</t>
   </si>
   <si>
+    <t>What’s New in Web? 2026 Edition</t>
+  </si>
+  <si>
+    <t>Christian is a member of the World Wide Web’s architecture board, the Technical Architecture Group (TAG) of W3C. As such, he has insights into what’s going on in the web platform. In his session, you'll gain insights into the latest discussions among standards bodies, browser vendors, and web developers. And you have the opportunity to report your wishes back to the Web’s architecture board. Don't miss this opportunity to stay updated on the forefront of web technologies.</t>
+  </si>
+  <si>
+    <t>Christian Liebel</t>
+  </si>
+  <si>
+    <t>christian@liebel.org</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>d7da8026-334b-42d8-aec9-324bf1bb6ec4</t>
+  </si>
+  <si>
     <t>Hack the Job Title: Il lavoro reale dietro i titoli tech</t>
   </si>
   <si>
@@ -454,34 +470,18 @@
     <t>e57ecc81-7677-4f95-a6ed-fc1ed67ec883, 1123eb91-f592-42a9-bf03-0d8bd91e9813, b9946904-9607-412b-bcc9-4eb160da4881, dd7b13a9-c8b7-4428-b4bf-10224b38b3ef</t>
   </si>
   <si>
-    <t>Build a photo restoration app using Genkit Go and Nano Banana Pro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In this codelab, we are going to build GlowUp, a photo restoration tool. GlowUp uses AI to restore old, damaged, or black-and-white photos, creating high-quality 4K color images. You can use this tool to give a new life to your family photos, or even adapt it to restore damaged illustrations, drawings, paintings or other forms of images._x000D_
-_x000D_
-You will use Genkit Go to implement the application logic and Gemini 3 Pro Image (also known as Nano Banana Pro) as the model to process the photos._x000D_
-_x000D_
-Previous knowledge of Go is not strictly required, but recommended.</t>
-  </si>
-  <si>
-    <t>It is doable in 1 hour, but can be done in a more relaxed pace if more time is allocated</t>
-  </si>
-  <si>
-    <t>60fps o niente: Rendering Pipeline a suon di esempi pratici!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se un'animazione scatta o una UI risponde in ritardo, non imprecare: la colpa non e' sempre del browser! Hai mai sentito parlare della rendering pipeline? Se la risposta è no, ti assicuriamo che avresti dovuto!_x000D_
-_x000D_
-Ottenere le giuste performance non è sempre gratis...impariamo quindi cosa sia la render pipeline e capiamo come quanto stupefacente ottimizzare ogni scelta alle API e alle proprieta coinvolte, sia lato CSS sia lato JavaScript._x000D_
-_x000D_
-Facciamo una scorpacciata di criteri chiari, esempi riutilizzabili e animazioni fluide su browser e webview reali...con una coppia che solo a vederla vi farà passare il reflow!_x000D_
-</t>
-  </si>
-  <si>
-    <t>Francesco Sciuti, Emiliano Pisu</t>
-  </si>
-  <si>
-    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b, 05ed4b4a-5d57-4602-bb4e-8d55efad3e0f</t>
+    <t>Inferenza locale o remota: un viaggio andata e ritorno!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Come possiamo rendere una nostra web application resiliente, in modo che si possa fare inferenza in locale con Gemini Nano o in remoto con il potente Gemini Pro e far si che il lavoro offline non sia più un problema?_x000D_
+_x000D_
+Beh, in questo workshop avremo modo di capire insieme come fare e come pensare alle strategie per una soluzione basata su modelli locali e modelli SOTA...il tutto in salsa Gemini!</t>
+  </si>
+  <si>
+    <t>1h 30m</t>
+  </si>
+  <si>
+    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b</t>
   </si>
   <si>
     <t>Il bug non era nel codice: era nel team!</t>
@@ -665,7 +665,10 @@
     <t>Claude Code Internals</t>
   </si>
   <si>
-    <t xml:space="preserve">Thanks to the Antropic source code leak we can now learn how a top AI player has built a successfull agentic platform out of a traditional LLM server. </t>
+    <t xml:space="preserve">Thanks to the Anthropic source code leak we can now learn how a top AI player has built a successful agentic platform out of a traditional LLM server._x000D_
+_x000D_
+This talk shows the fundamental features of many existing Agentic platforms but also some undocumented and unreleased features that anticipate the future._x000D_
+</t>
   </si>
   <si>
     <t>Cristian Burrini</t>
@@ -692,7 +695,10 @@
 </t>
   </si>
   <si>
-    <t>e57ecc81-7677-4f95-a6ed-fc1ed67ec883</t>
+    <t>Chiara Corrado, Veronica Domestico, Adriana Torelli, Paola Nicoli</t>
+  </si>
+  <si>
+    <t>e57ecc81-7677-4f95-a6ed-fc1ed67ec883, d2bff94e-b91d-4cc7-ac4c-1a147b7ef61a, f564a47f-2e4d-4935-8350-341bcc4c108e, d21306a5-6233-4d2f-94f7-5fb3d5630b4d</t>
   </si>
   <si>
     <t>L'essenziale è invisibile agli occhi (ma non a Python): un’introduzione alla steganografia</t>
@@ -1785,6 +1791,30 @@
     <t>https://sessionize.com/image/291e-400o400o1-fZ88yJQ1jSUdb8xqVryTQ5.jpg</t>
   </si>
   <si>
+    <t>d21306a5-6233-4d2f-94f7-5fb3d5630b4d</t>
+  </si>
+  <si>
+    <t>Paola</t>
+  </si>
+  <si>
+    <t>Nicoli</t>
+  </si>
+  <si>
+    <t>paola.ncl@gmail.com</t>
+  </si>
+  <si>
+    <t>Ingegnera biomedica | Solution Developer (Enterprise Platforms)</t>
+  </si>
+  <si>
+    <t>Ingegnera biomedica di formazione, è sviluppatrice nel settore tech, dove progetta e realizza soluzioni digitali per aziende. Porta particolare attenzione a inclusività, accessibilità e medicina di genere, integrando questi principi nello sviluppo software. È attiva anche come volontaria in progetti tecnologici a impatto sociale, contribuendo sia allo sviluppo che alla divulgazione.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/paola-nicoli-bab42437/</t>
+  </si>
+  <si>
+    <t>https://sessionize.com/image/6608-400o400o1-fQpCZYe9sknA587wZtkspH.jpg</t>
+  </si>
+  <si>
     <t>Federico</t>
   </si>
   <si>
@@ -1808,6 +1838,38 @@
   </si>
   <si>
     <t>https://sessionize.com/image/b997-400o400o1-QFQS8XG5q7icL3QukAu6kK.jpg</t>
+  </si>
+  <si>
+    <t>d2bff94e-b91d-4cc7-ac4c-1a147b7ef61a</t>
+  </si>
+  <si>
+    <t>Veronica</t>
+  </si>
+  <si>
+    <t>Domestico</t>
+  </si>
+  <si>
+    <t>veronicadomestico@gmail.com</t>
+  </si>
+  <si>
+    <t>Technical Leader @ RJC Soft</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Veronica Domestico è Software Engineer e Technical Leader, con esperienza nello sviluppo di applicazioni mobile e web in contesti complessi e ad alto impatto._x000D_
+Si occupa di analisi dei requisiti, progettazione architetturale e guida dei team di sviluppo, trasformando bisogni funzionali in soluzioni tecniche scalabili ed efficaci._x000D_
+È Ambassador di SheTech, dove promuove l’inclusione e la crescita delle donne nel mondo della tecnologia.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/veronica-domestico</t>
+  </si>
+  <si>
+    <t>https://www.rjcsoft.it/</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/veronica_domestico?igsh=enZsaW8xMnc4Mm0x</t>
+  </si>
+  <si>
+    <t>https://sessionize.com/image/6006-400o400o1-pXFGUWtYDmaJi3DTRo2tE9.jpg</t>
   </si>
   <si>
     <t>Mohamed Mortadha</t>
@@ -1918,6 +1980,9 @@
     <t>https://sessionize.com/image/09ed-400o400o1-Mtu422U1R2UjEixBL8dDea.jpg</t>
   </si>
   <si>
+    <t>e57ecc81-7677-4f95-a6ed-fc1ed67ec883</t>
+  </si>
+  <si>
     <t>Chiara</t>
   </si>
   <si>
@@ -1939,6 +2004,28 @@
   </si>
   <si>
     <t>https://sessionize.com/image/bbe0-400o400o1-GC45U3jx4Sw9b64DsYA27P.jpg</t>
+  </si>
+  <si>
+    <t>f564a47f-2e4d-4935-8350-341bcc4c108e</t>
+  </si>
+  <si>
+    <t>Adriana</t>
+  </si>
+  <si>
+    <t>Torelli</t>
+  </si>
+  <si>
+    <t>torelli.adriana@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scientific Programming Engineer, AI &amp; ML specialist. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adriana Torelli is a Scientific Programming Engineer and Software Developer and AI &amp; ML Specialist at CMCC, where she builds data-driven solutions for land monitoring and erosion risk assessment. She works with transformer models, Earth Observation and Copernicus data to turn climate complexity into actionable insight. _x000D_
+Because the future of our planet is also built one line of code at a time.</t>
+  </si>
+  <si>
+    <t>https://sessionize.com/image/1f14-400o400o1-wPfge8JtmUSmWetThpqSGf.jpg</t>
   </si>
   <si>
     <t>Daniela</t>
@@ -2609,7 +2696,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0">
-        <v>1203376</v>
+        <v>1155551</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>85</v>
@@ -2618,40 +2705,40 @@
         <v>86</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="G10" s="0" t="s">
         <v>26</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="I10" s="0" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="K10" s="0" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L10" s="0" t="s">
         <v>31</v>
       </c>
       <c r="M10" s="0" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="N10" s="5">
-        <v>46120.84242144676</v>
-      </c>
-      <c r="O10" s="0" t="s">
-        <v>33</v>
+        <v>46080.807078935184</v>
+      </c>
+      <c r="O10" s="5">
+        <v>46090.637796145835</v>
       </c>
       <c r="P10" s="0" t="s">
         <v>44</v>
@@ -2666,7 +2753,7 @@
         <v>0</v>
       </c>
       <c r="V10" s="0" t="s">
-        <v>91</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11">
@@ -2674,19 +2761,19 @@
         <v>1098869</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="E11" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="C11" s="0" t="s">
-        <v>93</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>95</v>
-      </c>
       <c r="F11" s="0" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G11" s="0" t="s">
         <v>26</v>
@@ -2695,7 +2782,7 @@
         <v>40</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="J11" s="0" t="s">
         <v>29</v>
@@ -2707,7 +2794,7 @@
         <v>33</v>
       </c>
       <c r="M11" s="0" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="N11" s="5">
         <v>46044.86471519676</v>
@@ -2728,30 +2815,30 @@
         <v>0</v>
       </c>
       <c r="V11" s="0" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0">
-        <v>1147593</v>
+        <v>1148344</v>
       </c>
       <c r="B12" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="C12" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>102</v>
-      </c>
       <c r="F12" s="0" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="H12" s="0" t="s">
         <v>40</v>
@@ -2760,25 +2847,25 @@
         <v>28</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>58</v>
+        <v>29</v>
       </c>
       <c r="K12" s="0" t="s">
         <v>30</v>
       </c>
       <c r="L12" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="M12" s="0" t="s">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="N12" s="5">
-        <v>46087.774690972219</v>
+        <v>46087.776362002311</v>
       </c>
       <c r="O12" s="5">
-        <v>46087.783132638884</v>
+        <v>46090.396714201386</v>
       </c>
       <c r="P12" s="0" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="Q12" s="5">
         <v>46130.5</v>
@@ -2790,30 +2877,30 @@
         <v>0</v>
       </c>
       <c r="V12" s="0" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0">
-        <v>1148344</v>
+        <v>1155640</v>
       </c>
       <c r="B13" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="F13" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="G13" s="0" t="s">
         <v>106</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="E13" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="G13" s="0" t="s">
-        <v>77</v>
       </c>
       <c r="H13" s="0" t="s">
         <v>40</v>
@@ -2822,25 +2909,25 @@
         <v>28</v>
       </c>
       <c r="J13" s="0" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="K13" s="0" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="L13" s="0" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="M13" s="0" t="s">
         <v>43</v>
       </c>
       <c r="N13" s="5">
-        <v>46087.776362002311</v>
+        <v>46087.774690972219</v>
       </c>
       <c r="O13" s="5">
-        <v>46090.396714201386</v>
+        <v>46090.30420543981</v>
       </c>
       <c r="P13" s="0" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="Q13" s="5">
         <v>46130.5</v>
@@ -2852,7 +2939,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="0" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14">
@@ -2860,19 +2947,19 @@
         <v>1132787</v>
       </c>
       <c r="B14" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="E14" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="C14" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>113</v>
-      </c>
-      <c r="E14" s="0" t="s">
-        <v>114</v>
-      </c>
       <c r="F14" s="0" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="G14" s="0" t="s">
         <v>26</v>
@@ -2893,7 +2980,7 @@
         <v>33</v>
       </c>
       <c r="M14" s="0" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="N14" s="5">
         <v>46056.871177777779</v>
@@ -2914,33 +3001,33 @@
         <v>0</v>
       </c>
       <c r="V14" s="0" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0">
-        <v>1148023</v>
+        <v>1147593</v>
       </c>
       <c r="B15" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="C15" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="E15" s="0" t="s">
-        <v>120</v>
-      </c>
       <c r="F15" s="0" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="I15" s="0" t="s">
         <v>28</v>
@@ -2949,101 +3036,101 @@
         <v>58</v>
       </c>
       <c r="K15" s="0" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="M15" s="0" t="s">
-        <v>43</v>
+        <v>118</v>
       </c>
       <c r="N15" s="5">
-        <v>46087.776362002311</v>
+        <v>46087.774690972219</v>
       </c>
       <c r="O15" s="5">
-        <v>46087.777946678238</v>
+        <v>46087.783132638884</v>
       </c>
       <c r="P15" s="0" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="Q15" s="5">
         <v>46130.597222222219</v>
       </c>
       <c r="R15" s="0">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="U15" s="0">
         <v>0</v>
       </c>
       <c r="V15" s="0" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0">
-        <v>1155551</v>
+        <v>1148023</v>
       </c>
       <c r="B16" s="0" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="E16" s="0" t="s">
         <v>123</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="F16" s="0" t="s">
         <v>124</v>
       </c>
-      <c r="D16" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" s="0" t="s">
-        <v>24</v>
-      </c>
       <c r="G16" s="0" t="s">
-        <v>26</v>
+        <v>77</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>125</v>
+        <v>28</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="K16" s="0" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="L16" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="M16" s="0" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="N16" s="5">
-        <v>46080.807078935184</v>
+        <v>46087.776362002311</v>
       </c>
       <c r="O16" s="5">
-        <v>46090.637796145835</v>
+        <v>46087.777946678238</v>
       </c>
       <c r="P16" s="0" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="Q16" s="5">
         <v>46130.597222222219</v>
       </c>
       <c r="R16" s="0">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="U16" s="0">
         <v>0</v>
       </c>
       <c r="V16" s="0" t="s">
-        <v>35</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0">
-        <v>1155640</v>
+        <v>1203376</v>
       </c>
       <c r="B17" s="0" t="s">
         <v>126</v>
@@ -3052,22 +3139,22 @@
         <v>127</v>
       </c>
       <c r="D17" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="H17" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="E17" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" s="0" t="s">
+      <c r="I17" s="0" t="s">
         <v>128</v>
-      </c>
-      <c r="G17" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="H17" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="I17" s="0" t="s">
-        <v>28</v>
       </c>
       <c r="J17" s="0" t="s">
         <v>41</v>
@@ -3082,19 +3169,19 @@
         <v>43</v>
       </c>
       <c r="N17" s="5">
-        <v>46087.774690972219</v>
+        <v>46120.84242144676</v>
       </c>
       <c r="O17" s="5">
-        <v>46090.30420543981</v>
+        <v>46122.386397303242</v>
       </c>
       <c r="P17" s="0" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="Q17" s="5">
         <v>46130.597222222219</v>
       </c>
       <c r="R17" s="0">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="U17" s="0">
         <v>0</v>
@@ -3575,7 +3662,7 @@
         <v>33</v>
       </c>
       <c r="M25" s="0" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="N25" s="5">
         <v>46080.807078935184</v>
@@ -3672,13 +3759,13 @@
         <v>182</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>119</v>
+        <v>183</v>
       </c>
       <c r="G27" s="0" t="s">
         <v>77</v>
@@ -3720,7 +3807,7 @@
         <v>0</v>
       </c>
       <c r="V27" s="0" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="28">
@@ -3728,19 +3815,19 @@
         <v>1105608</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E28" s="0" t="s">
+        <v>188</v>
+      </c>
+      <c r="F28" s="0" t="s">
         <v>187</v>
-      </c>
-      <c r="F28" s="0" t="s">
-        <v>186</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>141</v>
@@ -3782,7 +3869,7 @@
         <v>0</v>
       </c>
       <c r="V28" s="0" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29">
@@ -3790,19 +3877,19 @@
         <v>1145869</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E29" s="0" t="s">
+        <v>193</v>
+      </c>
+      <c r="F29" s="0" t="s">
         <v>192</v>
-      </c>
-      <c r="F29" s="0" t="s">
-        <v>191</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>26</v>
@@ -3844,7 +3931,7 @@
         <v>0</v>
       </c>
       <c r="V29" s="0" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30">
@@ -3852,19 +3939,19 @@
         <v>1124260</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E30" s="0" t="s">
+        <v>198</v>
+      </c>
+      <c r="F30" s="0" t="s">
         <v>197</v>
-      </c>
-      <c r="F30" s="0" t="s">
-        <v>196</v>
       </c>
       <c r="G30" s="0" t="s">
         <v>173</v>
@@ -3906,7 +3993,7 @@
         <v>0</v>
       </c>
       <c r="V30" s="0" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31">
@@ -3914,22 +4001,22 @@
         <v>1125184</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E31" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="F31" s="0" t="s">
         <v>202</v>
       </c>
-      <c r="F31" s="0" t="s">
-        <v>201</v>
-      </c>
       <c r="G31" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H31" s="0" t="s">
         <v>40</v>
@@ -3968,7 +4055,7 @@
         <v>0</v>
       </c>
       <c r="V31" s="0" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="32">
@@ -3976,28 +4063,28 @@
         <v>1133878</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E32" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="F32" s="0" t="s">
         <v>208</v>
-      </c>
-      <c r="F32" s="0" t="s">
-        <v>207</v>
       </c>
       <c r="G32" s="0" t="s">
         <v>26</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J32" s="0" t="s">
         <v>58</v>
@@ -4030,7 +4117,7 @@
         <v>0</v>
       </c>
       <c r="V32" s="0" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="33">
@@ -4038,19 +4125,19 @@
         <v>1147845</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E33" s="0" t="s">
+        <v>215</v>
+      </c>
+      <c r="F33" s="0" t="s">
         <v>214</v>
-      </c>
-      <c r="F33" s="0" t="s">
-        <v>213</v>
       </c>
       <c r="G33" s="0" t="s">
         <v>26</v>
@@ -4092,7 +4179,7 @@
         <v>0</v>
       </c>
       <c r="V33" s="0" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="34">
@@ -4100,19 +4187,19 @@
         <v>1148589</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G34" s="0" t="s">
         <v>173</v>
@@ -4154,7 +4241,7 @@
         <v>0</v>
       </c>
       <c r="V34" s="0" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="35">
@@ -4162,22 +4249,22 @@
         <v>1154675</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H35" s="0" t="s">
         <v>40</v>
@@ -4216,7 +4303,7 @@
         <v>0</v>
       </c>
       <c r="V35" s="0" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36">
@@ -4224,19 +4311,19 @@
         <v>1143717</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E36" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="F36" s="0" t="s">
         <v>231</v>
-      </c>
-      <c r="F36" s="0" t="s">
-        <v>230</v>
       </c>
       <c r="G36" s="0" t="s">
         <v>173</v>
@@ -4257,7 +4344,7 @@
         <v>31</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N36" s="5">
         <v>46063.895173379628</v>
@@ -4278,7 +4365,7 @@
         <v>0</v>
       </c>
       <c r="V36" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -4288,45 +4375,45 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="xr">
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2">
@@ -4334,28 +4421,28 @@
         <v>84</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>83</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3">
@@ -4363,124 +4450,124 @@
         <v>147</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>146</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="L3" s="0" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J4" s="0" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L4" s="0" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E5" s="0" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="L5" s="0" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>281</v>
+      </c>
+      <c r="D6" s="0" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>279</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>280</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>214</v>
-      </c>
       <c r="E6" s="0" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J6" s="0" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L6" s="0" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7">
@@ -4488,54 +4575,54 @@
         <v>174</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D7" s="0" t="s">
         <v>172</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L7" s="0" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F8" s="0" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L8" s="0" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="9">
@@ -4543,28 +4630,28 @@
         <v>163</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D9" s="0" t="s">
         <v>162</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L9" s="0" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10">
@@ -4572,31 +4659,31 @@
         <v>52</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>49</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J10" s="0" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="L10" s="0" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11">
@@ -4604,162 +4691,162 @@
         <v>152</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D11" s="0" t="s">
         <v>151</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F11" s="0" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="I11" s="0" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="L11" s="0" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="J12" s="0" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="K12" s="0" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="L12" s="0" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>56</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="L13" s="0" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J14" s="0" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="L14" s="0" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="I15" s="0" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="16">
@@ -4767,167 +4854,167 @@
         <v>168</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D16" s="0" t="s">
         <v>167</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J16" s="0" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K16" s="0" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="L16" s="0" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="L17" s="0" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="L18" s="0" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D19" s="0" t="s">
         <v>133</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L19" s="0" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="L20" s="0" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>401</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>402</v>
+      </c>
+      <c r="D21" s="0" t="s">
         <v>193</v>
       </c>
-      <c r="B21" s="0" t="s">
-        <v>400</v>
-      </c>
-      <c r="C21" s="0" t="s">
-        <v>401</v>
-      </c>
-      <c r="D21" s="0" t="s">
-        <v>192</v>
-      </c>
       <c r="E21" s="0" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="L21" s="0" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="22">
@@ -4935,63 +5022,63 @@
         <v>158</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D22" s="0" t="s">
         <v>156</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="I22" s="0" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="L22" s="0" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="L23" s="0" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="24">
@@ -4999,34 +5086,34 @@
         <v>45</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D24" s="0" t="s">
         <v>39</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="I24" s="0" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="L24" s="0" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="25">
@@ -5034,28 +5121,28 @@
         <v>180</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D25" s="0" t="s">
         <v>178</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="L25" s="0" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
     </row>
     <row r="26">
@@ -5063,31 +5150,31 @@
         <v>67</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D26" s="0" t="s">
         <v>64</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="I26" s="0" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="L26" s="0" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="27">
@@ -5095,214 +5182,214 @@
         <v>72</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D27" s="0" t="s">
         <v>71</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="J27" s="0" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="L27" s="0" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="L28" s="0" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="I29" s="0" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J29" s="0" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K29" s="0" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="L29" s="0" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E30" s="0" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F30" s="0" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="I30" s="0" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="K30" s="0" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="L30" s="0" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>482</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>483</v>
+      </c>
+      <c r="D31" s="0" t="s">
         <v>188</v>
       </c>
-      <c r="B31" s="0" t="s">
-        <v>481</v>
-      </c>
-      <c r="C31" s="0" t="s">
-        <v>482</v>
-      </c>
-      <c r="D31" s="0" t="s">
-        <v>187</v>
-      </c>
       <c r="E31" s="0" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F31" s="0" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="I31" s="0" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="L31" s="0" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D32" s="0" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="E32" s="0" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F32" s="0" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="I32" s="0" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="L32" s="0" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>497</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>498</v>
+      </c>
+      <c r="D33" s="0" t="s">
         <v>198</v>
       </c>
-      <c r="B33" s="0" t="s">
-        <v>496</v>
-      </c>
-      <c r="C33" s="0" t="s">
-        <v>497</v>
-      </c>
-      <c r="D33" s="0" t="s">
-        <v>197</v>
-      </c>
       <c r="E33" s="0" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F33" s="0" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="J33" s="0" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="L33" s="0" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="34">
@@ -5310,144 +5397,132 @@
         <v>79</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D34" s="0" t="s">
         <v>76</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F34" s="0" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J34" s="0" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="L34" s="0" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="D35" s="0" t="s">
         <v>139</v>
       </c>
       <c r="E35" s="0" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F35" s="0" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="H35" s="0" t="s">
+        <v>519</v>
+      </c>
+      <c r="I35" s="0" t="s">
+        <v>520</v>
+      </c>
+      <c r="J35" s="0" t="s">
         <v>518</v>
       </c>
-      <c r="I35" s="0" t="s">
-        <v>519</v>
-      </c>
-      <c r="J35" s="0" t="s">
-        <v>517</v>
-      </c>
       <c r="L35" s="0" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
-        <v>204</v>
+        <v>522</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>202</v>
+        <v>525</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="F36" s="0" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>525</v>
-      </c>
-      <c r="H36" s="0" t="s">
-        <v>526</v>
-      </c>
-      <c r="J36" s="0" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="L36" s="0" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>98</v>
+        <v>205</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>95</v>
+        <v>203</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F37" s="0" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>534</v>
-      </c>
-      <c r="I37" s="0" t="s">
         <v>535</v>
       </c>
       <c r="J37" s="0" t="s">
         <v>536</v>
       </c>
-      <c r="K37" s="0" t="s">
+      <c r="L37" s="0" t="s">
         <v>537</v>
-      </c>
-      <c r="L37" s="0" t="s">
-        <v>538</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
-        <v>105</v>
+        <v>538</v>
       </c>
       <c r="B38" s="0" t="s">
         <v>539</v>
@@ -5456,150 +5531,243 @@
         <v>540</v>
       </c>
       <c r="D38" s="0" t="s">
-        <v>102</v>
+        <v>541</v>
       </c>
       <c r="E38" s="0" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F38" s="0" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="I38" s="0" t="s">
-        <v>545</v>
-      </c>
-      <c r="J38" s="0" t="s">
         <v>546</v>
       </c>
-      <c r="K38" s="0" t="s">
+      <c r="L38" s="0" t="s">
         <v>547</v>
-      </c>
-      <c r="L38" s="0" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>548</v>
+      </c>
+      <c r="C39" s="0" t="s">
         <v>549</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="D39" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="E39" s="0" t="s">
         <v>550</v>
       </c>
-      <c r="C39" s="0" t="s">
+      <c r="F39" s="0" t="s">
         <v>551</v>
       </c>
-      <c r="D39" s="0" t="s">
+      <c r="G39" s="0" t="s">
         <v>552</v>
       </c>
-      <c r="E39" s="0" t="s">
+      <c r="H39" s="0" t="s">
         <v>553</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="I39" s="0" t="s">
         <v>554</v>
       </c>
-      <c r="G39" s="0" t="s">
+      <c r="J39" s="0" t="s">
         <v>555</v>
       </c>
+      <c r="K39" s="0" t="s">
+        <v>556</v>
+      </c>
       <c r="L39" s="0" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="s">
-        <v>210</v>
+        <v>119</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>423</v>
+        <v>558</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>208</v>
+        <v>117</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="F40" s="0" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>561</v>
+        <v>563</v>
+      </c>
+      <c r="I40" s="0" t="s">
+        <v>564</v>
       </c>
       <c r="J40" s="0" t="s">
-        <v>562</v>
+        <v>565</v>
+      </c>
+      <c r="K40" s="0" t="s">
+        <v>566</v>
       </c>
       <c r="L40" s="0" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>183</v>
+        <v>568</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>564</v>
+        <v>569</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>120</v>
+        <v>571</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="F41" s="0" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>568</v>
-      </c>
-      <c r="J41" s="0" t="s">
-        <v>569</v>
+        <v>574</v>
       </c>
       <c r="L41" s="0" t="s">
-        <v>570</v>
+        <v>575</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>424</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>576</v>
+      </c>
+      <c r="D42" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E42" s="0" t="s">
+        <v>577</v>
+      </c>
+      <c r="F42" s="0" t="s">
+        <v>578</v>
+      </c>
+      <c r="G42" s="0" t="s">
+        <v>579</v>
+      </c>
+      <c r="H42" s="0" t="s">
+        <v>580</v>
+      </c>
+      <c r="J42" s="0" t="s">
+        <v>581</v>
+      </c>
+      <c r="L42" s="0" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="s">
+        <v>583</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>584</v>
+      </c>
+      <c r="C43" s="0" t="s">
+        <v>585</v>
+      </c>
+      <c r="D43" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="E43" s="0" t="s">
+        <v>586</v>
+      </c>
+      <c r="F43" s="0" t="s">
+        <v>587</v>
+      </c>
+      <c r="G43" s="0" t="s">
+        <v>588</v>
+      </c>
+      <c r="J43" s="0" t="s">
+        <v>589</v>
+      </c>
+      <c r="L43" s="0" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="s">
+        <v>591</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>592</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>593</v>
+      </c>
+      <c r="D44" s="0" t="s">
+        <v>594</v>
+      </c>
+      <c r="E44" s="0" t="s">
+        <v>595</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>596</v>
+      </c>
+      <c r="L44" s="0" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="B42" s="0" t="s">
-        <v>571</v>
-      </c>
-      <c r="C42" s="0" t="s">
-        <v>572</v>
-      </c>
-      <c r="D42" s="0" t="s">
+      <c r="B45" s="0" t="s">
+        <v>598</v>
+      </c>
+      <c r="C45" s="0" t="s">
+        <v>599</v>
+      </c>
+      <c r="D45" s="0" t="s">
         <v>25</v>
       </c>
-      <c r="E42" s="0" t="s">
-        <v>573</v>
-      </c>
-      <c r="F42" s="0" t="s">
-        <v>574</v>
-      </c>
-      <c r="G42" s="0" t="s">
-        <v>575</v>
-      </c>
-      <c r="H42" s="0" t="s">
-        <v>576</v>
-      </c>
-      <c r="J42" s="0" t="s">
-        <v>577</v>
-      </c>
-      <c r="L42" s="0" t="s">
-        <v>578</v>
+      <c r="E45" s="0" t="s">
+        <v>600</v>
+      </c>
+      <c r="F45" s="0" t="s">
+        <v>601</v>
+      </c>
+      <c r="G45" s="0" t="s">
+        <v>602</v>
+      </c>
+      <c r="H45" s="0" t="s">
+        <v>603</v>
+      </c>
+      <c r="J45" s="0" t="s">
+        <v>604</v>
+      </c>
+      <c r="L45" s="0" t="s">
+        <v>605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update session language to Italian and ensure Instagram links are consistent
</commit_message>
<xml_diff>
--- a/src/assets/sessionize/data-advanced.xlsx
+++ b/src/assets/sessionize/data-advanced.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="621">
   <si>
     <t>Session Id</t>
   </si>
@@ -644,9 +644,6 @@
     <t>jack.lilhammers@gmail.com</t>
   </si>
   <si>
-    <t>English, Italian</t>
-  </si>
-  <si>
     <t>82b493da-0b26-4e1f-9c81-54c9609a4b50</t>
   </si>
   <si>
@@ -929,12 +926,12 @@
     <t>Company Website</t>
   </si>
   <si>
+    <t>Blog</t>
+  </si>
+  <si>
     <t>Instagram</t>
   </si>
   <si>
-    <t>Blog</t>
-  </si>
-  <si>
     <t>Facebook</t>
   </si>
   <si>
@@ -1006,10 +1003,10 @@
     <t>https://devdojo.it</t>
   </si>
   <si>
+    <t>https://dout.dev</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/pixu1980/</t>
-  </si>
-  <si>
-    <t>https://dout.dev</t>
   </si>
   <si>
     <t>https://sessionize.com/image/fd3b-400o400o1-BwkHXp3qRbEw3D5V2gPbAY.png</t>
@@ -1209,10 +1206,10 @@
     <t>https://fractal.cloud</t>
   </si>
   <si>
+    <t>https://michelmurabito.com</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/michel_murabito/</t>
-  </si>
-  <si>
-    <t>https://michelmurabito.com</t>
   </si>
   <si>
     <t>https://www.facebook.com/michelmurabito</t>
@@ -1298,10 +1295,10 @@
     <t>https://bit.ly/pantarei-mb</t>
   </si>
   <si>
+    <t>https://sites.google.com/view/pantarei-mb-en/blog</t>
+  </si>
+  <si>
     <t>https://instagram.com/pantarei_mb</t>
-  </si>
-  <si>
-    <t>https://sites.google.com/view/pantarei-mb-en/blog</t>
   </si>
   <si>
     <t>https://sessionize.com/image/677e-400o400o1-shpurTgXp4EfDBWu3fPXrZ.jpg</t>
@@ -1521,10 +1518,10 @@
     <t>https://pescara.python.it/</t>
   </si>
   <si>
+    <t>https://www.lucadivita.it/</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/luca_di_vita_</t>
-  </si>
-  <si>
-    <t>https://www.lucadivita.it/</t>
   </si>
   <si>
     <t>https://sessionize.com/image/77c6-400o400o1-hMWZzLKMh7xt3XWNZALNnt.jpg</t>
@@ -1643,10 +1640,10 @@
     <t>https://devmy.it</t>
   </si>
   <si>
+    <t>https://devmy.it/blog</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/Devmy.it/</t>
-  </si>
-  <si>
-    <t>https://devmy.it/blog</t>
   </si>
   <si>
     <t>https://www.facebook.com/francesco.sciuti/</t>
@@ -1776,10 +1773,10 @@
     <t>https://monjadariva.it</t>
   </si>
   <si>
+    <t>https://monjadariva.it/blog</t>
+  </si>
+  <si>
     <t>https://instagram.com/monja.dariva</t>
-  </si>
-  <si>
-    <t>https://monjadariva.it/blog</t>
   </si>
   <si>
     <t>https://sessionize.com/image/3e16-400o400o1-7jvdkF5R8VCzcbkb33Ty6R.jpg</t>
@@ -1918,12 +1915,12 @@
     <t>https://learnbydo.ing/</t>
   </si>
   <si>
+    <t>http://fabiobiondi.dev/</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/biondifabio/</t>
   </si>
   <si>
-    <t>http://fabiobiondi.dev/</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/groups/fabiobiondi.training</t>
   </si>
   <si>
@@ -1948,12 +1945,12 @@
     <t>https://www.mann-ai.com/</t>
   </si>
   <si>
+    <t>https://manaimortadha.medium.com/</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/mortadha_mannai/</t>
   </si>
   <si>
-    <t>https://manaimortadha.medium.com/</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/profile.php?id=100004306062352</t>
   </si>
   <si>
@@ -1978,10 +1975,10 @@
     <t>https://www.thinktecture.com</t>
   </si>
   <si>
+    <t>https://christianliebel.com</t>
+  </si>
+  <si>
     <t>https://www.instagram.com/chliebel/</t>
-  </si>
-  <si>
-    <t>https://christianliebel.com</t>
   </si>
   <si>
     <t>https://www.facebook.com/christianliebel</t>
@@ -3640,7 +3637,7 @@
         <v>79</v>
       </c>
       <c r="K24" s="0" t="s">
-        <v>170</v>
+        <v>42</v>
       </c>
       <c r="L24" s="0" t="s">
         <v>31</v>
@@ -3667,7 +3664,7 @@
         <v>0</v>
       </c>
       <c r="V24" s="0" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25">
@@ -3675,19 +3672,19 @@
         <v>1149383</v>
       </c>
       <c r="B25" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="C25" s="0" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="D25" s="0" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="E25" s="0" t="s">
         <v>174</v>
       </c>
-      <c r="E25" s="0" t="s">
-        <v>175</v>
-      </c>
       <c r="F25" s="0" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G25" s="0" t="s">
         <v>38</v>
@@ -3729,7 +3726,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="26">
@@ -3737,19 +3734,19 @@
         <v>1151362</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>177</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="D26" s="0" t="s">
         <v>178</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="E26" s="0" t="s">
         <v>179</v>
       </c>
-      <c r="E26" s="0" t="s">
-        <v>180</v>
-      </c>
       <c r="F26" s="0" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G26" s="0" t="s">
         <v>38</v>
@@ -3791,7 +3788,7 @@
         <v>0</v>
       </c>
       <c r="V26" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="27">
@@ -3799,19 +3796,19 @@
         <v>1155630</v>
       </c>
       <c r="B27" s="0" t="s">
+        <v>181</v>
+      </c>
+      <c r="C27" s="0" t="s">
         <v>182</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="D27" s="0" t="s">
         <v>183</v>
       </c>
-      <c r="D27" s="0" t="s">
+      <c r="E27" s="0" t="s">
         <v>184</v>
       </c>
-      <c r="E27" s="0" t="s">
-        <v>185</v>
-      </c>
       <c r="F27" s="0" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G27" s="0" t="s">
         <v>71</v>
@@ -3853,7 +3850,7 @@
         <v>0</v>
       </c>
       <c r="V27" s="0" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28">
@@ -3861,19 +3858,19 @@
         <v>1200474</v>
       </c>
       <c r="B28" s="0" t="s">
+        <v>186</v>
+      </c>
+      <c r="C28" s="0" t="s">
         <v>187</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="D28" s="0" t="s">
         <v>188</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="E28" s="0" t="s">
         <v>189</v>
       </c>
-      <c r="E28" s="0" t="s">
-        <v>190</v>
-      </c>
       <c r="F28" s="0" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>38</v>
@@ -3891,7 +3888,7 @@
         <v>42</v>
       </c>
       <c r="L28" s="0" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="M28" s="0" t="s">
         <v>32</v>
@@ -3915,7 +3912,7 @@
         <v>0</v>
       </c>
       <c r="V28" s="0" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29">
@@ -3923,10 +3920,10 @@
         <v>1203288</v>
       </c>
       <c r="B29" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="C29" s="0" t="s">
         <v>193</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>194</v>
       </c>
       <c r="D29" s="0" t="s">
         <v>133</v>
@@ -3935,7 +3932,7 @@
         <v>134</v>
       </c>
       <c r="F29" s="0" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G29" s="0" t="s">
         <v>26</v>
@@ -3977,7 +3974,7 @@
         <v>0</v>
       </c>
       <c r="V29" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30">
@@ -3985,19 +3982,19 @@
         <v>1105608</v>
       </c>
       <c r="B30" s="0" t="s">
+        <v>196</v>
+      </c>
+      <c r="C30" s="0" t="s">
         <v>197</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="D30" s="0" t="s">
         <v>198</v>
       </c>
-      <c r="D30" s="0" t="s">
+      <c r="E30" s="0" t="s">
         <v>199</v>
       </c>
-      <c r="E30" s="0" t="s">
-        <v>200</v>
-      </c>
       <c r="F30" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G30" s="0" t="s">
         <v>154</v>
@@ -4039,7 +4036,7 @@
         <v>0</v>
       </c>
       <c r="V30" s="0" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31">
@@ -4047,19 +4044,19 @@
         <v>1145869</v>
       </c>
       <c r="B31" s="0" t="s">
+        <v>201</v>
+      </c>
+      <c r="C31" s="0" t="s">
         <v>202</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="D31" s="0" t="s">
         <v>203</v>
       </c>
-      <c r="D31" s="0" t="s">
+      <c r="E31" s="0" t="s">
         <v>204</v>
       </c>
-      <c r="E31" s="0" t="s">
-        <v>205</v>
-      </c>
       <c r="F31" s="0" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G31" s="0" t="s">
         <v>38</v>
@@ -4101,7 +4098,7 @@
         <v>0</v>
       </c>
       <c r="V31" s="0" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="32">
@@ -4109,19 +4106,19 @@
         <v>1124260</v>
       </c>
       <c r="B32" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="C32" s="0" t="s">
         <v>207</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="D32" s="0" t="s">
         <v>208</v>
       </c>
-      <c r="D32" s="0" t="s">
+      <c r="E32" s="0" t="s">
         <v>209</v>
       </c>
-      <c r="E32" s="0" t="s">
-        <v>210</v>
-      </c>
       <c r="F32" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G32" s="0" t="s">
         <v>71</v>
@@ -4163,7 +4160,7 @@
         <v>0</v>
       </c>
       <c r="V32" s="0" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33">
@@ -4171,22 +4168,22 @@
         <v>1125184</v>
       </c>
       <c r="B33" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="C33" s="0" t="s">
         <v>212</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="D33" s="0" t="s">
         <v>213</v>
       </c>
-      <c r="D33" s="0" t="s">
+      <c r="E33" s="0" t="s">
         <v>214</v>
       </c>
-      <c r="E33" s="0" t="s">
+      <c r="F33" s="0" t="s">
+        <v>213</v>
+      </c>
+      <c r="G33" s="0" t="s">
         <v>215</v>
-      </c>
-      <c r="F33" s="0" t="s">
-        <v>214</v>
-      </c>
-      <c r="G33" s="0" t="s">
-        <v>216</v>
       </c>
       <c r="H33" s="0" t="s">
         <v>27</v>
@@ -4225,7 +4222,7 @@
         <v>0</v>
       </c>
       <c r="V33" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="34">
@@ -4233,19 +4230,19 @@
         <v>1133878</v>
       </c>
       <c r="B34" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="C34" s="0" t="s">
         <v>218</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="D34" s="0" t="s">
         <v>219</v>
       </c>
-      <c r="D34" s="0" t="s">
+      <c r="E34" s="0" t="s">
         <v>220</v>
       </c>
-      <c r="E34" s="0" t="s">
-        <v>221</v>
-      </c>
       <c r="F34" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G34" s="0" t="s">
         <v>38</v>
@@ -4254,7 +4251,7 @@
         <v>39</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="J34" s="0" t="s">
         <v>79</v>
@@ -4287,7 +4284,7 @@
         <v>0</v>
       </c>
       <c r="V34" s="0" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="35">
@@ -4295,19 +4292,19 @@
         <v>1147845</v>
       </c>
       <c r="B35" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="C35" s="0" t="s">
         <v>224</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="D35" s="0" t="s">
         <v>225</v>
       </c>
-      <c r="D35" s="0" t="s">
+      <c r="E35" s="0" t="s">
         <v>226</v>
       </c>
-      <c r="E35" s="0" t="s">
-        <v>227</v>
-      </c>
       <c r="F35" s="0" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G35" s="0" t="s">
         <v>38</v>
@@ -4349,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="V35" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="36">
@@ -4357,19 +4354,19 @@
         <v>1143717</v>
       </c>
       <c r="B36" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="C36" s="0" t="s">
         <v>229</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="D36" s="0" t="s">
         <v>230</v>
       </c>
-      <c r="D36" s="0" t="s">
+      <c r="E36" s="0" t="s">
         <v>231</v>
       </c>
-      <c r="E36" s="0" t="s">
-        <v>232</v>
-      </c>
       <c r="F36" s="0" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G36" s="0" t="s">
         <v>71</v>
@@ -4390,7 +4387,7 @@
         <v>43</v>
       </c>
       <c r="M36" s="0" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="N36" s="5">
         <v>46063.895173379628</v>
@@ -4411,7 +4408,7 @@
         <v>0</v>
       </c>
       <c r="V36" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="37">
@@ -4419,22 +4416,22 @@
         <v>1154675</v>
       </c>
       <c r="B37" s="0" t="s">
+        <v>234</v>
+      </c>
+      <c r="C37" s="0" t="s">
         <v>235</v>
       </c>
-      <c r="C37" s="0" t="s">
+      <c r="D37" s="0" t="s">
         <v>236</v>
       </c>
-      <c r="D37" s="0" t="s">
+      <c r="E37" s="0" t="s">
         <v>237</v>
       </c>
-      <c r="E37" s="0" t="s">
+      <c r="F37" s="0" t="s">
         <v>238</v>
       </c>
-      <c r="F37" s="0" t="s">
-        <v>239</v>
-      </c>
       <c r="G37" s="0" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H37" s="0" t="s">
         <v>27</v>
@@ -4473,7 +4470,7 @@
         <v>0</v>
       </c>
       <c r="V37" s="0" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -4488,40 +4485,40 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="2">
@@ -4529,28 +4526,28 @@
         <v>103</v>
       </c>
       <c r="B2" s="0" t="s">
+        <v>252</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>253</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>254</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>102</v>
       </c>
       <c r="E2" s="0" t="s">
+        <v>254</v>
+      </c>
+      <c r="F2" s="0" t="s">
         <v>255</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G2" s="0" t="s">
         <v>256</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H2" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="L2" s="0" t="s">
         <v>257</v>
-      </c>
-      <c r="H2" s="0" t="s">
-        <v>257</v>
-      </c>
-      <c r="L2" s="0" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="3">
@@ -4558,208 +4555,208 @@
         <v>160</v>
       </c>
       <c r="B3" s="0" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>259</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>260</v>
       </c>
       <c r="D3" s="0" t="s">
         <v>159</v>
       </c>
       <c r="E3" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="F3" s="0" t="s">
         <v>261</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="G3" s="0" t="s">
         <v>262</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="H3" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="L3" s="0" t="s">
         <v>264</v>
-      </c>
-      <c r="L3" s="0" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
+        <v>265</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>266</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="C4" s="0" t="s">
         <v>267</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="D4" s="0" t="s">
         <v>268</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="E4" s="0" t="s">
         <v>269</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="F4" s="0" t="s">
         <v>270</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="G4" s="0" t="s">
         <v>271</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="H4" s="0" t="s">
         <v>272</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="I4" s="0" t="s">
         <v>273</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="J4" s="0" t="s">
         <v>274</v>
       </c>
-      <c r="J4" s="0" t="s">
+      <c r="L4" s="0" t="s">
         <v>275</v>
-      </c>
-      <c r="L4" s="0" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
+        <v>276</v>
+      </c>
+      <c r="B5" s="0" t="s">
         <v>277</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="C5" s="0" t="s">
         <v>278</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>279</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="E5" s="0" t="s">
         <v>280</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="F5" s="0" t="s">
         <v>281</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="G5" s="0" t="s">
         <v>282</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="H5" s="0" t="s">
         <v>283</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="L5" s="0" t="s">
         <v>284</v>
-      </c>
-      <c r="L5" s="0" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B6" s="0" t="s">
+        <v>285</v>
+      </c>
+      <c r="C6" s="0" t="s">
         <v>286</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="D6" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="E6" s="0" t="s">
         <v>287</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>227</v>
-      </c>
-      <c r="E6" s="0" t="s">
+      <c r="F6" s="0" t="s">
         <v>288</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="G6" s="0" t="s">
         <v>289</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="H6" s="0" t="s">
         <v>290</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="I6" s="0" t="s">
         <v>291</v>
       </c>
-      <c r="J6" s="0" t="s">
+      <c r="L6" s="0" t="s">
         <v>292</v>
-      </c>
-      <c r="L6" s="0" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>293</v>
+      </c>
+      <c r="C7" s="0" t="s">
         <v>294</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="D7" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="E7" s="0" t="s">
         <v>295</v>
       </c>
-      <c r="D7" s="0" t="s">
-        <v>185</v>
-      </c>
-      <c r="E7" s="0" t="s">
+      <c r="F7" s="0" t="s">
         <v>296</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="G7" s="0" t="s">
         <v>297</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="L7" s="0" t="s">
         <v>298</v>
-      </c>
-      <c r="L7" s="0" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
+        <v>299</v>
+      </c>
+      <c r="B8" s="0" t="s">
         <v>300</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="C8" s="0" t="s">
         <v>301</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="D8" s="0" t="s">
         <v>302</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="E8" s="0" t="s">
         <v>303</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="F8" s="0" t="s">
         <v>304</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="G8" s="0" t="s">
         <v>305</v>
       </c>
-      <c r="G8" s="0" t="s">
+      <c r="H8" s="0" t="s">
         <v>306</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="L8" s="0" t="s">
         <v>307</v>
-      </c>
-      <c r="L8" s="0" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>308</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="D9" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="E9" s="0" t="s">
         <v>310</v>
       </c>
-      <c r="D9" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="E9" s="0" t="s">
+      <c r="F9" s="0" t="s">
         <v>311</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="G9" s="0" t="s">
         <v>312</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="H9" s="0" t="s">
         <v>313</v>
       </c>
-      <c r="H9" s="0" t="s">
+      <c r="L9" s="0" t="s">
         <v>314</v>
-      </c>
-      <c r="L9" s="0" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="10">
@@ -4767,31 +4764,31 @@
         <v>65</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>315</v>
+      </c>
+      <c r="C10" s="0" t="s">
         <v>316</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>317</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>62</v>
       </c>
       <c r="E10" s="0" t="s">
+        <v>317</v>
+      </c>
+      <c r="F10" s="0" t="s">
         <v>318</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="G10" s="0" t="s">
         <v>319</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="H10" s="0" t="s">
         <v>320</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="I10" s="0" t="s">
         <v>321</v>
       </c>
-      <c r="J10" s="0" t="s">
+      <c r="L10" s="0" t="s">
         <v>322</v>
-      </c>
-      <c r="L10" s="0" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="11">
@@ -4799,127 +4796,127 @@
         <v>165</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>323</v>
+      </c>
+      <c r="C11" s="0" t="s">
         <v>324</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>325</v>
       </c>
       <c r="D11" s="0" t="s">
         <v>164</v>
       </c>
       <c r="E11" s="0" t="s">
+        <v>325</v>
+      </c>
+      <c r="F11" s="0" t="s">
         <v>326</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="G11" s="0" t="s">
         <v>327</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="J11" s="0" t="s">
         <v>328</v>
       </c>
-      <c r="I11" s="0" t="s">
+      <c r="L11" s="0" t="s">
         <v>329</v>
-      </c>
-      <c r="L11" s="0" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
+        <v>330</v>
+      </c>
+      <c r="B12" s="0" t="s">
         <v>331</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="C12" s="0" t="s">
         <v>332</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="D12" s="0" t="s">
+        <v>237</v>
+      </c>
+      <c r="E12" s="0" t="s">
         <v>333</v>
       </c>
-      <c r="D12" s="0" t="s">
-        <v>238</v>
-      </c>
-      <c r="E12" s="0" t="s">
+      <c r="F12" s="0" t="s">
         <v>334</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="G12" s="0" t="s">
         <v>335</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="H12" s="0" t="s">
         <v>336</v>
       </c>
-      <c r="H12" s="0" t="s">
+      <c r="I12" s="0" t="s">
         <v>337</v>
       </c>
-      <c r="I12" s="0" t="s">
+      <c r="J12" s="0" t="s">
         <v>338</v>
       </c>
-      <c r="J12" s="0" t="s">
+      <c r="K12" s="0" t="s">
         <v>339</v>
       </c>
-      <c r="K12" s="0" t="s">
+      <c r="L12" s="0" t="s">
         <v>340</v>
-      </c>
-      <c r="L12" s="0" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
+        <v>341</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>342</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="C13" s="0" t="s">
         <v>343</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>344</v>
       </c>
       <c r="D13" s="0" t="s">
         <v>77</v>
       </c>
       <c r="E13" s="0" t="s">
+        <v>344</v>
+      </c>
+      <c r="F13" s="0" t="s">
         <v>345</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="G13" s="0" t="s">
         <v>346</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="H13" s="0" t="s">
         <v>347</v>
       </c>
-      <c r="H13" s="0" t="s">
+      <c r="L13" s="0" t="s">
         <v>348</v>
-      </c>
-      <c r="L13" s="0" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
+        <v>349</v>
+      </c>
+      <c r="B14" s="0" t="s">
         <v>350</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="C14" s="0" t="s">
         <v>351</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="D14" s="0" t="s">
         <v>352</v>
       </c>
-      <c r="D14" s="0" t="s">
+      <c r="E14" s="0" t="s">
         <v>353</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="F14" s="0" t="s">
         <v>354</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="G14" s="0" t="s">
         <v>355</v>
       </c>
-      <c r="G14" s="0" t="s">
+      <c r="H14" s="0" t="s">
         <v>356</v>
       </c>
-      <c r="H14" s="0" t="s">
+      <c r="I14" s="0" t="s">
         <v>357</v>
       </c>
-      <c r="J14" s="0" t="s">
+      <c r="L14" s="0" t="s">
         <v>358</v>
-      </c>
-      <c r="L14" s="0" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="15">
@@ -4927,266 +4924,266 @@
         <v>124</v>
       </c>
       <c r="B15" s="0" t="s">
+        <v>359</v>
+      </c>
+      <c r="C15" s="0" t="s">
         <v>360</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>361</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>122</v>
       </c>
       <c r="E15" s="0" t="s">
+        <v>361</v>
+      </c>
+      <c r="F15" s="0" t="s">
         <v>362</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="G15" s="0" t="s">
         <v>363</v>
       </c>
-      <c r="G15" s="0" t="s">
+      <c r="H15" s="0" t="s">
         <v>364</v>
       </c>
-      <c r="H15" s="0" t="s">
+      <c r="I15" s="0" t="s">
         <v>365</v>
       </c>
-      <c r="I15" s="0" t="s">
+      <c r="J15" s="0" t="s">
         <v>366</v>
       </c>
-      <c r="J15" s="0" t="s">
+      <c r="L15" s="0" t="s">
         <v>367</v>
-      </c>
-      <c r="L15" s="0" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B16" s="0" t="s">
+        <v>368</v>
+      </c>
+      <c r="C16" s="0" t="s">
         <v>369</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="D16" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" s="0" t="s">
         <v>370</v>
       </c>
-      <c r="D16" s="0" t="s">
-        <v>180</v>
-      </c>
-      <c r="E16" s="0" t="s">
+      <c r="F16" s="0" t="s">
         <v>371</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="G16" s="0" t="s">
         <v>372</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="H16" s="0" t="s">
         <v>373</v>
       </c>
-      <c r="H16" s="0" t="s">
+      <c r="I16" s="0" t="s">
         <v>374</v>
       </c>
-      <c r="J16" s="0" t="s">
+      <c r="K16" s="0" t="s">
         <v>375</v>
       </c>
-      <c r="K16" s="0" t="s">
+      <c r="L16" s="0" t="s">
         <v>376</v>
-      </c>
-      <c r="L16" s="0" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="B17" s="0" t="s">
         <v>378</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="C17" s="0" t="s">
         <v>379</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="D17" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="E17" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="F17" s="0" t="s">
         <v>382</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="G17" s="0" t="s">
         <v>383</v>
       </c>
-      <c r="G17" s="0" t="s">
+      <c r="L17" s="0" t="s">
         <v>384</v>
-      </c>
-      <c r="L17" s="0" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
+        <v>385</v>
+      </c>
+      <c r="B18" s="0" t="s">
         <v>386</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="C18" s="0" t="s">
         <v>387</v>
-      </c>
-      <c r="C18" s="0" t="s">
-        <v>388</v>
       </c>
       <c r="D18" s="0" t="s">
         <v>69</v>
       </c>
       <c r="E18" s="0" t="s">
+        <v>388</v>
+      </c>
+      <c r="F18" s="0" t="s">
         <v>389</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="G18" s="0" t="s">
         <v>390</v>
       </c>
-      <c r="G18" s="0" t="s">
+      <c r="H18" s="0" t="s">
         <v>391</v>
       </c>
-      <c r="H18" s="0" t="s">
+      <c r="L18" s="0" t="s">
         <v>392</v>
-      </c>
-      <c r="L18" s="0" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
+        <v>393</v>
+      </c>
+      <c r="B19" s="0" t="s">
         <v>394</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="C19" s="0" t="s">
         <v>395</v>
-      </c>
-      <c r="C19" s="0" t="s">
-        <v>396</v>
       </c>
       <c r="D19" s="0" t="s">
         <v>146</v>
       </c>
       <c r="E19" s="0" t="s">
+        <v>396</v>
+      </c>
+      <c r="F19" s="0" t="s">
         <v>397</v>
       </c>
-      <c r="F19" s="0" t="s">
+      <c r="H19" s="0" t="s">
+        <v>306</v>
+      </c>
+      <c r="L19" s="0" t="s">
         <v>398</v>
-      </c>
-      <c r="H19" s="0" t="s">
-        <v>307</v>
-      </c>
-      <c r="L19" s="0" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
+        <v>399</v>
+      </c>
+      <c r="B20" s="0" t="s">
         <v>400</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="C20" s="0" t="s">
         <v>401</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="D20" s="0" t="s">
         <v>402</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="E20" s="0" t="s">
         <v>403</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="F20" s="0" t="s">
         <v>404</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="L20" s="0" t="s">
         <v>405</v>
-      </c>
-      <c r="L20" s="0" t="s">
-        <v>406</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B21" s="0" t="s">
+        <v>406</v>
+      </c>
+      <c r="C21" s="0" t="s">
         <v>407</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="D21" s="0" t="s">
+        <v>204</v>
+      </c>
+      <c r="E21" s="0" t="s">
         <v>408</v>
       </c>
-      <c r="D21" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="E21" s="0" t="s">
+      <c r="F21" s="0" t="s">
         <v>409</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="G21" s="0" t="s">
         <v>410</v>
       </c>
-      <c r="G21" s="0" t="s">
+      <c r="H21" s="0" t="s">
         <v>411</v>
       </c>
-      <c r="H21" s="0" t="s">
+      <c r="L21" s="0" t="s">
         <v>412</v>
-      </c>
-      <c r="L21" s="0" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B22" s="0" t="s">
+        <v>413</v>
+      </c>
+      <c r="C22" s="0" t="s">
         <v>414</v>
-      </c>
-      <c r="C22" s="0" t="s">
-        <v>415</v>
       </c>
       <c r="D22" s="0" t="s">
         <v>169</v>
       </c>
       <c r="E22" s="0" t="s">
+        <v>415</v>
+      </c>
+      <c r="F22" s="0" t="s">
         <v>416</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="G22" s="0" t="s">
         <v>417</v>
       </c>
-      <c r="G22" s="0" t="s">
+      <c r="H22" s="0" t="s">
         <v>418</v>
       </c>
-      <c r="H22" s="0" t="s">
+      <c r="J22" s="0" t="s">
         <v>419</v>
       </c>
-      <c r="I22" s="0" t="s">
+      <c r="L22" s="0" t="s">
         <v>420</v>
-      </c>
-      <c r="L22" s="0" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>421</v>
+      </c>
+      <c r="C23" s="0" t="s">
         <v>422</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="D23" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="E23" s="0" t="s">
         <v>423</v>
       </c>
-      <c r="D23" s="0" t="s">
-        <v>232</v>
-      </c>
-      <c r="E23" s="0" t="s">
+      <c r="F23" s="0" t="s">
         <v>424</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="G23" s="0" t="s">
         <v>425</v>
       </c>
-      <c r="G23" s="0" t="s">
+      <c r="H23" s="0" t="s">
         <v>426</v>
       </c>
-      <c r="H23" s="0" t="s">
+      <c r="I23" s="0" t="s">
         <v>427</v>
       </c>
-      <c r="J23" s="0" t="s">
+      <c r="L23" s="0" t="s">
         <v>428</v>
-      </c>
-      <c r="L23" s="0" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="24">
@@ -5194,63 +5191,63 @@
         <v>58</v>
       </c>
       <c r="B24" s="0" t="s">
+        <v>429</v>
+      </c>
+      <c r="C24" s="0" t="s">
         <v>430</v>
-      </c>
-      <c r="C24" s="0" t="s">
-        <v>431</v>
       </c>
       <c r="D24" s="0" t="s">
         <v>56</v>
       </c>
       <c r="E24" s="0" t="s">
+        <v>431</v>
+      </c>
+      <c r="F24" s="0" t="s">
         <v>432</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="G24" s="0" t="s">
         <v>433</v>
       </c>
-      <c r="G24" s="0" t="s">
+      <c r="H24" s="0" t="s">
         <v>434</v>
       </c>
-      <c r="H24" s="0" t="s">
+      <c r="I24" s="0" t="s">
         <v>435</v>
       </c>
-      <c r="I24" s="0" t="s">
+      <c r="J24" s="0" t="s">
         <v>436</v>
       </c>
-      <c r="J24" s="0" t="s">
+      <c r="L24" s="0" t="s">
         <v>437</v>
-      </c>
-      <c r="L24" s="0" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B25" s="0" t="s">
+        <v>438</v>
+      </c>
+      <c r="C25" s="0" t="s">
         <v>439</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="D25" s="0" t="s">
+        <v>189</v>
+      </c>
+      <c r="E25" s="0" t="s">
         <v>440</v>
       </c>
-      <c r="D25" s="0" t="s">
-        <v>190</v>
-      </c>
-      <c r="E25" s="0" t="s">
+      <c r="F25" s="0" t="s">
         <v>441</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="G25" s="0" t="s">
         <v>442</v>
       </c>
-      <c r="G25" s="0" t="s">
+      <c r="H25" s="0" t="s">
         <v>443</v>
       </c>
-      <c r="H25" s="0" t="s">
+      <c r="L25" s="0" t="s">
         <v>444</v>
-      </c>
-      <c r="L25" s="0" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="26">
@@ -5258,31 +5255,31 @@
         <v>87</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>445</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>446</v>
-      </c>
-      <c r="C26" s="0" t="s">
-        <v>447</v>
       </c>
       <c r="D26" s="0" t="s">
         <v>85</v>
       </c>
       <c r="E26" s="0" t="s">
+        <v>447</v>
+      </c>
+      <c r="F26" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="F26" s="0" t="s">
+      <c r="G26" s="0" t="s">
         <v>449</v>
       </c>
-      <c r="G26" s="0" t="s">
+      <c r="H26" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="H26" s="0" t="s">
+      <c r="J26" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="I26" s="0" t="s">
+      <c r="L26" s="0" t="s">
         <v>452</v>
-      </c>
-      <c r="L26" s="0" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="27">
@@ -5290,51 +5287,51 @@
         <v>92</v>
       </c>
       <c r="B27" s="0" t="s">
+        <v>453</v>
+      </c>
+      <c r="C27" s="0" t="s">
         <v>454</v>
-      </c>
-      <c r="C27" s="0" t="s">
-        <v>455</v>
       </c>
       <c r="D27" s="0" t="s">
         <v>91</v>
       </c>
       <c r="E27" s="0" t="s">
+        <v>455</v>
+      </c>
+      <c r="F27" s="0" t="s">
         <v>456</v>
       </c>
-      <c r="F27" s="0" t="s">
+      <c r="G27" s="0" t="s">
         <v>457</v>
       </c>
-      <c r="G27" s="0" t="s">
+      <c r="I27" s="0" t="s">
         <v>458</v>
       </c>
-      <c r="J27" s="0" t="s">
+      <c r="L27" s="0" t="s">
         <v>459</v>
-      </c>
-      <c r="L27" s="0" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
+        <v>460</v>
+      </c>
+      <c r="B28" s="0" t="s">
         <v>461</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="C28" s="0" t="s">
         <v>462</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="D28" s="0" t="s">
         <v>463</v>
       </c>
-      <c r="D28" s="0" t="s">
+      <c r="E28" s="0" t="s">
         <v>464</v>
       </c>
-      <c r="E28" s="0" t="s">
+      <c r="F28" s="0" t="s">
         <v>465</v>
       </c>
-      <c r="F28" s="0" t="s">
+      <c r="L28" s="0" t="s">
         <v>466</v>
-      </c>
-      <c r="L28" s="0" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="29">
@@ -5342,98 +5339,98 @@
         <v>44</v>
       </c>
       <c r="B29" s="0" t="s">
+        <v>467</v>
+      </c>
+      <c r="C29" s="0" t="s">
         <v>468</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>469</v>
       </c>
       <c r="D29" s="0" t="s">
         <v>37</v>
       </c>
       <c r="E29" s="0" t="s">
+        <v>469</v>
+      </c>
+      <c r="F29" s="0" t="s">
         <v>470</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="G29" s="0" t="s">
         <v>471</v>
       </c>
-      <c r="G29" s="0" t="s">
+      <c r="H29" s="0" t="s">
         <v>472</v>
       </c>
-      <c r="H29" s="0" t="s">
+      <c r="I29" s="0" t="s">
         <v>473</v>
       </c>
-      <c r="I29" s="0" t="s">
+      <c r="J29" s="0" t="s">
         <v>474</v>
       </c>
-      <c r="J29" s="0" t="s">
+      <c r="K29" s="0" t="s">
         <v>475</v>
       </c>
-      <c r="K29" s="0" t="s">
+      <c r="L29" s="0" t="s">
         <v>476</v>
-      </c>
-      <c r="L29" s="0" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
+        <v>477</v>
+      </c>
+      <c r="B30" s="0" t="s">
         <v>478</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="C30" s="0" t="s">
         <v>479</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="D30" s="0" t="s">
         <v>480</v>
       </c>
-      <c r="D30" s="0" t="s">
+      <c r="E30" s="0" t="s">
         <v>481</v>
       </c>
-      <c r="E30" s="0" t="s">
+      <c r="F30" s="0" t="s">
         <v>482</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="G30" s="0" t="s">
         <v>483</v>
       </c>
-      <c r="G30" s="0" t="s">
+      <c r="J30" s="0" t="s">
         <v>484</v>
       </c>
-      <c r="I30" s="0" t="s">
+      <c r="K30" s="0" t="s">
         <v>485</v>
       </c>
-      <c r="K30" s="0" t="s">
+      <c r="L30" s="0" t="s">
         <v>486</v>
-      </c>
-      <c r="L30" s="0" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B31" s="0" t="s">
+        <v>487</v>
+      </c>
+      <c r="C31" s="0" t="s">
         <v>488</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="D31" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="E31" s="0" t="s">
         <v>489</v>
       </c>
-      <c r="D31" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="E31" s="0" t="s">
+      <c r="F31" s="0" t="s">
         <v>490</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="G31" s="0" t="s">
         <v>491</v>
       </c>
-      <c r="G31" s="0" t="s">
+      <c r="J31" s="0" t="s">
         <v>492</v>
       </c>
-      <c r="I31" s="0" t="s">
+      <c r="L31" s="0" t="s">
         <v>493</v>
-      </c>
-      <c r="L31" s="0" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="32">
@@ -5441,63 +5438,63 @@
         <v>33</v>
       </c>
       <c r="B32" s="0" t="s">
+        <v>494</v>
+      </c>
+      <c r="C32" s="0" t="s">
         <v>495</v>
-      </c>
-      <c r="C32" s="0" t="s">
-        <v>496</v>
       </c>
       <c r="D32" s="0" t="s">
         <v>25</v>
       </c>
       <c r="E32" s="0" t="s">
+        <v>496</v>
+      </c>
+      <c r="F32" s="0" t="s">
         <v>497</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="G32" s="0" t="s">
         <v>498</v>
       </c>
-      <c r="G32" s="0" t="s">
+      <c r="H32" s="0" t="s">
         <v>499</v>
       </c>
-      <c r="H32" s="0" t="s">
+      <c r="J32" s="0" t="s">
         <v>500</v>
       </c>
-      <c r="I32" s="0" t="s">
+      <c r="L32" s="0" t="s">
         <v>501</v>
-      </c>
-      <c r="L32" s="0" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B33" s="0" t="s">
+        <v>502</v>
+      </c>
+      <c r="C33" s="0" t="s">
         <v>503</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="D33" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E33" s="0" t="s">
         <v>504</v>
       </c>
-      <c r="D33" s="0" t="s">
-        <v>210</v>
-      </c>
-      <c r="E33" s="0" t="s">
+      <c r="F33" s="0" t="s">
         <v>505</v>
       </c>
-      <c r="F33" s="0" t="s">
+      <c r="G33" s="0" t="s">
         <v>506</v>
       </c>
-      <c r="G33" s="0" t="s">
+      <c r="H33" s="0" t="s">
         <v>507</v>
       </c>
-      <c r="H33" s="0" t="s">
+      <c r="I33" s="0" t="s">
+        <v>507</v>
+      </c>
+      <c r="L33" s="0" t="s">
         <v>508</v>
-      </c>
-      <c r="J33" s="0" t="s">
-        <v>508</v>
-      </c>
-      <c r="L33" s="0" t="s">
-        <v>509</v>
       </c>
     </row>
     <row r="34">
@@ -5505,159 +5502,159 @@
         <v>98</v>
       </c>
       <c r="B34" s="0" t="s">
+        <v>509</v>
+      </c>
+      <c r="C34" s="0" t="s">
         <v>510</v>
-      </c>
-      <c r="C34" s="0" t="s">
-        <v>511</v>
       </c>
       <c r="D34" s="0" t="s">
         <v>96</v>
       </c>
       <c r="E34" s="0" t="s">
+        <v>511</v>
+      </c>
+      <c r="F34" s="0" t="s">
         <v>512</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="G34" s="0" t="s">
         <v>513</v>
       </c>
-      <c r="G34" s="0" t="s">
+      <c r="H34" s="0" t="s">
         <v>514</v>
       </c>
-      <c r="H34" s="0" t="s">
+      <c r="I34" s="0" t="s">
         <v>515</v>
       </c>
-      <c r="I34" s="0" t="s">
+      <c r="J34" s="0" t="s">
         <v>516</v>
       </c>
-      <c r="J34" s="0" t="s">
+      <c r="L34" s="0" t="s">
         <v>517</v>
-      </c>
-      <c r="L34" s="0" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
+        <v>518</v>
+      </c>
+      <c r="B35" s="0" t="s">
         <v>519</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="C35" s="0" t="s">
         <v>520</v>
-      </c>
-      <c r="C35" s="0" t="s">
-        <v>521</v>
       </c>
       <c r="D35" s="0" t="s">
         <v>152</v>
       </c>
       <c r="E35" s="0" t="s">
+        <v>521</v>
+      </c>
+      <c r="F35" s="0" t="s">
         <v>522</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="G35" s="0" t="s">
         <v>523</v>
       </c>
-      <c r="G35" s="0" t="s">
+      <c r="H35" s="0" t="s">
         <v>524</v>
       </c>
-      <c r="H35" s="0" t="s">
+      <c r="I35" s="0" t="s">
+        <v>523</v>
+      </c>
+      <c r="J35" s="0" t="s">
         <v>525</v>
       </c>
-      <c r="I35" s="0" t="s">
+      <c r="L35" s="0" t="s">
         <v>526</v>
-      </c>
-      <c r="J35" s="0" t="s">
-        <v>524</v>
-      </c>
-      <c r="L35" s="0" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="s">
+        <v>527</v>
+      </c>
+      <c r="B36" s="0" t="s">
         <v>528</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="C36" s="0" t="s">
         <v>529</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="D36" s="0" t="s">
         <v>530</v>
       </c>
-      <c r="D36" s="0" t="s">
+      <c r="E36" s="0" t="s">
         <v>531</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="F36" s="0" t="s">
         <v>532</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="G36" s="0" t="s">
         <v>533</v>
       </c>
-      <c r="G36" s="0" t="s">
+      <c r="L36" s="0" t="s">
         <v>534</v>
-      </c>
-      <c r="L36" s="0" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B37" s="0" t="s">
+        <v>535</v>
+      </c>
+      <c r="C37" s="0" t="s">
         <v>536</v>
       </c>
-      <c r="C37" s="0" t="s">
+      <c r="D37" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="E37" s="0" t="s">
         <v>537</v>
       </c>
-      <c r="D37" s="0" t="s">
-        <v>215</v>
-      </c>
-      <c r="E37" s="0" t="s">
+      <c r="F37" s="0" t="s">
         <v>538</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="G37" s="0" t="s">
         <v>539</v>
       </c>
-      <c r="G37" s="0" t="s">
+      <c r="H37" s="0" t="s">
         <v>540</v>
       </c>
-      <c r="H37" s="0" t="s">
+      <c r="I37" s="0" t="s">
         <v>541</v>
       </c>
-      <c r="J37" s="0" t="s">
+      <c r="L37" s="0" t="s">
         <v>542</v>
-      </c>
-      <c r="L37" s="0" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="s">
+        <v>543</v>
+      </c>
+      <c r="B38" s="0" t="s">
         <v>544</v>
       </c>
-      <c r="B38" s="0" t="s">
+      <c r="C38" s="0" t="s">
         <v>545</v>
       </c>
-      <c r="C38" s="0" t="s">
+      <c r="D38" s="0" t="s">
         <v>546</v>
       </c>
-      <c r="D38" s="0" t="s">
+      <c r="E38" s="0" t="s">
         <v>547</v>
       </c>
-      <c r="E38" s="0" t="s">
+      <c r="F38" s="0" t="s">
         <v>548</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="G38" s="0" t="s">
         <v>549</v>
       </c>
-      <c r="G38" s="0" t="s">
+      <c r="H38" s="0" t="s">
         <v>550</v>
       </c>
-      <c r="H38" s="0" t="s">
+      <c r="J38" s="0" t="s">
         <v>551</v>
       </c>
-      <c r="I38" s="0" t="s">
+      <c r="L38" s="0" t="s">
         <v>552</v>
-      </c>
-      <c r="L38" s="0" t="s">
-        <v>553</v>
       </c>
     </row>
     <row r="39">
@@ -5665,37 +5662,37 @@
         <v>142</v>
       </c>
       <c r="B39" s="0" t="s">
+        <v>553</v>
+      </c>
+      <c r="C39" s="0" t="s">
         <v>554</v>
-      </c>
-      <c r="C39" s="0" t="s">
-        <v>555</v>
       </c>
       <c r="D39" s="0" t="s">
         <v>140</v>
       </c>
       <c r="E39" s="0" t="s">
+        <v>555</v>
+      </c>
+      <c r="F39" s="0" t="s">
         <v>556</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="G39" s="0" t="s">
         <v>557</v>
       </c>
-      <c r="G39" s="0" t="s">
+      <c r="H39" s="0" t="s">
         <v>558</v>
       </c>
-      <c r="H39" s="0" t="s">
+      <c r="I39" s="0" t="s">
         <v>559</v>
       </c>
-      <c r="I39" s="0" t="s">
+      <c r="J39" s="0" t="s">
         <v>560</v>
       </c>
-      <c r="J39" s="0" t="s">
+      <c r="K39" s="0" t="s">
         <v>561</v>
       </c>
-      <c r="K39" s="0" t="s">
+      <c r="L39" s="0" t="s">
         <v>562</v>
-      </c>
-      <c r="L39" s="0" t="s">
-        <v>563</v>
       </c>
     </row>
     <row r="40">
@@ -5703,37 +5700,37 @@
         <v>113</v>
       </c>
       <c r="B40" s="0" t="s">
+        <v>563</v>
+      </c>
+      <c r="C40" s="0" t="s">
         <v>564</v>
-      </c>
-      <c r="C40" s="0" t="s">
-        <v>565</v>
       </c>
       <c r="D40" s="0" t="s">
         <v>110</v>
       </c>
       <c r="E40" s="0" t="s">
+        <v>565</v>
+      </c>
+      <c r="F40" s="0" t="s">
         <v>566</v>
       </c>
-      <c r="F40" s="0" t="s">
+      <c r="G40" s="0" t="s">
         <v>567</v>
       </c>
-      <c r="G40" s="0" t="s">
+      <c r="H40" s="0" t="s">
         <v>568</v>
       </c>
-      <c r="H40" s="0" t="s">
+      <c r="I40" s="0" t="s">
         <v>569</v>
       </c>
-      <c r="I40" s="0" t="s">
+      <c r="J40" s="0" t="s">
         <v>570</v>
       </c>
-      <c r="J40" s="0" t="s">
+      <c r="K40" s="0" t="s">
         <v>571</v>
       </c>
-      <c r="K40" s="0" t="s">
+      <c r="L40" s="0" t="s">
         <v>572</v>
-      </c>
-      <c r="L40" s="0" t="s">
-        <v>573</v>
       </c>
     </row>
     <row r="41">
@@ -5741,147 +5738,147 @@
         <v>130</v>
       </c>
       <c r="B41" s="0" t="s">
+        <v>573</v>
+      </c>
+      <c r="C41" s="0" t="s">
         <v>574</v>
-      </c>
-      <c r="C41" s="0" t="s">
-        <v>575</v>
       </c>
       <c r="D41" s="0" t="s">
         <v>128</v>
       </c>
       <c r="E41" s="0" t="s">
+        <v>575</v>
+      </c>
+      <c r="F41" s="0" t="s">
         <v>576</v>
       </c>
-      <c r="F41" s="0" t="s">
+      <c r="G41" s="0" t="s">
         <v>577</v>
       </c>
-      <c r="G41" s="0" t="s">
+      <c r="H41" s="0" t="s">
         <v>578</v>
       </c>
-      <c r="H41" s="0" t="s">
+      <c r="I41" s="0" t="s">
         <v>579</v>
       </c>
-      <c r="I41" s="0" t="s">
+      <c r="J41" s="0" t="s">
         <v>580</v>
       </c>
-      <c r="J41" s="0" t="s">
+      <c r="K41" s="0" t="s">
         <v>581</v>
       </c>
-      <c r="K41" s="0" t="s">
+      <c r="L41" s="0" t="s">
         <v>582</v>
-      </c>
-      <c r="L41" s="0" t="s">
-        <v>583</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="s">
+        <v>583</v>
+      </c>
+      <c r="B42" s="0" t="s">
         <v>584</v>
       </c>
-      <c r="B42" s="0" t="s">
+      <c r="C42" s="0" t="s">
         <v>585</v>
       </c>
-      <c r="C42" s="0" t="s">
+      <c r="D42" s="0" t="s">
         <v>586</v>
       </c>
-      <c r="D42" s="0" t="s">
+      <c r="E42" s="0" t="s">
         <v>587</v>
       </c>
-      <c r="E42" s="0" t="s">
+      <c r="F42" s="0" t="s">
         <v>588</v>
       </c>
-      <c r="F42" s="0" t="s">
+      <c r="G42" s="0" t="s">
         <v>589</v>
       </c>
-      <c r="G42" s="0" t="s">
+      <c r="L42" s="0" t="s">
         <v>590</v>
-      </c>
-      <c r="L42" s="0" t="s">
-        <v>591</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C43" s="0" t="s">
+        <v>591</v>
+      </c>
+      <c r="D43" s="0" t="s">
+        <v>220</v>
+      </c>
+      <c r="E43" s="0" t="s">
         <v>592</v>
       </c>
-      <c r="D43" s="0" t="s">
-        <v>221</v>
-      </c>
-      <c r="E43" s="0" t="s">
+      <c r="F43" s="0" t="s">
         <v>593</v>
       </c>
-      <c r="F43" s="0" t="s">
+      <c r="G43" s="0" t="s">
         <v>594</v>
       </c>
-      <c r="G43" s="0" t="s">
+      <c r="H43" s="0" t="s">
         <v>595</v>
       </c>
-      <c r="H43" s="0" t="s">
+      <c r="I43" s="0" t="s">
         <v>596</v>
       </c>
-      <c r="J43" s="0" t="s">
+      <c r="L43" s="0" t="s">
         <v>597</v>
-      </c>
-      <c r="L43" s="0" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="s">
+        <v>598</v>
+      </c>
+      <c r="B44" s="0" t="s">
         <v>599</v>
       </c>
-      <c r="B44" s="0" t="s">
+      <c r="C44" s="0" t="s">
         <v>600</v>
-      </c>
-      <c r="C44" s="0" t="s">
-        <v>601</v>
       </c>
       <c r="D44" s="0" t="s">
         <v>134</v>
       </c>
       <c r="E44" s="0" t="s">
+        <v>601</v>
+      </c>
+      <c r="F44" s="0" t="s">
         <v>602</v>
       </c>
-      <c r="F44" s="0" t="s">
+      <c r="G44" s="0" t="s">
         <v>603</v>
       </c>
-      <c r="G44" s="0" t="s">
+      <c r="I44" s="0" t="s">
         <v>604</v>
       </c>
-      <c r="J44" s="0" t="s">
+      <c r="L44" s="0" t="s">
         <v>605</v>
-      </c>
-      <c r="L44" s="0" t="s">
-        <v>606</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="0" t="s">
+        <v>606</v>
+      </c>
+      <c r="B45" s="0" t="s">
         <v>607</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="C45" s="0" t="s">
         <v>608</v>
       </c>
-      <c r="C45" s="0" t="s">
+      <c r="D45" s="0" t="s">
         <v>609</v>
       </c>
-      <c r="D45" s="0" t="s">
+      <c r="E45" s="0" t="s">
         <v>610</v>
       </c>
-      <c r="E45" s="0" t="s">
+      <c r="F45" s="0" t="s">
         <v>611</v>
       </c>
-      <c r="F45" s="0" t="s">
+      <c r="L45" s="0" t="s">
         <v>612</v>
-      </c>
-      <c r="L45" s="0" t="s">
-        <v>613</v>
       </c>
     </row>
     <row r="46">
@@ -5889,31 +5886,31 @@
         <v>52</v>
       </c>
       <c r="B46" s="0" t="s">
+        <v>613</v>
+      </c>
+      <c r="C46" s="0" t="s">
         <v>614</v>
-      </c>
-      <c r="C46" s="0" t="s">
-        <v>615</v>
       </c>
       <c r="D46" s="0" t="s">
         <v>48</v>
       </c>
       <c r="E46" s="0" t="s">
+        <v>615</v>
+      </c>
+      <c r="F46" s="0" t="s">
         <v>616</v>
       </c>
-      <c r="F46" s="0" t="s">
+      <c r="G46" s="0" t="s">
         <v>617</v>
       </c>
-      <c r="G46" s="0" t="s">
+      <c r="H46" s="0" t="s">
         <v>618</v>
       </c>
-      <c r="H46" s="0" t="s">
+      <c r="I46" s="0" t="s">
         <v>619</v>
       </c>
-      <c r="J46" s="0" t="s">
+      <c r="L46" s="0" t="s">
         <v>620</v>
-      </c>
-      <c r="L46" s="0" t="s">
-        <v>621</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update session and speaker data for upcoming event
</commit_message>
<xml_diff>
--- a/src/assets/sessionize/data-advanced.xlsx
+++ b/src/assets/sessionize/data-advanced.xlsx
@@ -418,24 +418,25 @@
     <t>d3f982bf-06f2-4a7a-ac5a-2479f4cec0b2</t>
   </si>
   <si>
-    <t>60fps o niente: Rendering Pipeline a suon di esempi pratici!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se un'animazione scatta o una UI risponde in ritardo, non imprecare: la colpa non e' sempre del browser! Hai mai sentito parlare della rendering pipeline? Se la risposta è no, ti assicuriamo che avresti dovuto!_x000D_
-_x000D_
-Ottenere le giuste performance non è sempre gratis...impariamo quindi cosa sia la render pipeline e capiamo come quanto stupefacente ottimizzare ogni scelta alle API e alle proprieta coinvolte, sia lato CSS sia lato JavaScript._x000D_
-_x000D_
-Facciamo una scorpacciata di criteri chiari, esempi riutilizzabili e animazioni fluide su browser e webview reali...con una coppia che solo a vederla vi farà passare il reflow!_x000D_
+    <t>Claude Code Internals</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thanks to the Anthropic source code leak we can now learn how a top AI player has built a successful agentic platform out of a traditional LLM server._x000D_
+_x000D_
+This talk shows the fundamental features of many existing Agentic platforms but also some undocumented and unreleased features that anticipate the future._x000D_
 </t>
   </si>
   <si>
-    <t>Francesco Sciuti, Emiliano Pisu</t>
-  </si>
-  <si>
-    <t>Web</t>
-  </si>
-  <si>
-    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b, 05ed4b4a-5d57-4602-bb4e-8d55efad3e0f</t>
+    <t>Cristian Burrini</t>
+  </si>
+  <si>
+    <t>cristian.burrini@gmail.com</t>
+  </si>
+  <si>
+    <t>Yes, but I won't be applying with Google's speaker program</t>
+  </si>
+  <si>
+    <t>9bf00943-d891-4eb3-9400-430ab2430d1e</t>
   </si>
   <si>
     <t>Developer Mezzosangue: Padroneggiare l'Alchimia dell'IA e del Personal Branding</t>
@@ -481,6 +482,9 @@
   </si>
   <si>
     <t>christian@liebel.org</t>
+  </si>
+  <si>
+    <t>Web</t>
   </si>
   <si>
     <t>Germany</t>
@@ -705,25 +709,21 @@
     <t>24ce44ea-d436-4476-88ac-08695de0acfa</t>
   </si>
   <si>
-    <t>Claude Code Internals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thanks to the Anthropic source code leak we can now learn how a top AI player has built a successful agentic platform out of a traditional LLM server._x000D_
-_x000D_
-This talk shows the fundamental features of many existing Agentic platforms but also some undocumented and unreleased features that anticipate the future._x000D_
+    <t>60fps o niente: Rendering Pipeline a suon di esempi pratici!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se un'animazione scatta o una UI risponde in ritardo, non imprecare: la colpa non e' sempre del browser! Hai mai sentito parlare della rendering pipeline? Se la risposta è no, ti assicuriamo che avresti dovuto!_x000D_
+_x000D_
+Ottenere le giuste performance non è sempre gratis...impariamo quindi cosa sia la render pipeline e capiamo come quanto stupefacente ottimizzare ogni scelta alle API e alle proprieta coinvolte, sia lato CSS sia lato JavaScript._x000D_
+_x000D_
+Facciamo una scorpacciata di criteri chiari, esempi riutilizzabili e animazioni fluide su browser e webview reali...con una coppia che solo a vederla vi farà passare il reflow!_x000D_
 </t>
   </si>
   <si>
-    <t>Cristian Burrini</t>
-  </si>
-  <si>
-    <t>cristian.burrini@gmail.com</t>
-  </si>
-  <si>
-    <t>Yes, but I won't be applying with Google's speaker program</t>
-  </si>
-  <si>
-    <t>9bf00943-d891-4eb3-9400-430ab2430d1e</t>
+    <t>Francesco Sciuti, Emiliano Pisu</t>
+  </si>
+  <si>
+    <t>b8b99b42-456a-4934-a1ac-414d4ba2990b, 05ed4b4a-5d57-4602-bb4e-8d55efad3e0f</t>
   </si>
   <si>
     <t>IWD Panel: Quando il futuro era donna</t>
@@ -926,12 +926,12 @@
     <t>Company Website</t>
   </si>
   <si>
+    <t>Instagram</t>
+  </si>
+  <si>
     <t>Blog</t>
   </si>
   <si>
-    <t>Instagram</t>
-  </si>
-  <si>
     <t>Facebook</t>
   </si>
   <si>
@@ -1003,10 +1003,10 @@
     <t>https://devdojo.it</t>
   </si>
   <si>
+    <t>https://www.instagram.com/pixu1980/</t>
+  </si>
+  <si>
     <t>https://dout.dev</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/pixu1980/</t>
   </si>
   <si>
     <t>https://sessionize.com/image/fd3b-400o400o1-BwkHXp3qRbEw3D5V2gPbAY.png</t>
@@ -1206,10 +1206,10 @@
     <t>https://fractal.cloud</t>
   </si>
   <si>
+    <t>https://www.instagram.com/michel_murabito/</t>
+  </si>
+  <si>
     <t>https://michelmurabito.com</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/michel_murabito/</t>
   </si>
   <si>
     <t>https://www.facebook.com/michelmurabito</t>
@@ -1295,10 +1295,10 @@
     <t>https://bit.ly/pantarei-mb</t>
   </si>
   <si>
+    <t>https://instagram.com/pantarei_mb</t>
+  </si>
+  <si>
     <t>https://sites.google.com/view/pantarei-mb-en/blog</t>
-  </si>
-  <si>
-    <t>https://instagram.com/pantarei_mb</t>
   </si>
   <si>
     <t>https://sessionize.com/image/677e-400o400o1-shpurTgXp4EfDBWu3fPXrZ.jpg</t>
@@ -1518,10 +1518,10 @@
     <t>https://pescara.python.it/</t>
   </si>
   <si>
+    <t>https://www.instagram.com/luca_di_vita_</t>
+  </si>
+  <si>
     <t>https://www.lucadivita.it/</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/luca_di_vita_</t>
   </si>
   <si>
     <t>https://sessionize.com/image/77c6-400o400o1-hMWZzLKMh7xt3XWNZALNnt.jpg</t>
@@ -1640,10 +1640,10 @@
     <t>https://devmy.it</t>
   </si>
   <si>
+    <t>https://www.instagram.com/Devmy.it/</t>
+  </si>
+  <si>
     <t>https://devmy.it/blog</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/Devmy.it/</t>
   </si>
   <si>
     <t>https://www.facebook.com/francesco.sciuti/</t>
@@ -1773,10 +1773,10 @@
     <t>https://monjadariva.it</t>
   </si>
   <si>
+    <t>https://instagram.com/monja.dariva</t>
+  </si>
+  <si>
     <t>https://monjadariva.it/blog</t>
-  </si>
-  <si>
-    <t>https://instagram.com/monja.dariva</t>
   </si>
   <si>
     <t>https://sessionize.com/image/3e16-400o400o1-7jvdkF5R8VCzcbkb33Ty6R.jpg</t>
@@ -1915,12 +1915,12 @@
     <t>https://learnbydo.ing/</t>
   </si>
   <si>
+    <t>https://www.instagram.com/biondifabio/</t>
+  </si>
+  <si>
     <t>http://fabiobiondi.dev/</t>
   </si>
   <si>
-    <t>https://www.instagram.com/biondifabio/</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/groups/fabiobiondi.training</t>
   </si>
   <si>
@@ -1945,12 +1945,12 @@
     <t>https://www.mann-ai.com/</t>
   </si>
   <si>
+    <t>https://www.instagram.com/mortadha_mannai/</t>
+  </si>
+  <si>
     <t>https://manaimortadha.medium.com/</t>
   </si>
   <si>
-    <t>https://www.instagram.com/mortadha_mannai/</t>
-  </si>
-  <si>
     <t>https://www.facebook.com/profile.php?id=100004306062352</t>
   </si>
   <si>
@@ -1975,10 +1975,10 @@
     <t>https://www.thinktecture.com</t>
   </si>
   <si>
+    <t>https://www.instagram.com/chliebel/</t>
+  </si>
+  <si>
     <t>https://christianliebel.com</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/chliebel/</t>
   </si>
   <si>
     <t>https://www.facebook.com/christianliebel</t>
@@ -3049,7 +3049,7 @@
     </row>
     <row r="15">
       <c r="A15" s="0">
-        <v>1155640</v>
+        <v>1200474</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>114</v>
@@ -3058,16 +3058,16 @@
         <v>115</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>36</v>
+        <v>116</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>37</v>
+        <v>117</v>
       </c>
       <c r="F15" s="0" t="s">
         <v>116</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>117</v>
+        <v>38</v>
       </c>
       <c r="H15" s="0" t="s">
         <v>27</v>
@@ -3076,22 +3076,22 @@
         <v>28</v>
       </c>
       <c r="J15" s="0" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="K15" s="0" t="s">
         <v>42</v>
       </c>
       <c r="L15" s="0" t="s">
-        <v>43</v>
+        <v>118</v>
       </c>
       <c r="M15" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N15" s="5">
-        <v>46087.774690972219</v>
+        <v>46120.84242144676</v>
       </c>
       <c r="O15" s="5">
-        <v>46090.30420543981</v>
+        <v>46120.882133599538</v>
       </c>
       <c r="P15" s="0" t="s">
         <v>51</v>
@@ -3106,7 +3106,7 @@
         <v>0</v>
       </c>
       <c r="V15" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16">
@@ -3114,19 +3114,19 @@
         <v>1132787</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E16" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="F16" s="0" t="s">
         <v>122</v>
-      </c>
-      <c r="F16" s="0" t="s">
-        <v>121</v>
       </c>
       <c r="G16" s="0" t="s">
         <v>38</v>
@@ -3147,7 +3147,7 @@
         <v>31</v>
       </c>
       <c r="M16" s="0" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N16" s="5">
         <v>46056.871177777779</v>
@@ -3168,7 +3168,7 @@
         <v>0</v>
       </c>
       <c r="V16" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17">
@@ -3176,22 +3176,22 @@
         <v>1147593</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E17" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="F17" s="0" t="s">
         <v>128</v>
       </c>
-      <c r="F17" s="0" t="s">
-        <v>127</v>
-      </c>
       <c r="G17" s="0" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="H17" s="0" t="s">
         <v>27</v>
@@ -3209,7 +3209,7 @@
         <v>43</v>
       </c>
       <c r="M17" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N17" s="5">
         <v>46087.774690972219</v>
@@ -3230,7 +3230,7 @@
         <v>0</v>
       </c>
       <c r="V17" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18">
@@ -3238,19 +3238,19 @@
         <v>1148023</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F18" s="0" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G18" s="0" t="s">
         <v>26</v>
@@ -3292,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="V18" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19">
@@ -3300,19 +3300,19 @@
         <v>1208979</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F19" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G19" s="0" t="s">
         <v>38</v>
@@ -3321,7 +3321,7 @@
         <v>39</v>
       </c>
       <c r="I19" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J19" s="0" t="s">
         <v>79</v>
@@ -3354,7 +3354,7 @@
         <v>0</v>
       </c>
       <c r="V19" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20">
@@ -3362,19 +3362,19 @@
         <v>1148693</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E20" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F20" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G20" s="0" t="s">
         <v>26</v>
@@ -3416,7 +3416,7 @@
         <v>0</v>
       </c>
       <c r="V20" s="0" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21">
@@ -3424,22 +3424,22 @@
         <v>1123087</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F21" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H21" s="0" t="s">
         <v>27</v>
@@ -3478,7 +3478,7 @@
         <v>0</v>
       </c>
       <c r="V21" s="0" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="22">
@@ -3486,19 +3486,19 @@
         <v>1149006</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F22" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G22" s="0" t="s">
         <v>26</v>
@@ -3540,7 +3540,7 @@
         <v>0</v>
       </c>
       <c r="V22" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23">
@@ -3548,19 +3548,19 @@
         <v>1154402</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F23" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G23" s="0" t="s">
         <v>38</v>
@@ -3602,7 +3602,7 @@
         <v>0</v>
       </c>
       <c r="V23" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="24">
@@ -3610,19 +3610,19 @@
         <v>1149301</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E24" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F24" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G24" s="0" t="s">
         <v>26</v>
@@ -3664,7 +3664,7 @@
         <v>0</v>
       </c>
       <c r="V24" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25">
@@ -3672,19 +3672,19 @@
         <v>1149383</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F25" s="0" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G25" s="0" t="s">
         <v>38</v>
@@ -3726,7 +3726,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="0" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="26">
@@ -3734,19 +3734,19 @@
         <v>1151362</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F26" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G26" s="0" t="s">
         <v>38</v>
@@ -3788,7 +3788,7 @@
         <v>0</v>
       </c>
       <c r="V26" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27">
@@ -3796,19 +3796,19 @@
         <v>1155630</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F27" s="0" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G27" s="0" t="s">
         <v>71</v>
@@ -3829,7 +3829,7 @@
         <v>31</v>
       </c>
       <c r="M27" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="N27" s="5">
         <v>46080.807078935184</v>
@@ -3850,30 +3850,30 @@
         <v>0</v>
       </c>
       <c r="V27" s="0" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0">
-        <v>1200474</v>
+        <v>1155640</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>188</v>
+        <v>36</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>189</v>
+        <v>37</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>38</v>
+        <v>130</v>
       </c>
       <c r="H28" s="0" t="s">
         <v>27</v>
@@ -3882,22 +3882,22 @@
         <v>28</v>
       </c>
       <c r="J28" s="0" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="K28" s="0" t="s">
         <v>42</v>
       </c>
       <c r="L28" s="0" t="s">
-        <v>190</v>
+        <v>43</v>
       </c>
       <c r="M28" s="0" t="s">
         <v>32</v>
       </c>
       <c r="N28" s="5">
-        <v>46120.84242144676</v>
+        <v>46087.774690972219</v>
       </c>
       <c r="O28" s="5">
-        <v>46120.882133599538</v>
+        <v>46090.30420543981</v>
       </c>
       <c r="P28" s="0" t="s">
         <v>57</v>
@@ -3926,10 +3926,10 @@
         <v>193</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F29" s="0" t="s">
         <v>194</v>
@@ -3997,7 +3997,7 @@
         <v>198</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H30" s="0" t="s">
         <v>72</v>
@@ -4552,7 +4552,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>258</v>
@@ -4561,7 +4561,7 @@
         <v>259</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E3" s="0" t="s">
         <v>260</v>
@@ -4668,7 +4668,7 @@
       <c r="H6" s="0" t="s">
         <v>290</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="J6" s="0" t="s">
         <v>291</v>
       </c>
       <c r="L6" s="0" t="s">
@@ -4677,7 +4677,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>293</v>
@@ -4686,7 +4686,7 @@
         <v>294</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E7" s="0" t="s">
         <v>295</v>
@@ -4732,7 +4732,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>308</v>
@@ -4741,7 +4741,7 @@
         <v>309</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E9" s="0" t="s">
         <v>310</v>
@@ -4784,7 +4784,7 @@
       <c r="H10" s="0" t="s">
         <v>320</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="J10" s="0" t="s">
         <v>321</v>
       </c>
       <c r="L10" s="0" t="s">
@@ -4793,7 +4793,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>323</v>
@@ -4802,7 +4802,7 @@
         <v>324</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E11" s="0" t="s">
         <v>325</v>
@@ -4813,7 +4813,7 @@
       <c r="G11" s="0" t="s">
         <v>327</v>
       </c>
-      <c r="J11" s="0" t="s">
+      <c r="I11" s="0" t="s">
         <v>328</v>
       </c>
       <c r="L11" s="0" t="s">
@@ -4912,7 +4912,7 @@
       <c r="H14" s="0" t="s">
         <v>356</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="J14" s="0" t="s">
         <v>357</v>
       </c>
       <c r="L14" s="0" t="s">
@@ -4921,7 +4921,7 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>359</v>
@@ -4930,7 +4930,7 @@
         <v>360</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E15" s="0" t="s">
         <v>361</v>
@@ -4956,7 +4956,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>368</v>
@@ -4965,7 +4965,7 @@
         <v>369</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E16" s="0" t="s">
         <v>370</v>
@@ -4979,7 +4979,7 @@
       <c r="H16" s="0" t="s">
         <v>373</v>
       </c>
-      <c r="I16" s="0" t="s">
+      <c r="J16" s="0" t="s">
         <v>374</v>
       </c>
       <c r="K16" s="0" t="s">
@@ -5055,7 +5055,7 @@
         <v>395</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E19" s="0" t="s">
         <v>396</v>
@@ -5124,7 +5124,7 @@
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B22" s="0" t="s">
         <v>413</v>
@@ -5133,7 +5133,7 @@
         <v>414</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E22" s="0" t="s">
         <v>415</v>
@@ -5147,7 +5147,7 @@
       <c r="H22" s="0" t="s">
         <v>418</v>
       </c>
-      <c r="J22" s="0" t="s">
+      <c r="I22" s="0" t="s">
         <v>419</v>
       </c>
       <c r="L22" s="0" t="s">
@@ -5179,7 +5179,7 @@
       <c r="H23" s="0" t="s">
         <v>426</v>
       </c>
-      <c r="I23" s="0" t="s">
+      <c r="J23" s="0" t="s">
         <v>427</v>
       </c>
       <c r="L23" s="0" t="s">
@@ -5223,7 +5223,7 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>191</v>
+        <v>119</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>438</v>
@@ -5232,7 +5232,7 @@
         <v>439</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>189</v>
+        <v>117</v>
       </c>
       <c r="E25" s="0" t="s">
         <v>440</v>
@@ -5275,7 +5275,7 @@
       <c r="H26" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="J26" s="0" t="s">
+      <c r="I26" s="0" t="s">
         <v>451</v>
       </c>
       <c r="L26" s="0" t="s">
@@ -5304,7 +5304,7 @@
       <c r="G27" s="0" t="s">
         <v>457</v>
       </c>
-      <c r="I27" s="0" t="s">
+      <c r="J27" s="0" t="s">
         <v>458</v>
       </c>
       <c r="L27" s="0" t="s">
@@ -5394,7 +5394,7 @@
       <c r="G30" s="0" t="s">
         <v>483</v>
       </c>
-      <c r="J30" s="0" t="s">
+      <c r="I30" s="0" t="s">
         <v>484</v>
       </c>
       <c r="K30" s="0" t="s">
@@ -5426,7 +5426,7 @@
       <c r="G31" s="0" t="s">
         <v>491</v>
       </c>
-      <c r="J31" s="0" t="s">
+      <c r="I31" s="0" t="s">
         <v>492</v>
       </c>
       <c r="L31" s="0" t="s">
@@ -5458,7 +5458,7 @@
       <c r="H32" s="0" t="s">
         <v>499</v>
       </c>
-      <c r="J32" s="0" t="s">
+      <c r="I32" s="0" t="s">
         <v>500</v>
       </c>
       <c r="L32" s="0" t="s">
@@ -5490,7 +5490,7 @@
       <c r="H33" s="0" t="s">
         <v>507</v>
       </c>
-      <c r="I33" s="0" t="s">
+      <c r="J33" s="0" t="s">
         <v>507</v>
       </c>
       <c r="L33" s="0" t="s">
@@ -5543,7 +5543,7 @@
         <v>520</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E35" s="0" t="s">
         <v>521</v>
@@ -5558,10 +5558,10 @@
         <v>524</v>
       </c>
       <c r="I35" s="0" t="s">
+        <v>525</v>
+      </c>
+      <c r="J35" s="0" t="s">
         <v>523</v>
-      </c>
-      <c r="J35" s="0" t="s">
-        <v>525</v>
       </c>
       <c r="L35" s="0" t="s">
         <v>526</v>
@@ -5618,7 +5618,7 @@
       <c r="H37" s="0" t="s">
         <v>540</v>
       </c>
-      <c r="I37" s="0" t="s">
+      <c r="J37" s="0" t="s">
         <v>541</v>
       </c>
       <c r="L37" s="0" t="s">
@@ -5650,7 +5650,7 @@
       <c r="H38" s="0" t="s">
         <v>550</v>
       </c>
-      <c r="J38" s="0" t="s">
+      <c r="I38" s="0" t="s">
         <v>551</v>
       </c>
       <c r="L38" s="0" t="s">
@@ -5659,7 +5659,7 @@
     </row>
     <row r="39">
       <c r="A39" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B39" s="0" t="s">
         <v>553</v>
@@ -5668,7 +5668,7 @@
         <v>554</v>
       </c>
       <c r="D39" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E39" s="0" t="s">
         <v>555</v>
@@ -5735,7 +5735,7 @@
     </row>
     <row r="41">
       <c r="A41" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B41" s="0" t="s">
         <v>573</v>
@@ -5744,7 +5744,7 @@
         <v>574</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E41" s="0" t="s">
         <v>575</v>
@@ -5822,7 +5822,7 @@
       <c r="H43" s="0" t="s">
         <v>595</v>
       </c>
-      <c r="I43" s="0" t="s">
+      <c r="J43" s="0" t="s">
         <v>596</v>
       </c>
       <c r="L43" s="0" t="s">
@@ -5840,7 +5840,7 @@
         <v>600</v>
       </c>
       <c r="D44" s="0" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E44" s="0" t="s">
         <v>601</v>
@@ -5851,7 +5851,7 @@
       <c r="G44" s="0" t="s">
         <v>603</v>
       </c>
-      <c r="I44" s="0" t="s">
+      <c r="J44" s="0" t="s">
         <v>604</v>
       </c>
       <c r="L44" s="0" t="s">
@@ -5906,7 +5906,7 @@
       <c r="H46" s="0" t="s">
         <v>618</v>
       </c>
-      <c r="I46" s="0" t="s">
+      <c r="J46" s="0" t="s">
         <v>619</v>
       </c>
       <c r="L46" s="0" t="s">

</xml_diff>